<commit_message>
Move C3 Betonas plant to Vilnius
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$70</definedName>
@@ -8045,38 +8045,38 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Stašėnai</t>
+          <t>Vilnius</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Jonavos r. sav.</t>
+          <t>Vilniaus m. sav.</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Dirvaliai, Šveicarijos sen., Jonavos r. sav.</t>
+          <t>Ušos g. 21, Vilnius, 02121 Vilniaus m. sav.</t>
         </is>
       </c>
       <c r="I67" s="3" t="n">
-        <v>55.033</v>
+        <v>54.6493094</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>24.183</v>
+        <v>25.3107972</v>
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
+          <t>Tikslus adreso taškas pagal geokodavimą</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas oficialus puslapis</t>
+          <t>ArcGIS geokodavimas pagal naudotojo pateiktą adresą</t>
         </is>
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://geocode.arcgis.com/arcgis/rest/services/World/GeocodeServer/findAddressCandidates</t>
         </is>
       </c>
       <c r="N67" s="2" t="inlineStr">
@@ -8091,12 +8091,12 @@
       </c>
       <c r="P67" s="2" t="inlineStr">
         <is>
-          <t>Stašėnai Plant</t>
+          <t>Vilnius Ušos g. Plant</t>
         </is>
       </c>
       <c r="Q67" s="2" t="inlineStr">
         <is>
-          <t>Ammann Elba Euromix C120, 3 m³</t>
+          <t>Nissbau Euromix C120, 3 m³</t>
         </is>
       </c>
       <c r="R67" s="2" t="inlineStr">
@@ -8111,7 +8111,7 @@
       </c>
       <c r="T67" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
+          <t>Betono mazgas Nissbau Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U67" s="5" t="n">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="Y67" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Perkelta iš Stašėnų lokacijos į Ušos g. 21, Vilnius pagal naudotojo pateiktą informaciją. Maišyklė pervadinta į Nissbau Euromix C120, 3 m³. Koordinatės geokoduotos pagal naują adresą.</t>
         </is>
       </c>
       <c r="Z67" s="2" t="inlineStr">
@@ -8611,7 +8611,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-07T09:56:29.575140+00:00</t>
+          <t>2026-09-14T04:36:38.879321+00:00</t>
         </is>
       </c>
     </row>
@@ -8666,7 +8666,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-07T09:56:29.575852+00:00</t>
+          <t>2026-09-14T04:36:38.880373+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Update Ponas betonas plant details
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -513,7 +513,7 @@
     <col width="40" customWidth="1" min="16" max="16"/>
     <col width="32" customWidth="1" min="17" max="17"/>
     <col width="30" customWidth="1" min="18" max="18"/>
-    <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="34" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="29" customWidth="1" min="21" max="21"/>
     <col width="42" customWidth="1" min="22" max="22"/>
@@ -8469,7 +8469,7 @@
       </c>
       <c r="P70" s="2" t="inlineStr">
         <is>
-          <t>Ponas betonas betono mazgas</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q70" s="2" t="inlineStr">
@@ -8484,12 +8484,12 @@
       </c>
       <c r="S70" s="4" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>2 matomi oficialioje nuotraukoje</t>
         </is>
       </c>
       <c r="T70" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame UAB Ponas betonas puslapyje nurodoma, kad įmonė turi nuosavą betono mazgą, gamina prekinį betoną ir jį pristato. Mazgo gamintojas, maišyklė, našumas ir silosų skaičius viešai nenurodyti.</t>
+          <t>Oficialiame UAB Ponas betonas puslapyje nurodoma, kad įmonė turi nuosavą betono mazgą, gamina prekinį betoną ir jį pristato. Puslapio hero nuotraukoje ant silosų matomas ELKON ženklinimas, todėl mazgo gamintojas identifikuotas kaip Elkon. Konkretus modelis, maišyklė ir našumas viešai nenurodyti; oficialioje nuotraukoje matomi 2 silosai.</t>
         </is>
       </c>
       <c r="U70" s="5" t="n">
@@ -8507,17 +8507,17 @@
       </c>
       <c r="X70" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/NxQohpnzv1q9DA6CA?g_st=ac</t>
+          <t>https://www.ponasbetonas.lt/</t>
         </is>
       </c>
       <c r="Y70" s="2" t="inlineStr">
         <is>
-          <t>Nuosavas betono mazgas ir prekinio betono gamyba patvirtinti oficialiame įmonės puslapyje. Tiksli mazgo lokacija paimta iš naudotojo pateiktos Google Maps nuorodos; vietovė patikslinta pagal OpenStreetMap. Įmonės kodas patvirtintas Registrų centro viešame juridinio asmens pranešime.</t>
+          <t>Nuosavas betono mazgas ir prekinio betono gamyba patvirtinti oficialiame įmonės puslapyje. Mazgo gamintojas nustatytas pagal oficialaus puslapio hero nuotraukoje ant silosų matomą ELKON ženklinimą; modelis, maišyklė ir našumas viešai nenurodyti. Tiksli mazgo lokacija paimta iš naudotojo pateiktos Google Maps nuorodos; vietovė patikslinta pagal OpenStreetMap. Įmonės kodas patvirtintas Registrų centro viešame juridinio asmens pranešime.</t>
         </is>
       </c>
       <c r="Z70" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -8611,7 +8611,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-14T04:36:38.879321+00:00</t>
+          <t>2026-09-14T04:47:15.098822+00:00</t>
         </is>
       </c>
     </row>
@@ -8666,7 +8666,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-14T04:36:38.880373+00:00</t>
+          <t>2026-09-14T04:47:15.100829+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Update competitor map data
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$70</definedName>
@@ -8611,7 +8611,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-14T04:47:15.098822+00:00</t>
+          <t>2026-09-14T10:18:58.753253+00:00</t>
         </is>
       </c>
     </row>
@@ -8666,7 +8666,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-14T04:47:15.100829+00:00</t>
+          <t>2026-09-14T10:18:58.753936+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Move Heidelberg Siaures plant to Glaudenai
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$70</definedName>
@@ -510,7 +510,7 @@
     <col width="42" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
     <col width="32" customWidth="1" min="15" max="15"/>
-    <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="42" customWidth="1" min="16" max="16"/>
     <col width="32" customWidth="1" min="17" max="17"/>
     <col width="30" customWidth="1" min="18" max="18"/>
     <col width="34" customWidth="1" min="19" max="19"/>
@@ -1777,38 +1777,38 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Vilnius</t>
+          <t>Glaudėnai</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus m. sav.</t>
+          <t>Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Šiaurės g. 2, Vilnius</t>
+          <t>Glaudėnų k., Sendvario sen., Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="I11" s="3" t="n">
-        <v>54.6921358</v>
+        <v>55.774886</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>25.3937728</v>
+        <v>21.160809</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas; adresas patikslintas reverse-geokodavimu</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>Naudotojo pateikta Google Maps lokacija</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://maps.app.goo.gl/WuHkJbkmPjqkPWgL8</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus betono gamykla, Šiaurės g.</t>
+          <t>Heidelberg Materials betono gamykla, Glaudėnai</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr"/>
@@ -1831,7 +1831,7 @@
       <c r="S11" s="4" t="inlineStr"/>
       <c r="T11" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Vilniuje.</t>
+          <t>Heidelberg Materials betono gamyklų tinklo taškas perkeltas iš Šiaurės g. 2, Vilnius į naudotojo pateiktą Google Maps lokaciją Glaudėnų k., Sendvario sen., Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="U11" s="5" t="n">
@@ -1849,17 +1849,17 @@
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+          <t>https://maps.app.goo.gl/WuHkJbkmPjqkPWgL8</t>
         </is>
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+          <t>Perkelta iš Šiaurės g. 2, Vilnius į naudotojo pateiktą Google Maps lokaciją. Google Maps nuoroda išsisprendė į koordinates 55.774886, 21.160809; vietovė patikslinta reverse-geokodavimu kaip Glaudėnų k., Sendvario sen., Klaipėdos r. sav. Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis paliktas kaip įmonės šaltinis.</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -8611,7 +8611,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-21T10:23:24.887386+00:00</t>
+          <t>2026-09-23T07:20:42.186376+00:00</t>
         </is>
       </c>
     </row>
@@ -8666,7 +8666,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-21T10:23:24.888084+00:00</t>
+          <t>2026-09-23T07:20:42.187391+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Update competitor points and add Zariju drive zone
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z70" headerRowCount="1">
-  <autoFilter ref="A1:Z70"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z68" headerRowCount="1">
+  <autoFilter ref="A1:Z68"/>
   <tableColumns count="26">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z70"/>
+  <dimension ref="A1:Z68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -6134,49 +6134,49 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>sausta-trakai</t>
+          <t>ginfa-kutiskiai</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>145744638</t>
+          <t>302680943</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>UAB Sausta</t>
+          <t>UAB GinFa</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Sausta</t>
+          <t>GinFa</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta</t>
+          <t>Papildomai rasta EVRK 23.63</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Trakai</t>
+          <t>Kutiškiai</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Trakų r. sav.</t>
+          <t>Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Karaimų g. 73, Trakai</t>
+          <t>Alyvų g. 8, Kutiškiai, Radviliškio r.</t>
         </is>
       </c>
       <c r="I50" s="3" t="n">
-        <v>54.6523614</v>
+        <v>55.8326273</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>24.9221724</v>
+        <v>23.4995317</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
@@ -6205,7 +6205,7 @@
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>Sausta betono mišinių veikla</t>
+          <t>GinFa betono gamyba</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr"/>
@@ -6213,26 +6213,22 @@
       <c r="S50" s="4" t="inlineStr"/>
       <c r="T50" s="2" t="inlineStr">
         <is>
-          <t>Viešame kataloge įmonė siejama su betono mišinių veikla.</t>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
       <c r="U50" s="5" t="n">
-        <v>0.62</v>
+        <v>0.82</v>
       </c>
       <c r="V50" s="2" t="inlineStr"/>
       <c r="W50" s="2" t="inlineStr">
         <is>
-          <t>https://www.1551.lt/sausta-uab-240915/</t>
-        </is>
-      </c>
-      <c r="X50" s="2" t="inlineStr">
-        <is>
-          <t>https://www.1551.lt/sausta-uab-240915/</t>
-        </is>
-      </c>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="X50" s="2" t="inlineStr"/>
       <c r="Y50" s="2" t="inlineStr">
         <is>
-          <t>Žemos pasitikėjimo įrašas; reikia patikslinti, ar gamyba vykdoma šiame taške.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z50" s="2" t="inlineStr">
@@ -6244,22 +6240,22 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>ginfa-kutiskiai</t>
+          <t>antano-gribino-imone-prienai</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>302680943</t>
+          <t>170687267</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>UAB GinFa</t>
+          <t>IĮ Antano Gribino gamybos ir komercinės veiklos įmonė</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>GinFa</t>
+          <t>Antano Gribino įmonė</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -6269,24 +6265,24 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Kutiškiai</t>
+          <t>Prienai</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Radviliškio r. sav.</t>
+          <t>Prienų r. sav.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Alyvų g. 8, Kutiškiai, Radviliškio r.</t>
+          <t>Kęstučio g. 95A, Prienai</t>
         </is>
       </c>
       <c r="I51" s="3" t="n">
-        <v>55.8326273</v>
+        <v>54.6523184</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>23.4995317</v>
+        <v>23.9696591</v>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6311,7 @@
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
-          <t>GinFa betono gamyba</t>
+          <t>Antano Gribino įmonės betono gamyba</t>
         </is>
       </c>
       <c r="Q51" s="2" t="inlineStr"/>
@@ -6350,22 +6346,22 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>antano-gribino-imone-prienai</t>
+          <t>kelsera-anavilis</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>170687267</t>
+          <t>304642165</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>IĮ Antano Gribino gamybos ir komercinės veiklos įmonė</t>
+          <t>UAB Kelsera</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Antano Gribino įmonė</t>
+          <t>Kelsera</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -6375,24 +6371,24 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Prienai</t>
+          <t>Anavilis</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Prienų r. sav.</t>
+          <t>Vilniaus r. sav.</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Kęstučio g. 95A, Prienai</t>
+          <t>Bitininkų g. 13, Anavilis, Vilniaus r.</t>
         </is>
       </c>
       <c r="I52" s="3" t="n">
-        <v>54.6523184</v>
+        <v>54.9463928</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>23.9696591</v>
+        <v>25.216796</v>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
@@ -6421,7 +6417,7 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>Antano Gribino įmonės betono gamyba</t>
+          <t>Kelsera betono gamyba</t>
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr"/>
@@ -6456,22 +6452,22 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>kelsera-anavilis</t>
+          <t>vinido-taurage</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>304642165</t>
+          <t>306258220</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>UAB Kelsera</t>
+          <t>UAB Vinido</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Kelsera</t>
+          <t>Vinido</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -6481,24 +6477,24 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Anavilis</t>
+          <t>Tauragė</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus r. sav.</t>
+          <t>Tauragės r. sav.</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Bitininkų g. 13, Anavilis, Vilniaus r.</t>
+          <t>Gaurės g. 32, Tauragė</t>
         </is>
       </c>
       <c r="I53" s="3" t="n">
-        <v>54.9463928</v>
+        <v>55.2492204</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>25.216796</v>
+        <v>22.3185845</v>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6523,7 @@
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>Kelsera betono gamyba</t>
+          <t>Vinido betono gamyba</t>
         </is>
       </c>
       <c r="Q53" s="2" t="inlineStr"/>
@@ -6541,16 +6537,24 @@
       <c r="U53" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V53" s="2" t="inlineStr"/>
+      <c r="V53" s="2" t="inlineStr">
+        <is>
+          <t>https://betonastaurageje.lt/</t>
+        </is>
+      </c>
       <c r="W53" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X53" s="2" t="inlineStr"/>
+          <t>https://betonastaurageje.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X53" s="2" t="inlineStr">
+        <is>
+          <t>https://betonastaurageje.lt/betonas/</t>
+        </is>
+      </c>
       <c r="Y53" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Oficiali Vinido svetainė patvirtina Gaurės g. 32 adresą, betono gamybą ir betono mazgą.</t>
         </is>
       </c>
       <c r="Z53" s="2" t="inlineStr">
@@ -6562,22 +6566,22 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>vinido-taurage</t>
+          <t>santvara-kedainiai</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>306258220</t>
+          <t>304915297</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>UAB Vinido</t>
+          <t>UAB Santvara</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Vinido</t>
+          <t>Santvara</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -6587,24 +6591,24 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Tauragė</t>
+          <t>Kėdainiai</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Tauragės r. sav.</t>
+          <t>Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Gaurės g. 32, Tauragė</t>
+          <t>Aruodų g. 34, Kėdainiai</t>
         </is>
       </c>
       <c r="I54" s="3" t="n">
-        <v>55.2492204</v>
+        <v>55.2634747</v>
       </c>
       <c r="J54" s="3" t="n">
-        <v>22.3185845</v>
+        <v>23.9440384</v>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
@@ -6633,7 +6637,7 @@
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>Vinido betono gamyba</t>
+          <t>Santvara betono gamyba</t>
         </is>
       </c>
       <c r="Q54" s="2" t="inlineStr"/>
@@ -6649,22 +6653,22 @@
       </c>
       <c r="V54" s="2" t="inlineStr">
         <is>
-          <t>https://betonastaurageje.lt/</t>
+          <t>https://santvara.eu/</t>
         </is>
       </c>
       <c r="W54" s="2" t="inlineStr">
         <is>
-          <t>https://betonastaurageje.lt/kontaktai/</t>
+          <t>https://santvara.eu/</t>
         </is>
       </c>
       <c r="X54" s="2" t="inlineStr">
         <is>
-          <t>https://betonastaurageje.lt/betonas/</t>
+          <t>https://santvara.eu/</t>
         </is>
       </c>
       <c r="Y54" s="2" t="inlineStr">
         <is>
-          <t>Oficiali Vinido svetainė patvirtina Gaurės g. 32 adresą, betono gamybą ir betono mazgą.</t>
+          <t>Oficiali Santvara svetainė patvirtina Aruodų g. 34 adresą ir betono bei birių medžiagų veiklą.</t>
         </is>
       </c>
       <c r="Z54" s="2" t="inlineStr">
@@ -6676,22 +6680,22 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>santvara-kedainiai</t>
+          <t>medis-ir-betonas-naujoji-akmene</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>304915297</t>
+          <t>153074073</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>UAB Santvara</t>
+          <t>AB Medis ir betonas</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Santvara</t>
+          <t>Medis ir betonas</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -6701,24 +6705,24 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Kėdainiai</t>
+          <t>Naujoji Akmenė</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Kėdainių r. sav.</t>
+          <t>Akmenės r. sav.</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Aruodų g. 34, Kėdainiai</t>
+          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
         </is>
       </c>
       <c r="I55" s="3" t="n">
-        <v>55.2634747</v>
+        <v>56.3143832</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>23.9440384</v>
+        <v>22.9130704</v>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
@@ -6747,7 +6751,7 @@
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>Santvara betono gamyba</t>
+          <t>Medis ir betonas gamyba</t>
         </is>
       </c>
       <c r="Q55" s="2" t="inlineStr"/>
@@ -6761,24 +6765,16 @@
       <c r="U55" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V55" s="2" t="inlineStr">
-        <is>
-          <t>https://santvara.eu/</t>
-        </is>
-      </c>
+      <c r="V55" s="2" t="inlineStr"/>
       <c r="W55" s="2" t="inlineStr">
         <is>
-          <t>https://santvara.eu/</t>
-        </is>
-      </c>
-      <c r="X55" s="2" t="inlineStr">
-        <is>
-          <t>https://santvara.eu/</t>
-        </is>
-      </c>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="X55" s="2" t="inlineStr"/>
       <c r="Y55" s="2" t="inlineStr">
         <is>
-          <t>Oficiali Santvara svetainė patvirtina Aruodų g. 34 adresą ir betono bei birių medžiagų veiklą.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z55" s="2" t="inlineStr">
@@ -6790,22 +6786,22 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>eurobetonas-visaginas</t>
+          <t>ekobetonas-marijampole</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>305191384</t>
+          <t>300636364</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>UAB Eurobetonas</t>
+          <t>UAB Ekobetonas</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Eurobetonas</t>
+          <t>Ekobetonas</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -6815,24 +6811,24 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Visaginas</t>
+          <t>Marijampolė</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Visagino sav.</t>
+          <t>Marijampolės sav.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Sandėlių g. 1, Karlų k., Visagino sav.</t>
+          <t>Gamyklų g. 3, Marijampolė</t>
         </is>
       </c>
       <c r="I56" s="3" t="n">
-        <v>55.5732062</v>
+        <v>54.5750142</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>26.4787145</v>
+        <v>23.3796805</v>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
@@ -6861,7 +6857,7 @@
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>Eurobetonas betono gamyba</t>
+          <t>Ekobetonas betono gamyba</t>
         </is>
       </c>
       <c r="Q56" s="2" t="inlineStr"/>
@@ -6873,18 +6869,26 @@
         </is>
       </c>
       <c r="U56" s="5" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="V56" s="2" t="inlineStr"/>
+        <v>0.82</v>
+      </c>
+      <c r="V56" s="2" t="inlineStr">
+        <is>
+          <t>https://ekobetonas.lt/</t>
+        </is>
+      </c>
       <c r="W56" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X56" s="2" t="inlineStr"/>
+          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
+        </is>
+      </c>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
+        </is>
+      </c>
       <c r="Y56" s="2" t="inlineStr">
         <is>
-          <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Visagino miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
+          <t>Oficialus Ekobetonas kontaktų puslapis patvirtina Gamyklų g. 3 adresą ir betono užsakymų kontaktus.</t>
         </is>
       </c>
       <c r="Z56" s="2" t="inlineStr">
@@ -6896,22 +6900,22 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>medis-ir-betonas-naujoji-akmene</t>
+          <t>rokbetonis-rokiskis</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>153074073</t>
+          <t>304184091</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>AB Medis ir betonas</t>
+          <t>MB Rokbetonis</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Medis ir betonas</t>
+          <t>Rokbetonis</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -6921,24 +6925,24 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Naujoji Akmenė</t>
+          <t>Rokiškis</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Akmenės r. sav.</t>
+          <t>Rokiškio r. sav.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
+          <t>Vydūno g. 12A, Parokiškė, Rokiškio r.</t>
         </is>
       </c>
       <c r="I57" s="3" t="n">
-        <v>56.3143832</v>
+        <v>55.9525796</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>22.9130704</v>
+        <v>25.5624197</v>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
@@ -6967,7 +6971,7 @@
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
-          <t>Medis ir betonas gamyba</t>
+          <t>Rokbetonis betono gamyba</t>
         </is>
       </c>
       <c r="Q57" s="2" t="inlineStr"/>
@@ -6979,7 +6983,7 @@
         </is>
       </c>
       <c r="U57" s="5" t="n">
-        <v>0.82</v>
+        <v>0.72</v>
       </c>
       <c r="V57" s="2" t="inlineStr"/>
       <c r="W57" s="2" t="inlineStr">
@@ -6990,7 +6994,7 @@
       <c r="X57" s="2" t="inlineStr"/>
       <c r="Y57" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Rokiškio miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
         </is>
       </c>
       <c r="Z57" s="2" t="inlineStr">
@@ -7002,22 +7006,22 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>ekobetonas-marijampole</t>
+          <t>beton-eura-dovainonys</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>300636364</t>
+          <t>302745280</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>UAB Ekobetonas</t>
+          <t>UAB Beton Eura</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Ekobetonas</t>
+          <t>Beton Eura</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -7027,24 +7031,24 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Marijampolė</t>
+          <t>Dovainonys</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Marijampolės sav.</t>
+          <t>Kaišiadorių r. sav.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Gamyklų g. 3, Marijampolė</t>
+          <t>Žilvičių g. 2, Dovainonys, Kaišiadorių r.</t>
         </is>
       </c>
       <c r="I58" s="3" t="n">
-        <v>54.5750142</v>
+        <v>54.8395918</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>23.3796805</v>
+        <v>24.2360193</v>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
@@ -7073,7 +7077,7 @@
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>Ekobetonas betono gamyba</t>
+          <t>Beton Eura betono gamyba</t>
         </is>
       </c>
       <c r="Q58" s="2" t="inlineStr"/>
@@ -7089,22 +7093,22 @@
       </c>
       <c r="V58" s="2" t="inlineStr">
         <is>
-          <t>https://ekobetonas.lt/</t>
+          <t>https://www.betoneura.lt/</t>
         </is>
       </c>
       <c r="W58" s="2" t="inlineStr">
         <is>
-          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
+          <t>https://www.betoneura.lt/kontaktai/</t>
         </is>
       </c>
       <c r="X58" s="2" t="inlineStr">
         <is>
-          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
+          <t>https://www.betoneura.lt/kontaktai/</t>
         </is>
       </c>
       <c r="Y58" s="2" t="inlineStr">
         <is>
-          <t>Oficialus Ekobetonas kontaktų puslapis patvirtina Gamyklų g. 3 adresą ir betono užsakymų kontaktus.</t>
+          <t>Oficialus Beton Eura kontaktų puslapis patvirtina Žilvičių g. 2 adresą ir rekvizitus.</t>
         </is>
       </c>
       <c r="Z58" s="2" t="inlineStr">
@@ -7116,22 +7120,22 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>rokbetonis-rokiskis</t>
+          <t>silutes-betonas-silute</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>304184091</t>
+          <t>177392928</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>MB Rokbetonis</t>
+          <t>UAB Šilutės betonas</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Rokbetonis</t>
+          <t>Šilutės betonas</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -7141,24 +7145,24 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Rokiškis</t>
+          <t>Šilutė</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Rokiškio r. sav.</t>
+          <t>Šilutės r. sav.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Vydūno g. 12A, Parokiškė, Rokiškio r.</t>
+          <t>Ramučių g. 1, Šilutė</t>
         </is>
       </c>
       <c r="I59" s="3" t="n">
-        <v>55.9525796</v>
+        <v>55.3538641</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>25.5624197</v>
+        <v>21.4796635</v>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
@@ -7187,7 +7191,7 @@
       </c>
       <c r="P59" s="2" t="inlineStr">
         <is>
-          <t>Rokbetonis betono gamyba</t>
+          <t>Šilutės betono gamyba</t>
         </is>
       </c>
       <c r="Q59" s="2" t="inlineStr"/>
@@ -7199,7 +7203,7 @@
         </is>
       </c>
       <c r="U59" s="5" t="n">
-        <v>0.72</v>
+        <v>0.82</v>
       </c>
       <c r="V59" s="2" t="inlineStr"/>
       <c r="W59" s="2" t="inlineStr">
@@ -7207,10 +7211,14 @@
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="X59" s="2" t="inlineStr"/>
+      <c r="X59" s="2" t="inlineStr">
+        <is>
+          <t>https://fsaskaita.lt/imone/uzdaroji-akcine-bendrove-silutes-betonas-177392928</t>
+        </is>
+      </c>
       <c r="Y59" s="2" t="inlineStr">
         <is>
-          <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Rokiškio miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z59" s="2" t="inlineStr">
@@ -7222,22 +7230,22 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>beton-eura-dovainonys</t>
+          <t>kruszbet-lithuania-jure</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>302745280</t>
+          <t>305173596</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>UAB Beton Eura</t>
+          <t>UAB KRUSZBET Lithuania</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Beton Eura</t>
+          <t>KRUSZBET Lithuania</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -7247,24 +7255,24 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Dovainonys</t>
+          <t>Jūrė</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Kaišiadorių r. sav.</t>
+          <t>Kazlų Rūdos sav.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Žilvičių g. 2, Dovainonys, Kaišiadorių r.</t>
+          <t>Medelyno g. 30A, Jūrė, Kazlų Rūdos sav.</t>
         </is>
       </c>
       <c r="I60" s="3" t="n">
-        <v>54.8395918</v>
+        <v>54.7706307</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>24.2360193</v>
+        <v>23.4998409</v>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
@@ -7293,7 +7301,7 @@
       </c>
       <c r="P60" s="2" t="inlineStr">
         <is>
-          <t>Beton Eura betono gamyba</t>
+          <t>KRUSZBET Lithuania betono gamyba</t>
         </is>
       </c>
       <c r="Q60" s="2" t="inlineStr"/>
@@ -7307,24 +7315,16 @@
       <c r="U60" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V60" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betoneura.lt/</t>
-        </is>
-      </c>
+      <c r="V60" s="2" t="inlineStr"/>
       <c r="W60" s="2" t="inlineStr">
         <is>
-          <t>https://www.betoneura.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="X60" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betoneura.lt/kontaktai/</t>
-        </is>
-      </c>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="X60" s="2" t="inlineStr"/>
       <c r="Y60" s="2" t="inlineStr">
         <is>
-          <t>Oficialus Beton Eura kontaktų puslapis patvirtina Žilvičių g. 2 adresą ir rekvizitus.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z60" s="2" t="inlineStr">
@@ -7336,49 +7336,49 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>silutes-betonas-silute</t>
+          <t>telsiu-keliai-telsiai</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>177392928</t>
+          <t>180200843</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>UAB Šilutės betonas</t>
+          <t>UAB Telšių keliai</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>Šilutės betonas</t>
+          <t>Telšių keliai</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta EVRK 23.63</t>
+          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Šilutė</t>
+          <t>Telšiai</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Šilutės r. sav.</t>
+          <t>Telšių r. sav.</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Ramučių g. 1, Šilutė</t>
+          <t>Mažeikių g. 18, Telšiai</t>
         </is>
       </c>
       <c r="I61" s="3" t="n">
-        <v>55.3538641</v>
+        <v>56.0004158</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>21.4796635</v>
+        <v>22.2581129</v>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
@@ -7407,102 +7407,108 @@
       </c>
       <c r="P61" s="2" t="inlineStr">
         <is>
-          <t>Šilutės betono gamyba</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q61" s="2" t="inlineStr"/>
       <c r="R61" s="2" t="inlineStr"/>
-      <c r="S61" s="4" t="inlineStr"/>
+      <c r="S61" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T61" s="2" t="inlineStr">
         <is>
-          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai.</t>
         </is>
       </c>
       <c r="U61" s="5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="V61" s="2" t="inlineStr"/>
+        <v>0.86</v>
+      </c>
+      <c r="V61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/</t>
+        </is>
+      </c>
       <c r="W61" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
         </is>
       </c>
       <c r="X61" s="2" t="inlineStr">
         <is>
-          <t>https://fsaskaita.lt/imone/uzdaroji-akcine-bendrove-silutes-betonas-177392928</t>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
         </is>
       </c>
       <c r="Y61" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
         </is>
       </c>
       <c r="Z61" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>kruszbet-lithuania-jure</t>
+          <t>vpa-laistai</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>305173596</t>
+          <t>110185819</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>UAB KRUSZBET Lithuania</t>
+          <t>UAB V. Paulius &amp; Associates</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>KRUSZBET Lithuania</t>
+          <t>VPA</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta EVRK 23.63</t>
+          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Jūrė</t>
+          <t>Laistai</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Kazlų Rūdos sav.</t>
+          <t>Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Medelyno g. 30A, Jūrė, Kazlų Rūdos sav.</t>
+          <t>Stariškės g. 9, Laistų k., Dovilų sen., Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="I62" s="3" t="n">
-        <v>54.7706307</v>
+        <v>55.636908</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>23.4998409</v>
+        <v>21.209254</v>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Naudotojo pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>Google Maps nuoroda</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
         </is>
       </c>
       <c r="N62" s="2" t="inlineStr">
@@ -7517,98 +7523,116 @@
       </c>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t>KRUSZBET Lithuania betono gamyba</t>
-        </is>
-      </c>
-      <c r="Q62" s="2" t="inlineStr"/>
-      <c r="R62" s="2" t="inlineStr"/>
-      <c r="S62" s="4" t="inlineStr"/>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="inlineStr">
+        <is>
+          <t>3 m³</t>
+        </is>
+      </c>
+      <c r="R62" s="2" t="inlineStr">
+        <is>
+          <t>60-80 m³/h</t>
+        </is>
+      </c>
+      <c r="S62" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T62" s="2" t="inlineStr">
         <is>
-          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+          <t>VPA betono mazgas Klaipėdos rajone.</t>
         </is>
       </c>
       <c r="U62" s="5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="V62" s="2" t="inlineStr"/>
+        <v>0.7</v>
+      </c>
+      <c r="V62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vpa.lt/</t>
+        </is>
+      </c>
       <c r="W62" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X62" s="2" t="inlineStr"/>
+          <t>https://www.vpa.lt/?Kontaktai=</t>
+        </is>
+      </c>
+      <c r="X62" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+        </is>
+      </c>
       <c r="Y62" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Vieta nustatyta pagal naudotojo pateiktą Google Maps nuorodą. VPA kontaktų puslapis nurodo Stariškės g. 9, Laistų k. adresą. Techniniai mazgo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z62" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>telsiu-keliai-telsiai</t>
+          <t>c3-beton-baisogala</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>180200843</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>UAB Telšių keliai</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Telšių keliai</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
+          <t>Konkurentas</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Telšiai</t>
+          <t>Baisogala</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Telšių r. sav.</t>
+          <t>Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Mažeikių g. 18, Telšiai</t>
+          <t>Dvaro g., Baisogala, Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="I63" s="3" t="n">
-        <v>56.0004158</v>
+        <v>55.6372</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>22.2581129</v>
+        <v>23.7183</v>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>C3 Betonas oficialus puslapis</t>
         </is>
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="N63" s="2" t="inlineStr">
@@ -7623,108 +7647,118 @@
       </c>
       <c r="P63" s="2" t="inlineStr">
         <is>
-          <t>Elkon</t>
-        </is>
-      </c>
-      <c r="Q63" s="2" t="inlineStr"/>
-      <c r="R63" s="2" t="inlineStr"/>
-      <c r="S63" s="4" t="n">
-        <v>2</v>
+          <t>Baisiogala Plant</t>
+        </is>
+      </c>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="R63" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="S63" s="4" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
       </c>
       <c r="T63" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai.</t>
+          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
         </is>
       </c>
       <c r="U63" s="5" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="V63" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/</t>
+          <t>https://c3beton.com/</t>
         </is>
       </c>
       <c r="W63" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="X63" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="Y63" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
         </is>
       </c>
       <c r="Z63" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>vpa-laistai</t>
+          <t>c3-beton-martiniskis</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>110185819</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>UAB V. Paulius &amp; Associates</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>VPA</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
+          <t>Konkurentas</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Laistai</t>
+          <t>Martiniškis</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Klaipėdos r. sav.</t>
+          <t>Jonavos r. sav.</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Stariškės g. 9, Laistų k., Dovilų sen., Klaipėdos r. sav.</t>
+          <t>Vanagiškiai, Kulvos sen., Jonavos r. sav.</t>
         </is>
       </c>
       <c r="I64" s="3" t="n">
-        <v>55.636908</v>
+        <v>55.1441659</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>21.209254</v>
+        <v>24.1869636</v>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Naudotojo pateiktos Google Maps nuorodos taškas</t>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>Google Maps nuoroda</t>
+          <t>C3 Betonas oficialus puslapis</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
@@ -7739,60 +7773,62 @@
       </c>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>Liebherr</t>
+          <t>Martiniškis Plant</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>3 m³</t>
+          <t>Ammann Elba Euromix C120, 3 m³</t>
         </is>
       </c>
       <c r="R64" s="2" t="inlineStr">
         <is>
-          <t>60-80 m³/h</t>
-        </is>
-      </c>
-      <c r="S64" s="4" t="n">
-        <v>2</v>
+          <t>60–80 m³/val.</t>
+        </is>
+      </c>
+      <c r="S64" s="4" t="inlineStr">
+        <is>
+          <t>2x85 t</t>
+        </is>
       </c>
       <c r="T64" s="2" t="inlineStr">
         <is>
-          <t>VPA betono mazgas Klaipėdos rajone.</t>
+          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U64" s="5" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="V64" s="2" t="inlineStr">
         <is>
-          <t>https://www.vpa.lt/</t>
+          <t>https://c3beton.com/</t>
         </is>
       </c>
       <c r="W64" s="2" t="inlineStr">
         <is>
-          <t>https://www.vpa.lt/?Kontaktai=</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="X64" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="Y64" s="2" t="inlineStr">
         <is>
-          <t>Vieta nustatyta pagal naudotojo pateiktą Google Maps nuorodą. VPA kontaktų puslapis nurodo Stariškės g. 9, Laistų k. adresą. Techniniai mazgo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-baisogala</t>
+          <t>c3-beton-stasenai</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -7817,38 +7853,38 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Baisogala</t>
+          <t>Vilnius</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Radviliškio r. sav.</t>
+          <t>Vilniaus m. sav.</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Dvaro g., Baisogala, Radviliškio r. sav.</t>
+          <t>Ušos g. 21, Vilnius, 02121 Vilniaus m. sav.</t>
         </is>
       </c>
       <c r="I65" s="3" t="n">
-        <v>55.6372</v>
+        <v>54.6493094</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>23.7183</v>
+        <v>25.3107972</v>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
+          <t>Tikslus adreso taškas pagal geokodavimą</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas oficialus puslapis</t>
+          <t>ArcGIS geokodavimas pagal naudotojo pateiktą adresą</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://geocode.arcgis.com/arcgis/rest/services/World/GeocodeServer/findAddressCandidates</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
@@ -7863,27 +7899,27 @@
       </c>
       <c r="P65" s="2" t="inlineStr">
         <is>
-          <t>Baisiogala Plant</t>
+          <t>Vilnius Ušos g. Plant</t>
         </is>
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>Nissbau Euromix C120, 3 m³</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>60–80 m³/val.</t>
         </is>
       </c>
       <c r="S65" s="4" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>2x85 t</t>
         </is>
       </c>
       <c r="T65" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
+          <t>Betono mazgas Nissbau Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U65" s="5" t="n">
@@ -7906,7 +7942,7 @@
       </c>
       <c r="Y65" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
+          <t>Perkelta iš Stašėnų lokacijos į Ušos g. 21, Vilnius pagal naudotojo pateiktą informaciją. Maišyklė pervadinta į Nissbau Euromix C120, 3 m³. Koordinatės geokoduotos pagal naują adresą.</t>
         </is>
       </c>
       <c r="Z65" s="2" t="inlineStr">
@@ -7918,7 +7954,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-martiniskis</t>
+          <t>c3-beton-runeikiai</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -7943,24 +7979,24 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Martiniškis</t>
+          <t>Runeikiai</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Jonavos r. sav.</t>
+          <t>Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Vanagiškiai, Kulvos sen., Jonavos r. sav.</t>
+          <t>Paguiriai, Šėtos sen., Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="I66" s="3" t="n">
-        <v>55.1441659</v>
+        <v>55.3327393</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>24.1869636</v>
+        <v>24.3501308</v>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
@@ -7989,7 +8025,7 @@
       </c>
       <c r="P66" s="2" t="inlineStr">
         <is>
-          <t>Martiniškis Plant</t>
+          <t>Runeikiai Plant</t>
         </is>
       </c>
       <c r="Q66" s="2" t="inlineStr">
@@ -8044,22 +8080,22 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-stasenai</t>
+          <t>reljef-rukla</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>301731961</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas</t>
+          <t>UAB Reljef</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas</t>
+          <t>Reljef</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -8069,38 +8105,38 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Vilnius</t>
+          <t>Rukla</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus m. sav.</t>
+          <t>Jonavos r. sav.</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Ušos g. 21, Vilnius, 02121 Vilniaus m. sav.</t>
+          <t>Rukla, Jonavos r. sav.</t>
         </is>
       </c>
       <c r="I67" s="3" t="n">
-        <v>54.6493094</v>
+        <v>55.05225</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>25.3107972</v>
+        <v>24.4064167</v>
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas pagal geokodavimą</t>
+          <t>Tikslus naudotojo pateiktas taškas; adresas artimiausias pagal OpenStreetMap</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>ArcGIS geokodavimas pagal naudotojo pateiktą adresą</t>
+          <t>Naudotojo pateiktos koordinatės</t>
         </is>
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>https://geocode.arcgis.com/arcgis/rest/services/World/GeocodeServer/findAddressCandidates</t>
+          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
         </is>
       </c>
       <c r="N67" s="2" t="inlineStr">
@@ -8115,438 +8151,186 @@
       </c>
       <c r="P67" s="2" t="inlineStr">
         <is>
-          <t>Vilnius Ušos g. Plant</t>
+          <t>Ammann Elba</t>
         </is>
       </c>
       <c r="Q67" s="2" t="inlineStr">
         <is>
-          <t>Nissbau Euromix C120, 3 m³</t>
+          <t>Nenustatyta</t>
         </is>
       </c>
       <c r="R67" s="2" t="inlineStr">
         <is>
-          <t>60–80 m³/val.</t>
+          <t>Nenustatytas</t>
         </is>
       </c>
       <c r="S67" s="4" t="inlineStr">
         <is>
-          <t>2x85 t</t>
+          <t>2x65 t</t>
         </is>
       </c>
       <c r="T67" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgas Nissbau Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
+          <t>Rukloje veikiantis UAB Reljef betono mazgas: Ammann Elba, 2x65 t silosai. Maišyklė ir našumas nenustatyti.</t>
         </is>
       </c>
       <c r="U67" s="5" t="n">
-        <v>0.9</v>
+        <v>0.82</v>
       </c>
       <c r="V67" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/</t>
+          <t>https://www.reljef.lt/</t>
         </is>
       </c>
       <c r="W67" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.reljef.lt/</t>
         </is>
       </c>
       <c r="X67" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
         </is>
       </c>
       <c r="Y67" s="2" t="inlineStr">
         <is>
-          <t>Perkelta iš Stašėnų lokacijos į Ušos g. 21, Vilnius pagal naudotojo pateiktą informaciją. Maišyklė pervadinta į Nissbau Euromix C120, 3 m³. Koordinatės geokoduotos pagal naują adresą.</t>
+          <t>Įmonės rekvizitai paimti iš oficialaus UAB Reljef puslapio. Betono mazgo gamintojas, silosai ir lokacija įrašyti pagal naudotojo pateiktą informaciją. Artimiausias viešai geokoduotas adresas nustatytas pagal OpenStreetMap.</t>
         </is>
       </c>
       <c r="Z67" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-runeikiai</t>
+          <t>ponas-betonas-paraudondvariai</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
+          <t>306676006</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>UAB Ponas betonas</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Ponas betonas</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Konkurentas</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Paraudondvariai</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Vilniaus r. sav.</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Vilniaus g., Paraudondvariai, Riešės sen., Vilniaus r. sav.</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="n">
+        <v>54.8321418</v>
+      </c>
+      <c r="J68" s="3" t="n">
+        <v>25.2755596</v>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>Naudotojo pateikta Google Maps lokacija</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/NxQohpnzv1q9DA6CA?g_st=ac</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>Elkon</t>
+        </is>
+      </c>
+      <c r="Q68" s="2" t="inlineStr">
+        <is>
           <t>Nenurodyta viešai</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>C3 Betonas</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>C3 Betonas</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>Konkurentas</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>Runeikiai</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>Kėdainių r. sav.</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>Paguiriai, Šėtos sen., Kėdainių r. sav.</t>
-        </is>
-      </c>
-      <c r="I68" s="3" t="n">
-        <v>55.3327393</v>
-      </c>
-      <c r="J68" s="3" t="n">
-        <v>24.3501308</v>
-      </c>
-      <c r="K68" s="2" t="inlineStr">
-        <is>
-          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
-        </is>
-      </c>
-      <c r="L68" s="2" t="inlineStr">
-        <is>
-          <t>C3 Betonas oficialus puslapis</t>
-        </is>
-      </c>
-      <c r="M68" s="2" t="inlineStr">
-        <is>
-          <t>https://c3beton.com/lt/betonas</t>
-        </is>
-      </c>
-      <c r="N68" s="2" t="inlineStr">
-        <is>
-          <t>ready_mix_concrete</t>
-        </is>
-      </c>
-      <c r="O68" s="2" t="inlineStr">
-        <is>
-          <t>Betono mišiniai</t>
-        </is>
-      </c>
-      <c r="P68" s="2" t="inlineStr">
-        <is>
-          <t>Runeikiai Plant</t>
-        </is>
-      </c>
-      <c r="Q68" s="2" t="inlineStr">
-        <is>
-          <t>Ammann Elba Euromix C120, 3 m³</t>
-        </is>
-      </c>
       <c r="R68" s="2" t="inlineStr">
         <is>
-          <t>60–80 m³/val.</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="S68" s="4" t="inlineStr">
         <is>
-          <t>2x85 t</t>
+          <t>2 matomi oficialioje nuotraukoje</t>
         </is>
       </c>
       <c r="T68" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
+          <t>Oficialiame UAB Ponas betonas puslapyje nurodoma, kad įmonė turi nuosavą betono mazgą, gamina prekinį betoną ir jį pristato. Puslapio hero nuotraukoje ant silosų matomas ELKON ženklinimas, todėl mazgo gamintojas identifikuotas kaip Elkon. Konkretus modelis, maišyklė ir našumas viešai nenurodyti; oficialioje nuotraukoje matomi 2 silosai.</t>
         </is>
       </c>
       <c r="U68" s="5" t="n">
-        <v>0.9</v>
+        <v>0.98</v>
       </c>
       <c r="V68" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/</t>
+          <t>https://www.ponasbetonas.lt/</t>
         </is>
       </c>
       <c r="W68" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.ponasbetonas.lt/#Apiemus</t>
         </is>
       </c>
       <c r="X68" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.ponasbetonas.lt/</t>
         </is>
       </c>
       <c r="Y68" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Nuosavas betono mazgas ir prekinio betono gamyba patvirtinti oficialiame įmonės puslapyje. Mazgo gamintojas nustatytas pagal oficialaus puslapio hero nuotraukoje ant silosų matomą ELKON ženklinimą; modelis, maišyklė ir našumas viešai nenurodyti. Tiksli mazgo lokacija paimta iš naudotojo pateiktos Google Maps nuorodos; vietovė patikslinta pagal OpenStreetMap. Įmonės kodas patvirtintas Registrų centro viešame juridinio asmens pranešime.</t>
         </is>
       </c>
       <c r="Z68" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>reljef-rukla</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>301731961</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>UAB Reljef</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>Reljef</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>Konkurentas</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>Rukla</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="inlineStr">
-        <is>
-          <t>Jonavos r. sav.</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>Rukla, Jonavos r. sav.</t>
-        </is>
-      </c>
-      <c r="I69" s="3" t="n">
-        <v>55.05225</v>
-      </c>
-      <c r="J69" s="3" t="n">
-        <v>24.4064167</v>
-      </c>
-      <c r="K69" s="2" t="inlineStr">
-        <is>
-          <t>Tikslus naudotojo pateiktas taškas; adresas artimiausias pagal OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="L69" s="2" t="inlineStr">
-        <is>
-          <t>Naudotojo pateiktos koordinatės</t>
-        </is>
-      </c>
-      <c r="M69" s="2" t="inlineStr">
-        <is>
-          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
-        </is>
-      </c>
-      <c r="N69" s="2" t="inlineStr">
-        <is>
-          <t>ready_mix_concrete</t>
-        </is>
-      </c>
-      <c r="O69" s="2" t="inlineStr">
-        <is>
-          <t>Betono mišiniai</t>
-        </is>
-      </c>
-      <c r="P69" s="2" t="inlineStr">
-        <is>
-          <t>Ammann Elba</t>
-        </is>
-      </c>
-      <c r="Q69" s="2" t="inlineStr">
-        <is>
-          <t>Nenustatyta</t>
-        </is>
-      </c>
-      <c r="R69" s="2" t="inlineStr">
-        <is>
-          <t>Nenustatytas</t>
-        </is>
-      </c>
-      <c r="S69" s="4" t="inlineStr">
-        <is>
-          <t>2x65 t</t>
-        </is>
-      </c>
-      <c r="T69" s="2" t="inlineStr">
-        <is>
-          <t>Rukloje veikiantis UAB Reljef betono mazgas: Ammann Elba, 2x65 t silosai. Maišyklė ir našumas nenustatyti.</t>
-        </is>
-      </c>
-      <c r="U69" s="5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="V69" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reljef.lt/</t>
-        </is>
-      </c>
-      <c r="W69" s="2" t="inlineStr">
-        <is>
-          <t>https://www.reljef.lt/</t>
-        </is>
-      </c>
-      <c r="X69" s="2" t="inlineStr">
-        <is>
-          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
-        </is>
-      </c>
-      <c r="Y69" s="2" t="inlineStr">
-        <is>
-          <t>Įmonės rekvizitai paimti iš oficialaus UAB Reljef puslapio. Betono mazgo gamintojas, silosai ir lokacija įrašyti pagal naudotojo pateiktą informaciją. Artimiausias viešai geokoduotas adresas nustatytas pagal OpenStreetMap.</t>
-        </is>
-      </c>
-      <c r="Z69" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>ponas-betonas-paraudondvariai</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>306676006</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>UAB Ponas betonas</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>Ponas betonas</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>Konkurentas</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>Paraudondvariai</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>Vilniaus r. sav.</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>Vilniaus g., Paraudondvariai, Riešės sen., Vilniaus r. sav.</t>
-        </is>
-      </c>
-      <c r="I70" s="3" t="n">
-        <v>54.8321418</v>
-      </c>
-      <c r="J70" s="3" t="n">
-        <v>25.2755596</v>
-      </c>
-      <c r="K70" s="2" t="inlineStr">
-        <is>
-          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
-        </is>
-      </c>
-      <c r="L70" s="2" t="inlineStr">
-        <is>
-          <t>Naudotojo pateikta Google Maps lokacija</t>
-        </is>
-      </c>
-      <c r="M70" s="2" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/NxQohpnzv1q9DA6CA?g_st=ac</t>
-        </is>
-      </c>
-      <c r="N70" s="2" t="inlineStr">
-        <is>
-          <t>ready_mix_concrete</t>
-        </is>
-      </c>
-      <c r="O70" s="2" t="inlineStr">
-        <is>
-          <t>Betono mišiniai</t>
-        </is>
-      </c>
-      <c r="P70" s="2" t="inlineStr">
-        <is>
-          <t>Elkon</t>
-        </is>
-      </c>
-      <c r="Q70" s="2" t="inlineStr">
-        <is>
-          <t>Nenurodyta viešai</t>
-        </is>
-      </c>
-      <c r="R70" s="2" t="inlineStr">
-        <is>
-          <t>Nenurodyta viešai</t>
-        </is>
-      </c>
-      <c r="S70" s="4" t="inlineStr">
-        <is>
-          <t>2 matomi oficialioje nuotraukoje</t>
-        </is>
-      </c>
-      <c r="T70" s="2" t="inlineStr">
-        <is>
-          <t>Oficialiame UAB Ponas betonas puslapyje nurodoma, kad įmonė turi nuosavą betono mazgą, gamina prekinį betoną ir jį pristato. Puslapio hero nuotraukoje ant silosų matomas ELKON ženklinimas, todėl mazgo gamintojas identifikuotas kaip Elkon. Konkretus modelis, maišyklė ir našumas viešai nenurodyti; oficialioje nuotraukoje matomi 2 silosai.</t>
-        </is>
-      </c>
-      <c r="U70" s="5" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="V70" s="2" t="inlineStr">
-        <is>
-          <t>https://www.ponasbetonas.lt/</t>
-        </is>
-      </c>
-      <c r="W70" s="2" t="inlineStr">
-        <is>
-          <t>https://www.ponasbetonas.lt/#Apiemus</t>
-        </is>
-      </c>
-      <c r="X70" s="2" t="inlineStr">
-        <is>
-          <t>https://www.ponasbetonas.lt/</t>
-        </is>
-      </c>
-      <c r="Y70" s="2" t="inlineStr">
-        <is>
-          <t>Nuosavas betono mazgas ir prekinio betono gamyba patvirtinti oficialiame įmonės puslapyje. Mazgo gamintojas nustatytas pagal oficialaus puslapio hero nuotraukoje ant silosų matomą ELKON ženklinimą; modelis, maišyklė ir našumas viešai nenurodyti. Tiksli mazgo lokacija paimta iš naudotojo pateiktos Google Maps nuorodos; vietovė patikslinta pagal OpenStreetMap. Įmonės kodas patvirtintas Registrų centro viešame juridinio asmens pranešime.</t>
-        </is>
-      </c>
-      <c r="Z70" s="2" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z70"/>
+  <autoFilter ref="A1:Z68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8635,7 +8419,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-23T07:39:37.605548+00:00</t>
+          <t>2026-09-23T08:39:21.239190+00:00</t>
         </is>
       </c>
     </row>
@@ -8690,7 +8474,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-23T07:39:37.605548+00:00</t>
+          <t>2026-09-23T08:39:21.239190+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8704,7 +8488,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Pabrades concrete plant
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z67" headerRowCount="1">
-  <autoFilter ref="A1:Z67"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z68" headerRowCount="1">
+  <autoFilter ref="A1:Z68"/>
   <tableColumns count="26">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z67"/>
+  <dimension ref="A1:Z68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -8223,8 +8223,134 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>pabrades-betonas-pabrade</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>306177188</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>UAB Pabradės betonas</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Pabradės betonas</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Konkurentas</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Pabradė</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Švenčionių r. sav.</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Vilniaus g. 161, Pabradė, LT-18177 Švenčionių r.</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="n">
+        <v>54.9758768</v>
+      </c>
+      <c r="J68" s="3" t="n">
+        <v>25.7373849</v>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Tikslus oficialioje svetainėje pateiktos Google Maps nuorodos taškas</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>Oficiali Pabradės betono Google Maps nuoroda</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/TQBCVR8DczDRvQaeA</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>Liebherr (tikėtina)</t>
+        </is>
+      </c>
+      <c r="Q68" s="2" t="inlineStr">
+        <is>
+          <t>3 m³</t>
+        </is>
+      </c>
+      <c r="R68" s="2" t="inlineStr">
+        <is>
+          <t>60 m³/val.</t>
+        </is>
+      </c>
+      <c r="S68" s="4" t="inlineStr">
+        <is>
+          <t>3x65 t</t>
+        </is>
+      </c>
+      <c r="T68" s="2" t="inlineStr">
+        <is>
+          <t>UAB Pabradės betonas Vilniaus g. 161, Pabradėje, gamina sertifikuotą normalųjį betoną ir oficialiai nurodo dirbanti 50 km spinduliu aplink Pabradę. Oficialios galerijos nuotraukose matoma stacionari gamybos bazė su trimis cemento silosais. Mazgo gamintojas tikėtinai Liebherr pagal oficialiose nuotraukose matomą Liebherr įrangą ir gamyklos konstrukcijos vizualinius požymius; gamintojo lentelė viešai neparodyta.</t>
+        </is>
+      </c>
+      <c r="U68" s="5" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="V68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pabradesbetonas.lt/</t>
+        </is>
+      </c>
+      <c r="W68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pabradesbetonas.lt/</t>
+        </is>
+      </c>
+      <c r="X68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pabradesbetonas.lt/galerija/</t>
+        </is>
+      </c>
+      <c r="Y68" s="2" t="inlineStr">
+        <is>
+          <t>Adresas, įmonės kodas ir betono gamyba patvirtinti oficialioje svetainėje bei viešame gamybos kontrolės sertifikate. Koordinatės paimtos iš oficialioje svetainėje pateiktos Google Maps nuorodos. Maišyklės tūris 3 m³, realus našumas 60 m³/val. ir silosai 3x65 t įrašyti pagal naudotojo pateiktą informaciją. Gamintojas Liebherr nurodytas kaip tikėtinas pagal oficialios galerijos nuotraukas; viešo gamintojo ženklinimo ant paties mazgo nerasta.</t>
+        </is>
+      </c>
+      <c r="Z68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z67"/>
+  <autoFilter ref="A1:Z68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8313,7 +8439,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-23T09:23:09.140754+00:00</t>
+          <t>2026-09-23T09:44:17.027476+00:00</t>
         </is>
       </c>
     </row>
@@ -8368,7 +8494,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-23T09:23:09.140754+00:00</t>
+          <t>2026-09-23T09:44:17.028490+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8382,7 +8508,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atnaujinti Heidelberg Sandeliu betono mazga
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -2047,19 +2047,31 @@
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus betono gamykla, Sandėlių g.</t>
-        </is>
-      </c>
-      <c r="Q13" s="2" t="inlineStr"/>
-      <c r="R13" s="2" t="inlineStr"/>
-      <c r="S13" s="4" t="inlineStr"/>
+          <t>Wiggert</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>Wiggertmixer MO80</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>30 m³/val.</t>
+        </is>
+      </c>
+      <c r="S13" s="4" t="inlineStr">
+        <is>
+          <t>3x75 t</t>
+        </is>
+      </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiamas Heidelberg Materials betono gamyklų tinklo taškas Vilniuje.</t>
+          <t>Sandėlių g. 16 veikiantis mobilus Wiggert betono mazgas su Wiggertmixer MO80 priverstinio maišymo maišykle. Oficialus PAV dokumentas nurodo 30 m³/val. našumą, tris po 75 t cemento silosus ir iki 20 000 m³ metinę gamybą.</t>
         </is>
       </c>
       <c r="U13" s="5" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="V13" s="2" t="inlineStr">
         <is>
@@ -2073,17 +2085,17 @@
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
-          <t>https://www.betonas.heidelbergmaterials.lt/lt/kontaktine-informacija-0</t>
+          <t>https://old.gamta.lt/files/PAV%20atranka_0905.docx</t>
         </is>
       </c>
       <c r="Y13" s="2" t="inlineStr">
         <is>
-          <t>Oficialus Heidelberg Materials Lietuva Betonas kontaktų puslapis patvirtina betono užsakymų padalinius Lietuvoje.</t>
+          <t>Padalinio adresas patvirtintas oficialiame Heidelberg Materials kontaktų puslapyje. Gamintojas, maišyklės modelis, našumas ir silosų talpa paimti iš oficialaus 2016 m. Aplinkos apsaugos agentūros PAV dokumento Sandėlių g. 16 mazgui. Naudotojo pateikta nuotrauka atitinka dokumente aprašytą mobilų mazgą.</t>
         </is>
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
@@ -8439,7 +8451,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-23T09:44:17.027476+00:00</t>
+          <t>2026-09-23T15:17:04.691715+00:00</t>
         </is>
       </c>
     </row>
@@ -8494,7 +8506,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-23T09:44:17.028490+00:00</t>
+          <t>2026-09-23T15:17:04.691715+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Pasalinti Vilniaus betono gaminiu taska
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z68" headerRowCount="1">
-  <autoFilter ref="A1:Z68"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z67" headerRowCount="1">
+  <autoFilter ref="A1:Z67"/>
   <tableColumns count="26">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
@@ -492,13 +492,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z68"/>
+  <dimension ref="A1:Z67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
@@ -5038,18 +5038,18 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>vilniaus-betono-gaminiai-vilnius</t>
+          <t>pamario-grupe-kalnuvenai</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr"/>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>UAB Vilniaus betono gaminiai</t>
+          <t>UAB Pamario grupė</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>HAUS / Vilniaus betono gaminiai</t>
+          <t>Pamario grupė</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -5059,24 +5059,24 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Vilnius</t>
+          <t>Kalnuvėnai</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus m. sav.</t>
+          <t>Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>A. Jakšto g. 5, Vilnius</t>
+          <t>Kaukėnų g. 12, Kalnuvėnai, Klaipėdos r.</t>
         </is>
       </c>
       <c r="I40" s="3" t="n">
-        <v>54.6888177</v>
+        <v>55.7905468</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>25.2756813</v>
+        <v>21.1471136</v>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
@@ -5095,17 +5095,17 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>precast_concrete</t>
+          <t>ready_mix_concrete</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>Betono gaminiai</t>
+          <t>Betono mišiniai</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus betono gaminiai</t>
+          <t>Pamario grupės betono mazgas</t>
         </is>
       </c>
       <c r="Q40" s="2" t="inlineStr"/>
@@ -5113,30 +5113,30 @@
       <c r="S40" s="4" t="inlineStr"/>
       <c r="T40" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiamas HAUS blokelių ir betono gaminių gamintojas.</t>
+          <t>Viešai skelbiama betono mišinių veikla Klaipėdos rajone.</t>
         </is>
       </c>
       <c r="U40" s="5" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="V40" s="2" t="inlineStr">
         <is>
-          <t>https://www.vbg.lt/</t>
+          <t>https://pamariogrupe.lt/</t>
         </is>
       </c>
       <c r="W40" s="2" t="inlineStr">
         <is>
-          <t>https://www.vbg.lt/</t>
+          <t>https://pamariogrupe.lt/</t>
         </is>
       </c>
       <c r="X40" s="2" t="inlineStr">
         <is>
-          <t>https://www.vbg.lt/</t>
+          <t>https://pamariogrupe.lt/</t>
         </is>
       </c>
       <c r="Y40" s="2" t="inlineStr">
         <is>
-          <t>Žemėlapyje naudotas viešai skelbiamas įmonės adresas; gamybos vietą reikia patikslinti.</t>
+          <t>Reikia patikslinti našumą ir gamybos režimą.</t>
         </is>
       </c>
       <c r="Z40" s="2" t="inlineStr">
@@ -5148,18 +5148,18 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>pamario-grupe-kalnuvenai</t>
+          <t>betono-zona-klaipeda</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr"/>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>UAB Pamario grupė</t>
+          <t>UAB Betono zona</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Pamario grupė</t>
+          <t>Betono zona</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -5169,24 +5169,24 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Kalnuvėnai</t>
+          <t>Klaipėda</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Klaipėdos r. sav.</t>
+          <t>Klaipėdos m. sav.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Kaukėnų g. 12, Kalnuvėnai, Klaipėdos r.</t>
+          <t>Dvaro g. 6, Klaipėda</t>
         </is>
       </c>
       <c r="I41" s="3" t="n">
-        <v>55.7905468</v>
+        <v>55.7549809</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>21.1471136</v>
+        <v>21.150509</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
@@ -5205,17 +5205,17 @@
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>ready_mix_concrete</t>
+          <t>precast_concrete</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>Betono mišiniai</t>
+          <t>Betono gaminiai</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>Pamario grupės betono mazgas</t>
+          <t>Betono zona</t>
         </is>
       </c>
       <c r="Q41" s="2" t="inlineStr"/>
@@ -5223,30 +5223,30 @@
       <c r="S41" s="4" t="inlineStr"/>
       <c r="T41" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono mišinių veikla Klaipėdos rajone.</t>
+          <t>Viešai skelbiama betono gaminių veikla Klaipėdoje.</t>
         </is>
       </c>
       <c r="U41" s="5" t="n">
-        <v>0.75</v>
+        <v>0.65</v>
       </c>
       <c r="V41" s="2" t="inlineStr">
         <is>
-          <t>https://pamariogrupe.lt/</t>
+          <t>https://betonozona.lt/</t>
         </is>
       </c>
       <c r="W41" s="2" t="inlineStr">
         <is>
-          <t>https://pamariogrupe.lt/</t>
+          <t>https://betonozona.lt/</t>
         </is>
       </c>
       <c r="X41" s="2" t="inlineStr">
         <is>
-          <t>https://pamariogrupe.lt/</t>
+          <t>https://betonozona.lt/</t>
         </is>
       </c>
       <c r="Y41" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti našumą ir gamybos režimą.</t>
+          <t>Patikrinti, ar įmonė pati gamina, ar tik prekiauja betono gaminiais.</t>
         </is>
       </c>
       <c r="Z41" s="2" t="inlineStr">
@@ -5258,18 +5258,22 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>betono-zona-klaipeda</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr"/>
+          <t>topbeton-panevezys</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>307083610</t>
+        </is>
+      </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>UAB Betono zona</t>
+          <t>UAB Topbeton</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Betono zona</t>
+          <t>Topbeton</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -5279,24 +5283,24 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Klaipėda</t>
+          <t>Panevėžys</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Klaipėdos m. sav.</t>
+          <t>Panevėžio m. sav.</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Dvaro g. 6, Klaipėda</t>
+          <t>Beržų g. 5C, Panevėžys</t>
         </is>
       </c>
       <c r="I42" s="3" t="n">
-        <v>55.7549809</v>
+        <v>55.7168572</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>21.150509</v>
+        <v>24.3617863</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -5315,17 +5319,17 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>precast_concrete</t>
+          <t>ready_mix_concrete</t>
         </is>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>Betono gaminiai</t>
+          <t>Betono mišiniai</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>Betono zona</t>
+          <t>Topbeton betono mazgas</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr"/>
@@ -5333,30 +5337,30 @@
       <c r="S42" s="4" t="inlineStr"/>
       <c r="T42" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono gaminių veikla Klaipėdoje.</t>
+          <t>Viešai skelbiama betono mišinių gamyba Panevėžyje.</t>
         </is>
       </c>
       <c r="U42" s="5" t="n">
-        <v>0.65</v>
+        <v>0.78</v>
       </c>
       <c r="V42" s="2" t="inlineStr">
         <is>
-          <t>https://betonozona.lt/</t>
+          <t>https://topbeton.lt/</t>
         </is>
       </c>
       <c r="W42" s="2" t="inlineStr">
         <is>
-          <t>https://betonozona.lt/</t>
+          <t>https://www.topbeton.lt/kontaktai/</t>
         </is>
       </c>
       <c r="X42" s="2" t="inlineStr">
         <is>
-          <t>https://betonozona.lt/</t>
+          <t>https://www.topbeton.lt/kontaktai/</t>
         </is>
       </c>
       <c r="Y42" s="2" t="inlineStr">
         <is>
-          <t>Patikrinti, ar įmonė pati gamina, ar tik prekiauja betono gaminiais.</t>
+          <t>Oficialus kontaktų puslapis patvirtina Beržų g. 5C adresą.</t>
         </is>
       </c>
       <c r="Z42" s="2" t="inlineStr">
@@ -5368,22 +5372,18 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>topbeton-panevezys</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>307083610</t>
-        </is>
-      </c>
+          <t>gelzbetonio-gamyba-panevezys</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr"/>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>UAB Topbeton</t>
+          <t>MB Gelžbetonio gamyba</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Topbeton</t>
+          <t>Gelžbetonio gamyba</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -5403,14 +5403,14 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Beržų g. 5C, Panevėžys</t>
+          <t>S. Kerbedžio g. 52, Panevėžys</t>
         </is>
       </c>
       <c r="I43" s="3" t="n">
-        <v>55.7168572</v>
+        <v>55.7409491</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>24.3617863</v>
+        <v>24.3803541</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
@@ -5429,17 +5429,17 @@
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>ready_mix_concrete</t>
+          <t>precast_concrete</t>
         </is>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>Betono mišiniai</t>
+          <t>Gelžbetonis</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>Topbeton betono mazgas</t>
+          <t>Gelžbetonio gamyba Panevėžyje</t>
         </is>
       </c>
       <c r="Q43" s="2" t="inlineStr"/>
@@ -5447,30 +5447,30 @@
       <c r="S43" s="4" t="inlineStr"/>
       <c r="T43" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono mišinių gamyba Panevėžyje.</t>
+          <t>Viešai skelbiama gelžbetonio gaminių gamyba Panevėžyje.</t>
         </is>
       </c>
       <c r="U43" s="5" t="n">
-        <v>0.78</v>
+        <v>0.72</v>
       </c>
       <c r="V43" s="2" t="inlineStr">
         <is>
-          <t>https://topbeton.lt/</t>
+          <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
       <c r="W43" s="2" t="inlineStr">
         <is>
-          <t>https://www.topbeton.lt/kontaktai/</t>
+          <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
       <c r="X43" s="2" t="inlineStr">
         <is>
-          <t>https://www.topbeton.lt/kontaktai/</t>
+          <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
       <c r="Y43" s="2" t="inlineStr">
         <is>
-          <t>Oficialus kontaktų puslapis patvirtina Beržų g. 5C adresą.</t>
+          <t>Reikia patikslinti ryšį su kitomis S. Kerbedžio g. 52 įmonėmis.</t>
         </is>
       </c>
       <c r="Z43" s="2" t="inlineStr">
@@ -5482,18 +5482,18 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>gelzbetonio-gamyba-panevezys</t>
+          <t>inroma-pakruojis</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr"/>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>MB Gelžbetonio gamyba</t>
+          <t>UAB Inroma</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Gelžbetonio gamyba</t>
+          <t>Inroma</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -5503,24 +5503,24 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Panevėžys</t>
+          <t>Pakruojis</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Panevėžio m. sav.</t>
+          <t>Pakruojo r. sav.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>S. Kerbedžio g. 52, Panevėžys</t>
+          <t>Pramonės g. 5B, Pakruojis</t>
         </is>
       </c>
       <c r="I44" s="3" t="n">
-        <v>55.7409491</v>
+        <v>55.9763263</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>24.3803541</v>
+        <v>23.8584712</v>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
@@ -5539,17 +5539,17 @@
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>precast_concrete</t>
+          <t>ready_mix_concrete</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>Gelžbetonis</t>
+          <t>Betono mišiniai</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>Gelžbetonio gamyba Panevėžyje</t>
+          <t>Inroma betono mazgas</t>
         </is>
       </c>
       <c r="Q44" s="2" t="inlineStr"/>
@@ -5557,7 +5557,7 @@
       <c r="S44" s="4" t="inlineStr"/>
       <c r="T44" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama gelžbetonio gaminių gamyba Panevėžyje.</t>
+          <t>Viešai skelbiama betono mišinių veikla Pakruojyje.</t>
         </is>
       </c>
       <c r="U44" s="5" t="n">
@@ -5565,22 +5565,22 @@
       </c>
       <c r="V44" s="2" t="inlineStr">
         <is>
-          <t>https://gelzbetoniogamyba.lt/</t>
+          <t>https://inroma.lt/</t>
         </is>
       </c>
       <c r="W44" s="2" t="inlineStr">
         <is>
-          <t>https://gelzbetoniogamyba.lt/</t>
+          <t>https://inroma.lt/</t>
         </is>
       </c>
       <c r="X44" s="2" t="inlineStr">
         <is>
-          <t>https://gelzbetoniogamyba.lt/</t>
+          <t>https://inroma.lt/</t>
         </is>
       </c>
       <c r="Y44" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti ryšį su kitomis S. Kerbedžio g. 52 įmonėmis.</t>
+          <t>Reikia patikslinti našumą.</t>
         </is>
       </c>
       <c r="Z44" s="2" t="inlineStr">
@@ -5592,18 +5592,22 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>inroma-pakruojis</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr"/>
+          <t>utenos-betonas-utena</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>300904691</t>
+        </is>
+      </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>UAB Inroma</t>
+          <t>UAB Utenos betonas</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Inroma</t>
+          <t>Utenos betonas</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -5613,24 +5617,24 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Pakruojis</t>
+          <t>Utena</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Pakruojo r. sav.</t>
+          <t>Utenos r. sav.</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Pramonės g. 5B, Pakruojis</t>
+          <t>Metalo g. 9B, Utena</t>
         </is>
       </c>
       <c r="I45" s="3" t="n">
-        <v>55.9763263</v>
+        <v>55.4947607</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>23.8584712</v>
+        <v>25.6225075</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -5659,7 +5663,7 @@
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>Inroma betono mazgas</t>
+          <t>Utenos betono mazgas</t>
         </is>
       </c>
       <c r="Q45" s="2" t="inlineStr"/>
@@ -5667,30 +5671,30 @@
       <c r="S45" s="4" t="inlineStr"/>
       <c r="T45" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono mišinių veikla Pakruojyje.</t>
+          <t>Viešai skelbiama betono mišinių veikla Utenoje.</t>
         </is>
       </c>
       <c r="U45" s="5" t="n">
-        <v>0.72</v>
+        <v>0.78</v>
       </c>
       <c r="V45" s="2" t="inlineStr">
         <is>
-          <t>https://inroma.lt/</t>
+          <t>https://utenosbetonas.lt/</t>
         </is>
       </c>
       <c r="W45" s="2" t="inlineStr">
         <is>
-          <t>https://inroma.lt/</t>
+          <t>https://www.utenosbetonas.lt/kontaktai/</t>
         </is>
       </c>
       <c r="X45" s="2" t="inlineStr">
         <is>
-          <t>https://inroma.lt/</t>
+          <t>https://www.utenosbetonas.lt/kontaktai/</t>
         </is>
       </c>
       <c r="Y45" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti našumą.</t>
+          <t>Oficialus kontaktų puslapis patvirtina Metalo g. 9B adresą.</t>
         </is>
       </c>
       <c r="Z45" s="2" t="inlineStr">
@@ -5702,22 +5706,22 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>utenos-betonas-utena</t>
+          <t>sbetonas-jonava</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>300904691</t>
+          <t>300902683</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>UAB Utenos betonas</t>
+          <t>UAB Sbetonas</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Utenos betonas</t>
+          <t>Sbetonas</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -5727,24 +5731,24 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Utena</t>
+          <t>Jonava</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Utenos r. sav.</t>
+          <t>Jonavos r. sav.</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Metalo g. 9B, Utena</t>
+          <t>Skarulių g. 58, Jonava</t>
         </is>
       </c>
       <c r="I46" s="3" t="n">
-        <v>55.4947607</v>
+        <v>55.0786452</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>25.6225075</v>
+        <v>24.3199072</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
@@ -5773,7 +5777,7 @@
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>Utenos betono mazgas</t>
+          <t>Sbetonas betono mazgas</t>
         </is>
       </c>
       <c r="Q46" s="2" t="inlineStr"/>
@@ -5781,7 +5785,7 @@
       <c r="S46" s="4" t="inlineStr"/>
       <c r="T46" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono mišinių veikla Utenoje.</t>
+          <t>Viešai skelbiama prekinio betono gamyba Jonavoje.</t>
         </is>
       </c>
       <c r="U46" s="5" t="n">
@@ -5789,22 +5793,22 @@
       </c>
       <c r="V46" s="2" t="inlineStr">
         <is>
-          <t>https://utenosbetonas.lt/</t>
+          <t>https://sbetonas.lt/</t>
         </is>
       </c>
       <c r="W46" s="2" t="inlineStr">
         <is>
-          <t>https://www.utenosbetonas.lt/kontaktai/</t>
+          <t>https://sbetonas.lt/</t>
         </is>
       </c>
       <c r="X46" s="2" t="inlineStr">
         <is>
-          <t>https://www.utenosbetonas.lt/kontaktai/</t>
+          <t>https://sbetonas.lt/</t>
         </is>
       </c>
       <c r="Y46" s="2" t="inlineStr">
         <is>
-          <t>Oficialus kontaktų puslapis patvirtina Metalo g. 9B adresą.</t>
+          <t>Papildomai rasta pagal prekinio betono požymį.</t>
         </is>
       </c>
       <c r="Z46" s="2" t="inlineStr">
@@ -5816,22 +5820,18 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>sbetonas-jonava</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>300902683</t>
-        </is>
-      </c>
+          <t>kalcitas-naujoji-akmene</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr"/>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>UAB Sbetonas</t>
+          <t>AB Kalcitas</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Sbetonas</t>
+          <t>Kalcitas</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -5841,24 +5841,24 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Jonava</t>
+          <t>Naujoji Akmenė</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Jonavos r. sav.</t>
+          <t>Akmenės r. sav.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Skarulių g. 58, Jonava</t>
+          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
         </is>
       </c>
       <c r="I47" s="3" t="n">
-        <v>55.0786452</v>
+        <v>56.3143832</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>24.3199072</v>
+        <v>22.9130704</v>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
@@ -5887,7 +5887,7 @@
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>Sbetonas betono mazgas</t>
+          <t>Kalcitas betono mišinių gamybos linija</t>
         </is>
       </c>
       <c r="Q47" s="2" t="inlineStr"/>
@@ -5895,30 +5895,26 @@
       <c r="S47" s="4" t="inlineStr"/>
       <c r="T47" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama prekinio betono gamyba Jonavoje.</t>
+          <t>Viešame kataloge nurodomi betonas, betono mišiniai ir betono gamybos linija Naujojoje Akmenėje.</t>
         </is>
       </c>
       <c r="U47" s="5" t="n">
         <v>0.78</v>
       </c>
-      <c r="V47" s="2" t="inlineStr">
-        <is>
-          <t>https://sbetonas.lt/</t>
-        </is>
-      </c>
+      <c r="V47" s="2" t="inlineStr"/>
       <c r="W47" s="2" t="inlineStr">
         <is>
-          <t>https://sbetonas.lt/</t>
+          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
         </is>
       </c>
       <c r="X47" s="2" t="inlineStr">
         <is>
-          <t>https://sbetonas.lt/</t>
+          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
         </is>
       </c>
       <c r="Y47" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta pagal prekinio betono požymį.</t>
+          <t>Reikia patikslinti, ar veikla yra nuolat aktyvi.</t>
         </is>
       </c>
       <c r="Z47" s="2" t="inlineStr">
@@ -5930,18 +5926,18 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>kalcitas-naujoji-akmene</t>
+          <t>gelgaudiskio-gelzbetonis-gelgaudiskis</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr"/>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>AB Kalcitas</t>
+          <t>UAB Gelgaudiškio gelžbetonis</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Kalcitas</t>
+          <t>Gelgaudiškio gelžbetonis</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -5951,24 +5947,24 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Naujoji Akmenė</t>
+          <t>Gelgaudiškis</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Akmenės r. sav.</t>
+          <t>Šakių r. sav.</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
+          <t>Vakarų g. 33 D, 71431, Gelgaudiškis</t>
         </is>
       </c>
       <c r="I48" s="3" t="n">
-        <v>56.3143832</v>
+        <v>55.07067</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>22.9130704</v>
+        <v>22.976723</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
@@ -5977,27 +5973,27 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>GLG kontaktų puslapis</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://glg.lt/kontaktai/</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>ready_mix_concrete</t>
+          <t>precast_concrete</t>
         </is>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>Betono mišiniai</t>
+          <t>Betono mišiniai ir gelžbetonis</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>Kalcitas betono mišinių gamybos linija</t>
+          <t>Gelgaudiškio gelžbetonio gamykla</t>
         </is>
       </c>
       <c r="Q48" s="2" t="inlineStr"/>
@@ -6005,26 +6001,30 @@
       <c r="S48" s="4" t="inlineStr"/>
       <c r="T48" s="2" t="inlineStr">
         <is>
-          <t>Viešame kataloge nurodomi betonas, betono mišiniai ir betono gamybos linija Naujojoje Akmenėje.</t>
+          <t>Įmonė gamina gelžbetonio gaminius, prekinį ir hidrotechninį betoną bei smėlbetonio mišinius.</t>
         </is>
       </c>
       <c r="U48" s="5" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="V48" s="2" t="inlineStr"/>
+        <v>0.9</v>
+      </c>
+      <c r="V48" s="2" t="inlineStr">
+        <is>
+          <t>https://glg.lt/</t>
+        </is>
+      </c>
       <c r="W48" s="2" t="inlineStr">
         <is>
-          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
+          <t>https://glg.lt/kontaktai/</t>
         </is>
       </c>
       <c r="X48" s="2" t="inlineStr">
         <is>
-          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
+          <t>https://glg.lt/betonas/betono-misiniai/</t>
         </is>
       </c>
       <c r="Y48" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti, ar veikla yra nuolat aktyvi.</t>
+          <t>Patikslinta pagal oficialų glg.lt kontaktų ir įmonės aprašymo puslapius.</t>
         </is>
       </c>
       <c r="Z48" s="2" t="inlineStr">
@@ -6036,45 +6036,49 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>gelgaudiskio-gelzbetonis-gelgaudiskis</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr"/>
+          <t>ginfa-kutiskiai</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>302680943</t>
+        </is>
+      </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>UAB Gelgaudiškio gelžbetonis</t>
+          <t>UAB GinFa</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Gelgaudiškio gelžbetonis</t>
+          <t>GinFa</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta</t>
+          <t>Papildomai rasta EVRK 23.63</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Gelgaudiškis</t>
+          <t>Kutiškiai</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Šakių r. sav.</t>
+          <t>Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Vakarų g. 33 D, 71431, Gelgaudiškis</t>
+          <t>Alyvų g. 8, Kutiškiai, Radviliškio r.</t>
         </is>
       </c>
       <c r="I49" s="3" t="n">
-        <v>55.07067</v>
+        <v>55.8326273</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>22.976723</v>
+        <v>23.4995317</v>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
@@ -6083,27 +6087,27 @@
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>GLG kontaktų puslapis</t>
+          <t>Lietuvos geolokatorius</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>https://glg.lt/kontaktai/</t>
+          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
         </is>
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>precast_concrete</t>
+          <t>ready_mix_concrete</t>
         </is>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>Betono mišiniai ir gelžbetonis</t>
+          <t>Betono mišiniai</t>
         </is>
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>Gelgaudiškio gelžbetonio gamykla</t>
+          <t>GinFa betono gamyba</t>
         </is>
       </c>
       <c r="Q49" s="2" t="inlineStr"/>
@@ -6111,30 +6115,22 @@
       <c r="S49" s="4" t="inlineStr"/>
       <c r="T49" s="2" t="inlineStr">
         <is>
-          <t>Įmonė gamina gelžbetonio gaminius, prekinį ir hidrotechninį betoną bei smėlbetonio mišinius.</t>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
       <c r="U49" s="5" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="V49" s="2" t="inlineStr">
-        <is>
-          <t>https://glg.lt/</t>
-        </is>
-      </c>
+        <v>0.82</v>
+      </c>
+      <c r="V49" s="2" t="inlineStr"/>
       <c r="W49" s="2" t="inlineStr">
         <is>
-          <t>https://glg.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="X49" s="2" t="inlineStr">
-        <is>
-          <t>https://glg.lt/betonas/betono-misiniai/</t>
-        </is>
-      </c>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="X49" s="2" t="inlineStr"/>
       <c r="Y49" s="2" t="inlineStr">
         <is>
-          <t>Patikslinta pagal oficialų glg.lt kontaktų ir įmonės aprašymo puslapius.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z49" s="2" t="inlineStr">
@@ -6146,22 +6142,22 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>ginfa-kutiskiai</t>
+          <t>antano-gribino-imone-prienai</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>302680943</t>
+          <t>170687267</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>UAB GinFa</t>
+          <t>IĮ Antano Gribino gamybos ir komercinės veiklos įmonė</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>GinFa</t>
+          <t>Antano Gribino įmonė</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -6171,24 +6167,24 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Kutiškiai</t>
+          <t>Prienai</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Radviliškio r. sav.</t>
+          <t>Prienų r. sav.</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Alyvų g. 8, Kutiškiai, Radviliškio r.</t>
+          <t>Kęstučio g. 95A, Prienai</t>
         </is>
       </c>
       <c r="I50" s="3" t="n">
-        <v>55.8326273</v>
+        <v>54.6523184</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>23.4995317</v>
+        <v>23.9696591</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
@@ -6217,7 +6213,7 @@
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>GinFa betono gamyba</t>
+          <t>Antano Gribino įmonės betono gamyba</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr"/>
@@ -6252,22 +6248,22 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>antano-gribino-imone-prienai</t>
+          <t>vinido-taurage</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>170687267</t>
+          <t>306258220</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>IĮ Antano Gribino gamybos ir komercinės veiklos įmonė</t>
+          <t>UAB Vinido</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Antano Gribino įmonė</t>
+          <t>Vinido</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -6277,24 +6273,24 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Prienai</t>
+          <t>Tauragė</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Prienų r. sav.</t>
+          <t>Tauragės r. sav.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Kęstučio g. 95A, Prienai</t>
+          <t>Gaurės g. 32, Tauragė</t>
         </is>
       </c>
       <c r="I51" s="3" t="n">
-        <v>54.6523184</v>
+        <v>55.2492204</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>23.9696591</v>
+        <v>22.3185845</v>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
@@ -6323,7 +6319,7 @@
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
-          <t>Antano Gribino įmonės betono gamyba</t>
+          <t>Vinido betono gamyba</t>
         </is>
       </c>
       <c r="Q51" s="2" t="inlineStr"/>
@@ -6337,16 +6333,24 @@
       <c r="U51" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V51" s="2" t="inlineStr"/>
+      <c r="V51" s="2" t="inlineStr">
+        <is>
+          <t>https://betonastaurageje.lt/</t>
+        </is>
+      </c>
       <c r="W51" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X51" s="2" t="inlineStr"/>
+          <t>https://betonastaurageje.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X51" s="2" t="inlineStr">
+        <is>
+          <t>https://betonastaurageje.lt/betonas/</t>
+        </is>
+      </c>
       <c r="Y51" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Oficiali Vinido svetainė patvirtina Gaurės g. 32 adresą, betono gamybą ir betono mazgą.</t>
         </is>
       </c>
       <c r="Z51" s="2" t="inlineStr">
@@ -6358,22 +6362,22 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>vinido-taurage</t>
+          <t>santvara-kedainiai</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>306258220</t>
+          <t>304915297</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>UAB Vinido</t>
+          <t>UAB Santvara</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Vinido</t>
+          <t>Santvara</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -6383,24 +6387,24 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Tauragė</t>
+          <t>Kėdainiai</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Tauragės r. sav.</t>
+          <t>Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Gaurės g. 32, Tauragė</t>
+          <t>Aruodų g. 34, Kėdainiai</t>
         </is>
       </c>
       <c r="I52" s="3" t="n">
-        <v>55.2492204</v>
+        <v>55.2634747</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>22.3185845</v>
+        <v>23.9440384</v>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
@@ -6429,7 +6433,7 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>Vinido betono gamyba</t>
+          <t>Santvara betono gamyba</t>
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr"/>
@@ -6445,22 +6449,22 @@
       </c>
       <c r="V52" s="2" t="inlineStr">
         <is>
-          <t>https://betonastaurageje.lt/</t>
+          <t>https://santvara.eu/</t>
         </is>
       </c>
       <c r="W52" s="2" t="inlineStr">
         <is>
-          <t>https://betonastaurageje.lt/kontaktai/</t>
+          <t>https://santvara.eu/</t>
         </is>
       </c>
       <c r="X52" s="2" t="inlineStr">
         <is>
-          <t>https://betonastaurageje.lt/betonas/</t>
+          <t>https://santvara.eu/</t>
         </is>
       </c>
       <c r="Y52" s="2" t="inlineStr">
         <is>
-          <t>Oficiali Vinido svetainė patvirtina Gaurės g. 32 adresą, betono gamybą ir betono mazgą.</t>
+          <t>Oficiali Santvara svetainė patvirtina Aruodų g. 34 adresą ir betono bei birių medžiagų veiklą.</t>
         </is>
       </c>
       <c r="Z52" s="2" t="inlineStr">
@@ -6472,22 +6476,22 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>santvara-kedainiai</t>
+          <t>medis-ir-betonas-naujoji-akmene</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>304915297</t>
+          <t>153074073</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>UAB Santvara</t>
+          <t>AB Medis ir betonas</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Santvara</t>
+          <t>Medis ir betonas</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -6497,24 +6501,24 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Kėdainiai</t>
+          <t>Naujoji Akmenė</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Kėdainių r. sav.</t>
+          <t>Akmenės r. sav.</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Aruodų g. 34, Kėdainiai</t>
+          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
         </is>
       </c>
       <c r="I53" s="3" t="n">
-        <v>55.2634747</v>
+        <v>56.3143832</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>23.9440384</v>
+        <v>22.9130704</v>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
@@ -6543,7 +6547,7 @@
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>Santvara betono gamyba</t>
+          <t>Medis ir betonas gamyba</t>
         </is>
       </c>
       <c r="Q53" s="2" t="inlineStr"/>
@@ -6557,24 +6561,16 @@
       <c r="U53" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V53" s="2" t="inlineStr">
-        <is>
-          <t>https://santvara.eu/</t>
-        </is>
-      </c>
+      <c r="V53" s="2" t="inlineStr"/>
       <c r="W53" s="2" t="inlineStr">
         <is>
-          <t>https://santvara.eu/</t>
-        </is>
-      </c>
-      <c r="X53" s="2" t="inlineStr">
-        <is>
-          <t>https://santvara.eu/</t>
-        </is>
-      </c>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="X53" s="2" t="inlineStr"/>
       <c r="Y53" s="2" t="inlineStr">
         <is>
-          <t>Oficiali Santvara svetainė patvirtina Aruodų g. 34 adresą ir betono bei birių medžiagų veiklą.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z53" s="2" t="inlineStr">
@@ -6586,22 +6582,22 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>medis-ir-betonas-naujoji-akmene</t>
+          <t>ekobetonas-marijampole</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>153074073</t>
+          <t>300636364</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>AB Medis ir betonas</t>
+          <t>UAB Ekobetonas</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Medis ir betonas</t>
+          <t>Ekobetonas</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -6611,24 +6607,24 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Naujoji Akmenė</t>
+          <t>Marijampolė</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Akmenės r. sav.</t>
+          <t>Marijampolės sav.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
+          <t>Gamyklų g. 3, Marijampolė</t>
         </is>
       </c>
       <c r="I54" s="3" t="n">
-        <v>56.3143832</v>
+        <v>54.5750142</v>
       </c>
       <c r="J54" s="3" t="n">
-        <v>22.9130704</v>
+        <v>23.3796805</v>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
@@ -6657,7 +6653,7 @@
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>Medis ir betonas gamyba</t>
+          <t>Ekobetonas betono gamyba</t>
         </is>
       </c>
       <c r="Q54" s="2" t="inlineStr"/>
@@ -6671,16 +6667,24 @@
       <c r="U54" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V54" s="2" t="inlineStr"/>
+      <c r="V54" s="2" t="inlineStr">
+        <is>
+          <t>https://ekobetonas.lt/</t>
+        </is>
+      </c>
       <c r="W54" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X54" s="2" t="inlineStr"/>
+          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
+        </is>
+      </c>
+      <c r="X54" s="2" t="inlineStr">
+        <is>
+          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
+        </is>
+      </c>
       <c r="Y54" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Oficialus Ekobetonas kontaktų puslapis patvirtina Gamyklų g. 3 adresą ir betono užsakymų kontaktus.</t>
         </is>
       </c>
       <c r="Z54" s="2" t="inlineStr">
@@ -6692,22 +6696,22 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>ekobetonas-marijampole</t>
+          <t>rokbetonis-rokiskis</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>300636364</t>
+          <t>304184091</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>UAB Ekobetonas</t>
+          <t>MB Rokbetonis</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Ekobetonas</t>
+          <t>Rokbetonis</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -6717,24 +6721,24 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Marijampolė</t>
+          <t>Rokiškis</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Marijampolės sav.</t>
+          <t>Rokiškio r. sav.</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Gamyklų g. 3, Marijampolė</t>
+          <t>Vydūno g. 12A, Parokiškė, Rokiškio r.</t>
         </is>
       </c>
       <c r="I55" s="3" t="n">
-        <v>54.5750142</v>
+        <v>55.9525796</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>23.3796805</v>
+        <v>25.5624197</v>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
@@ -6763,7 +6767,7 @@
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>Ekobetonas betono gamyba</t>
+          <t>Rokbetonis betono gamyba</t>
         </is>
       </c>
       <c r="Q55" s="2" t="inlineStr"/>
@@ -6775,26 +6779,18 @@
         </is>
       </c>
       <c r="U55" s="5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="V55" s="2" t="inlineStr">
-        <is>
-          <t>https://ekobetonas.lt/</t>
-        </is>
-      </c>
+        <v>0.72</v>
+      </c>
+      <c r="V55" s="2" t="inlineStr"/>
       <c r="W55" s="2" t="inlineStr">
         <is>
-          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
-        </is>
-      </c>
-      <c r="X55" s="2" t="inlineStr">
-        <is>
-          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
-        </is>
-      </c>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="X55" s="2" t="inlineStr"/>
       <c r="Y55" s="2" t="inlineStr">
         <is>
-          <t>Oficialus Ekobetonas kontaktų puslapis patvirtina Gamyklų g. 3 adresą ir betono užsakymų kontaktus.</t>
+          <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Rokiškio miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
         </is>
       </c>
       <c r="Z55" s="2" t="inlineStr">
@@ -6806,22 +6802,22 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>rokbetonis-rokiskis</t>
+          <t>beton-eura-dovainonys</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>304184091</t>
+          <t>302745280</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>MB Rokbetonis</t>
+          <t>UAB Beton Eura</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Rokbetonis</t>
+          <t>Beton Eura</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -6831,24 +6827,24 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Rokiškis</t>
+          <t>Dovainonys</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Rokiškio r. sav.</t>
+          <t>Kaišiadorių r. sav.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Vydūno g. 12A, Parokiškė, Rokiškio r.</t>
+          <t>Žilvičių g. 2, Dovainonys, Kaišiadorių r.</t>
         </is>
       </c>
       <c r="I56" s="3" t="n">
-        <v>55.9525796</v>
+        <v>54.8395918</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>25.5624197</v>
+        <v>24.2360193</v>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
@@ -6877,7 +6873,7 @@
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>Rokbetonis betono gamyba</t>
+          <t>Beton Eura betono gamyba</t>
         </is>
       </c>
       <c r="Q56" s="2" t="inlineStr"/>
@@ -6889,18 +6885,26 @@
         </is>
       </c>
       <c r="U56" s="5" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="V56" s="2" t="inlineStr"/>
+        <v>0.82</v>
+      </c>
+      <c r="V56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betoneura.lt/</t>
+        </is>
+      </c>
       <c r="W56" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X56" s="2" t="inlineStr"/>
+          <t>https://www.betoneura.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.betoneura.lt/kontaktai/</t>
+        </is>
+      </c>
       <c r="Y56" s="2" t="inlineStr">
         <is>
-          <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Rokiškio miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
+          <t>Oficialus Beton Eura kontaktų puslapis patvirtina Žilvičių g. 2 adresą ir rekvizitus.</t>
         </is>
       </c>
       <c r="Z56" s="2" t="inlineStr">
@@ -6912,22 +6916,22 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>beton-eura-dovainonys</t>
+          <t>silutes-betonas-silute</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>302745280</t>
+          <t>177392928</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>UAB Beton Eura</t>
+          <t>UAB Šilutės betonas</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Beton Eura</t>
+          <t>Šilutės betonas</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -6937,24 +6941,24 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Dovainonys</t>
+          <t>Šilutė</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Kaišiadorių r. sav.</t>
+          <t>Šilutės r. sav.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Žilvičių g. 2, Dovainonys, Kaišiadorių r.</t>
+          <t>Ramučių g. 1, Šilutė</t>
         </is>
       </c>
       <c r="I57" s="3" t="n">
-        <v>54.8395918</v>
+        <v>55.3538641</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>24.2360193</v>
+        <v>21.4796635</v>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
@@ -6983,7 +6987,7 @@
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
-          <t>Beton Eura betono gamyba</t>
+          <t>Šilutės betono gamyba</t>
         </is>
       </c>
       <c r="Q57" s="2" t="inlineStr"/>
@@ -6997,24 +7001,20 @@
       <c r="U57" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V57" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betoneura.lt/</t>
-        </is>
-      </c>
+      <c r="V57" s="2" t="inlineStr"/>
       <c r="W57" s="2" t="inlineStr">
         <is>
-          <t>https://www.betoneura.lt/kontaktai/</t>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
       <c r="X57" s="2" t="inlineStr">
         <is>
-          <t>https://www.betoneura.lt/kontaktai/</t>
+          <t>https://fsaskaita.lt/imone/uzdaroji-akcine-bendrove-silutes-betonas-177392928</t>
         </is>
       </c>
       <c r="Y57" s="2" t="inlineStr">
         <is>
-          <t>Oficialus Beton Eura kontaktų puslapis patvirtina Žilvičių g. 2 adresą ir rekvizitus.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z57" s="2" t="inlineStr">
@@ -7026,22 +7026,22 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>silutes-betonas-silute</t>
+          <t>kruszbet-lithuania-jure</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>177392928</t>
+          <t>305173596</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>UAB Šilutės betonas</t>
+          <t>UAB KRUSZBET Lithuania</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Šilutės betonas</t>
+          <t>KRUSZBET Lithuania</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -7051,24 +7051,24 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Šilutė</t>
+          <t>Jūrė</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Šilutės r. sav.</t>
+          <t>Kazlų Rūdos sav.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Ramučių g. 1, Šilutė</t>
+          <t>Medelyno g. 30A, Jūrė, Kazlų Rūdos sav.</t>
         </is>
       </c>
       <c r="I58" s="3" t="n">
-        <v>55.3538641</v>
+        <v>54.7706307</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>21.4796635</v>
+        <v>23.4998409</v>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
@@ -7097,7 +7097,7 @@
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>Šilutės betono gamyba</t>
+          <t>KRUSZBET Lithuania betono gamyba</t>
         </is>
       </c>
       <c r="Q58" s="2" t="inlineStr"/>
@@ -7117,11 +7117,7 @@
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="X58" s="2" t="inlineStr">
-        <is>
-          <t>https://fsaskaita.lt/imone/uzdaroji-akcine-bendrove-silutes-betonas-177392928</t>
-        </is>
-      </c>
+      <c r="X58" s="2" t="inlineStr"/>
       <c r="Y58" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
@@ -7136,49 +7132,49 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>kruszbet-lithuania-jure</t>
+          <t>telsiu-keliai-telsiai</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>305173596</t>
+          <t>180200843</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>UAB KRUSZBET Lithuania</t>
+          <t>UAB Telšių keliai</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>KRUSZBET Lithuania</t>
+          <t>Telšių keliai</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta EVRK 23.63</t>
+          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Jūrė</t>
+          <t>Telšiai</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Kazlų Rūdos sav.</t>
+          <t>Telšių r. sav.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Medelyno g. 30A, Jūrė, Kazlų Rūdos sav.</t>
+          <t>Mažeikių g. 18, Telšiai</t>
         </is>
       </c>
       <c r="I59" s="3" t="n">
-        <v>54.7706307</v>
+        <v>56.0004158</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>23.4998409</v>
+        <v>22.2581129</v>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
@@ -7207,57 +7203,67 @@
       </c>
       <c r="P59" s="2" t="inlineStr">
         <is>
-          <t>KRUSZBET Lithuania betono gamyba</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q59" s="2" t="inlineStr"/>
       <c r="R59" s="2" t="inlineStr"/>
-      <c r="S59" s="4" t="inlineStr"/>
+      <c r="S59" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T59" s="2" t="inlineStr">
         <is>
-          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai.</t>
         </is>
       </c>
       <c r="U59" s="5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="V59" s="2" t="inlineStr"/>
+        <v>0.86</v>
+      </c>
+      <c r="V59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/</t>
+        </is>
+      </c>
       <c r="W59" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X59" s="2" t="inlineStr"/>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+        </is>
+      </c>
+      <c r="X59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+        </is>
+      </c>
       <c r="Y59" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
         </is>
       </c>
       <c r="Z59" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>telsiu-keliai-telsiai</t>
+          <t>vpa-laistai</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>180200843</t>
+          <t>110185819</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>UAB Telšių keliai</t>
+          <t>UAB V. Paulius &amp; Associates</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Telšių keliai</t>
+          <t>VPA</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -7267,38 +7273,38 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Telšiai</t>
+          <t>Laistai</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Telšių r. sav.</t>
+          <t>Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Mažeikių g. 18, Telšiai</t>
+          <t>Stariškės g. 9, Laistų k., Dovilų sen., Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="I60" s="3" t="n">
-        <v>56.0004158</v>
+        <v>55.636908</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>22.2581129</v>
+        <v>21.209254</v>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Naudotojo pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>Google Maps nuoroda</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
@@ -7313,108 +7319,116 @@
       </c>
       <c r="P60" s="2" t="inlineStr">
         <is>
-          <t>Elkon</t>
-        </is>
-      </c>
-      <c r="Q60" s="2" t="inlineStr"/>
-      <c r="R60" s="2" t="inlineStr"/>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>3 m³</t>
+        </is>
+      </c>
+      <c r="R60" s="2" t="inlineStr">
+        <is>
+          <t>60-80 m³/h</t>
+        </is>
+      </c>
       <c r="S60" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T60" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai.</t>
+          <t>VPA betono mazgas Klaipėdos rajone.</t>
         </is>
       </c>
       <c r="U60" s="5" t="n">
-        <v>0.86</v>
+        <v>0.7</v>
       </c>
       <c r="V60" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/</t>
+          <t>https://www.vpa.lt/</t>
         </is>
       </c>
       <c r="W60" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+          <t>https://www.vpa.lt/?Kontaktai=</t>
         </is>
       </c>
       <c r="X60" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
         </is>
       </c>
       <c r="Y60" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
+          <t>Vieta nustatyta pagal naudotojo pateiktą Google Maps nuorodą. VPA kontaktų puslapis nurodo Stariškės g. 9, Laistų k. adresą. Techniniai mazgo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>vpa-laistai</t>
+          <t>c3-beton-baisogala</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>110185819</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>UAB V. Paulius &amp; Associates</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>VPA</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
+          <t>Konkurentas</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Laistai</t>
+          <t>Baisogala</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Klaipėdos r. sav.</t>
+          <t>Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Stariškės g. 9, Laistų k., Dovilų sen., Klaipėdos r. sav.</t>
+          <t>Dvaro g., Baisogala, Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="I61" s="3" t="n">
-        <v>55.636908</v>
+        <v>55.6372</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>21.209254</v>
+        <v>23.7183</v>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>Naudotojo pateiktos Google Maps nuorodos taškas</t>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>Google Maps nuoroda</t>
+          <t>C3 Betonas oficialus puslapis</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="N61" s="2" t="inlineStr">
@@ -7429,60 +7443,62 @@
       </c>
       <c r="P61" s="2" t="inlineStr">
         <is>
-          <t>Liebherr</t>
+          <t>Baisiogala Plant</t>
         </is>
       </c>
       <c r="Q61" s="2" t="inlineStr">
         <is>
-          <t>3 m³</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="R61" s="2" t="inlineStr">
         <is>
-          <t>60-80 m³/h</t>
-        </is>
-      </c>
-      <c r="S61" s="4" t="n">
-        <v>2</v>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="S61" s="4" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
       </c>
       <c r="T61" s="2" t="inlineStr">
         <is>
-          <t>VPA betono mazgas Klaipėdos rajone.</t>
+          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
         </is>
       </c>
       <c r="U61" s="5" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="V61" s="2" t="inlineStr">
         <is>
-          <t>https://www.vpa.lt/</t>
+          <t>https://c3beton.com/</t>
         </is>
       </c>
       <c r="W61" s="2" t="inlineStr">
         <is>
-          <t>https://www.vpa.lt/?Kontaktai=</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="X61" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="Y61" s="2" t="inlineStr">
         <is>
-          <t>Vieta nustatyta pagal naudotojo pateiktą Google Maps nuorodą. VPA kontaktų puslapis nurodo Stariškės g. 9, Laistų k. adresą. Techniniai mazgo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
         </is>
       </c>
       <c r="Z61" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-baisogala</t>
+          <t>c3-beton-martiniskis</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -7507,24 +7523,24 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Baisogala</t>
+          <t>Martiniškis</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Radviliškio r. sav.</t>
+          <t>Jonavos r. sav.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Dvaro g., Baisogala, Radviliškio r. sav.</t>
+          <t>Vanagiškiai, Kulvos sen., Jonavos r. sav.</t>
         </is>
       </c>
       <c r="I62" s="3" t="n">
-        <v>55.6372</v>
+        <v>55.1441659</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>23.7183</v>
+        <v>24.1869636</v>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
@@ -7553,27 +7569,27 @@
       </c>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t>Baisiogala Plant</t>
+          <t>Martiniškis Plant</t>
         </is>
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>Ammann Elba Euromix C120, 3 m³</t>
         </is>
       </c>
       <c r="R62" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>60–80 m³/val.</t>
         </is>
       </c>
       <c r="S62" s="4" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>2x85 t</t>
         </is>
       </c>
       <c r="T62" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
+          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U62" s="5" t="n">
@@ -7596,7 +7612,7 @@
       </c>
       <c r="Y62" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z62" s="2" t="inlineStr">
@@ -7608,7 +7624,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-martiniskis</t>
+          <t>c3-beton-stasenai</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -7633,38 +7649,38 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Martiniškis</t>
+          <t>Vilnius</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Jonavos r. sav.</t>
+          <t>Vilniaus m. sav.</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Vanagiškiai, Kulvos sen., Jonavos r. sav.</t>
+          <t>Ušos g. 21, Vilnius, 02121 Vilniaus m. sav.</t>
         </is>
       </c>
       <c r="I63" s="3" t="n">
-        <v>55.1441659</v>
+        <v>54.6493094</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>24.1869636</v>
+        <v>25.3107972</v>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
+          <t>Tikslus adreso taškas pagal geokodavimą</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas oficialus puslapis</t>
+          <t>ArcGIS geokodavimas pagal naudotojo pateiktą adresą</t>
         </is>
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://geocode.arcgis.com/arcgis/rest/services/World/GeocodeServer/findAddressCandidates</t>
         </is>
       </c>
       <c r="N63" s="2" t="inlineStr">
@@ -7679,12 +7695,12 @@
       </c>
       <c r="P63" s="2" t="inlineStr">
         <is>
-          <t>Martiniškis Plant</t>
+          <t>Vilnius Ušos g. Plant</t>
         </is>
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>Ammann Elba Euromix C120, 3 m³</t>
+          <t>Nissbau Euromix C120, 3 m³</t>
         </is>
       </c>
       <c r="R63" s="2" t="inlineStr">
@@ -7699,7 +7715,7 @@
       </c>
       <c r="T63" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
+          <t>Betono mazgas Nissbau Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U63" s="5" t="n">
@@ -7722,7 +7738,7 @@
       </c>
       <c r="Y63" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Perkelta iš Stašėnų lokacijos į Ušos g. 21, Vilnius pagal naudotojo pateiktą informaciją. Maišyklė pervadinta į Nissbau Euromix C120, 3 m³. Koordinatės geokoduotos pagal naują adresą.</t>
         </is>
       </c>
       <c r="Z63" s="2" t="inlineStr">
@@ -7734,7 +7750,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-stasenai</t>
+          <t>c3-beton-runeikiai</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -7759,38 +7775,38 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Vilnius</t>
+          <t>Runeikiai</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus m. sav.</t>
+          <t>Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Ušos g. 21, Vilnius, 02121 Vilniaus m. sav.</t>
+          <t>Paguiriai, Šėtos sen., Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="I64" s="3" t="n">
-        <v>54.6493094</v>
+        <v>55.3327393</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>25.3107972</v>
+        <v>24.3501308</v>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas pagal geokodavimą</t>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>ArcGIS geokodavimas pagal naudotojo pateiktą adresą</t>
+          <t>C3 Betonas oficialus puslapis</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>https://geocode.arcgis.com/arcgis/rest/services/World/GeocodeServer/findAddressCandidates</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
@@ -7805,12 +7821,12 @@
       </c>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>Vilnius Ušos g. Plant</t>
+          <t>Runeikiai Plant</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>Nissbau Euromix C120, 3 m³</t>
+          <t>Ammann Elba Euromix C120, 3 m³</t>
         </is>
       </c>
       <c r="R64" s="2" t="inlineStr">
@@ -7825,7 +7841,7 @@
       </c>
       <c r="T64" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgas Nissbau Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
+          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U64" s="5" t="n">
@@ -7848,7 +7864,7 @@
       </c>
       <c r="Y64" s="2" t="inlineStr">
         <is>
-          <t>Perkelta iš Stašėnų lokacijos į Ušos g. 21, Vilnius pagal naudotojo pateiktą informaciją. Maišyklė pervadinta į Nissbau Euromix C120, 3 m³. Koordinatės geokoduotos pagal naują adresą.</t>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z64" s="2" t="inlineStr">
@@ -7860,22 +7876,22 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-runeikiai</t>
+          <t>reljef-rukla</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>301731961</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas</t>
+          <t>UAB Reljef</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas</t>
+          <t>Reljef</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -7885,38 +7901,38 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Runeikiai</t>
+          <t>Rukla</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Kėdainių r. sav.</t>
+          <t>Jonavos r. sav.</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Paguiriai, Šėtos sen., Kėdainių r. sav.</t>
+          <t>Rukla, Jonavos r. sav.</t>
         </is>
       </c>
       <c r="I65" s="3" t="n">
-        <v>55.3327393</v>
+        <v>55.05225</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>24.3501308</v>
+        <v>24.4064167</v>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
+          <t>Tikslus naudotojo pateiktas taškas; adresas artimiausias pagal OpenStreetMap</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas oficialus puslapis</t>
+          <t>Naudotojo pateiktos koordinatės</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
@@ -7931,77 +7947,77 @@
       </c>
       <c r="P65" s="2" t="inlineStr">
         <is>
-          <t>Runeikiai Plant</t>
+          <t>Ammann Elba</t>
         </is>
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>Ammann Elba Euromix C120, 3 m³</t>
+          <t>Nenustatyta</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr">
         <is>
-          <t>60–80 m³/val.</t>
+          <t>Nenustatytas</t>
         </is>
       </c>
       <c r="S65" s="4" t="inlineStr">
         <is>
-          <t>2x85 t</t>
+          <t>2x65 t</t>
         </is>
       </c>
       <c r="T65" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
+          <t>Rukloje veikiantis UAB Reljef betono mazgas: Ammann Elba, 2x65 t silosai. Maišyklė ir našumas nenustatyti.</t>
         </is>
       </c>
       <c r="U65" s="5" t="n">
-        <v>0.9</v>
+        <v>0.82</v>
       </c>
       <c r="V65" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/</t>
+          <t>https://www.reljef.lt/</t>
         </is>
       </c>
       <c r="W65" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.reljef.lt/</t>
         </is>
       </c>
       <c r="X65" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
         </is>
       </c>
       <c r="Y65" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Įmonės rekvizitai paimti iš oficialaus UAB Reljef puslapio. Betono mazgo gamintojas, silosai ir lokacija įrašyti pagal naudotojo pateiktą informaciją. Artimiausias viešai geokoduotas adresas nustatytas pagal OpenStreetMap.</t>
         </is>
       </c>
       <c r="Z65" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>reljef-rukla</t>
+          <t>ponas-betonas-paraudondvariai</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>301731961</t>
+          <t>306676006</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>UAB Reljef</t>
+          <t>UAB Ponas betonas</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Reljef</t>
+          <t>Ponas betonas</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -8011,38 +8027,38 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Rukla</t>
+          <t>Paraudondvariai</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Jonavos r. sav.</t>
+          <t>Vilniaus r. sav.</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Rukla, Jonavos r. sav.</t>
+          <t>Vilniaus g., Paraudondvariai, Riešės sen., Vilniaus r. sav.</t>
         </is>
       </c>
       <c r="I66" s="3" t="n">
-        <v>55.05225</v>
+        <v>54.8321418</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>24.4064167</v>
+        <v>25.2755596</v>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>Tikslus naudotojo pateiktas taškas; adresas artimiausias pagal OpenStreetMap</t>
+          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>Naudotojo pateiktos koordinatės</t>
+          <t>Naudotojo pateikta Google Maps lokacija</t>
         </is>
       </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
+          <t>https://maps.app.goo.gl/NxQohpnzv1q9DA6CA?g_st=ac</t>
         </is>
       </c>
       <c r="N66" s="2" t="inlineStr">
@@ -8057,77 +8073,77 @@
       </c>
       <c r="P66" s="2" t="inlineStr">
         <is>
-          <t>Ammann Elba</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q66" s="2" t="inlineStr">
         <is>
-          <t>Nenustatyta</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="R66" s="2" t="inlineStr">
         <is>
-          <t>Nenustatytas</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="S66" s="4" t="inlineStr">
         <is>
-          <t>2x65 t</t>
+          <t>2 matomi oficialioje nuotraukoje</t>
         </is>
       </c>
       <c r="T66" s="2" t="inlineStr">
         <is>
-          <t>Rukloje veikiantis UAB Reljef betono mazgas: Ammann Elba, 2x65 t silosai. Maišyklė ir našumas nenustatyti.</t>
+          <t>Oficialiame UAB Ponas betonas puslapyje nurodoma, kad įmonė turi nuosavą betono mazgą, gamina prekinį betoną ir jį pristato. Puslapio hero nuotraukoje ant silosų matomas ELKON ženklinimas, todėl mazgo gamintojas identifikuotas kaip Elkon. Konkretus modelis, maišyklė ir našumas viešai nenurodyti; oficialioje nuotraukoje matomi 2 silosai.</t>
         </is>
       </c>
       <c r="U66" s="5" t="n">
-        <v>0.82</v>
+        <v>0.98</v>
       </c>
       <c r="V66" s="2" t="inlineStr">
         <is>
-          <t>https://www.reljef.lt/</t>
+          <t>https://www.ponasbetonas.lt/</t>
         </is>
       </c>
       <c r="W66" s="2" t="inlineStr">
         <is>
-          <t>https://www.reljef.lt/</t>
+          <t>https://www.ponasbetonas.lt/#Apiemus</t>
         </is>
       </c>
       <c r="X66" s="2" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
+          <t>https://www.ponasbetonas.lt/</t>
         </is>
       </c>
       <c r="Y66" s="2" t="inlineStr">
         <is>
-          <t>Įmonės rekvizitai paimti iš oficialaus UAB Reljef puslapio. Betono mazgo gamintojas, silosai ir lokacija įrašyti pagal naudotojo pateiktą informaciją. Artimiausias viešai geokoduotas adresas nustatytas pagal OpenStreetMap.</t>
+          <t>Nuosavas betono mazgas ir prekinio betono gamyba patvirtinti oficialiame įmonės puslapyje. Mazgo gamintojas nustatytas pagal oficialaus puslapio hero nuotraukoje ant silosų matomą ELKON ženklinimą; modelis, maišyklė ir našumas viešai nenurodyti. Tiksli mazgo lokacija paimta iš naudotojo pateiktos Google Maps nuorodos; vietovė patikslinta pagal OpenStreetMap. Įmonės kodas patvirtintas Registrų centro viešame juridinio asmens pranešime.</t>
         </is>
       </c>
       <c r="Z66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>ponas-betonas-paraudondvariai</t>
+          <t>pabrades-betonas-pabrade</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>306676006</t>
+          <t>306177188</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>UAB Ponas betonas</t>
+          <t>UAB Pabradės betonas</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Ponas betonas</t>
+          <t>Pabradės betonas</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -8137,38 +8153,38 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Paraudondvariai</t>
+          <t>Pabradė</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus r. sav.</t>
+          <t>Švenčionių r. sav.</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus g., Paraudondvariai, Riešės sen., Vilniaus r. sav.</t>
+          <t>Vilniaus g. 161, Pabradė, LT-18177 Švenčionių r.</t>
         </is>
       </c>
       <c r="I67" s="3" t="n">
-        <v>54.8321418</v>
+        <v>54.9758768</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>25.2755596</v>
+        <v>25.7373849</v>
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
+          <t>Tikslus oficialioje svetainėje pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>Naudotojo pateikta Google Maps lokacija</t>
+          <t>Oficiali Pabradės betono Google Maps nuoroda</t>
         </is>
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/NxQohpnzv1q9DA6CA?g_st=ac</t>
+          <t>https://maps.app.goo.gl/TQBCVR8DczDRvQaeA</t>
         </is>
       </c>
       <c r="N67" s="2" t="inlineStr">
@@ -8183,186 +8199,60 @@
       </c>
       <c r="P67" s="2" t="inlineStr">
         <is>
-          <t>Elkon</t>
+          <t>Liebherr (tikėtina)</t>
         </is>
       </c>
       <c r="Q67" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>3 m³</t>
         </is>
       </c>
       <c r="R67" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>60 m³/val.</t>
         </is>
       </c>
       <c r="S67" s="4" t="inlineStr">
         <is>
-          <t>2 matomi oficialioje nuotraukoje</t>
+          <t>3x65 t</t>
         </is>
       </c>
       <c r="T67" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame UAB Ponas betonas puslapyje nurodoma, kad įmonė turi nuosavą betono mazgą, gamina prekinį betoną ir jį pristato. Puslapio hero nuotraukoje ant silosų matomas ELKON ženklinimas, todėl mazgo gamintojas identifikuotas kaip Elkon. Konkretus modelis, maišyklė ir našumas viešai nenurodyti; oficialioje nuotraukoje matomi 2 silosai.</t>
+          <t>UAB Pabradės betonas Vilniaus g. 161, Pabradėje, gamina sertifikuotą normalųjį betoną ir oficialiai nurodo dirbanti 50 km spinduliu aplink Pabradę. Oficialios galerijos nuotraukose matoma stacionari gamybos bazė su trimis cemento silosais. Mazgo gamintojas tikėtinai Liebherr pagal oficialiose nuotraukose matomą Liebherr įrangą ir gamyklos konstrukcijos vizualinius požymius; gamintojo lentelė viešai neparodyta.</t>
         </is>
       </c>
       <c r="U67" s="5" t="n">
-        <v>0.98</v>
+        <v>0.72</v>
       </c>
       <c r="V67" s="2" t="inlineStr">
         <is>
-          <t>https://www.ponasbetonas.lt/</t>
+          <t>https://www.pabradesbetonas.lt/</t>
         </is>
       </c>
       <c r="W67" s="2" t="inlineStr">
         <is>
-          <t>https://www.ponasbetonas.lt/#Apiemus</t>
+          <t>https://www.pabradesbetonas.lt/</t>
         </is>
       </c>
       <c r="X67" s="2" t="inlineStr">
         <is>
-          <t>https://www.ponasbetonas.lt/</t>
+          <t>https://www.pabradesbetonas.lt/galerija/</t>
         </is>
       </c>
       <c r="Y67" s="2" t="inlineStr">
         <is>
-          <t>Nuosavas betono mazgas ir prekinio betono gamyba patvirtinti oficialiame įmonės puslapyje. Mazgo gamintojas nustatytas pagal oficialaus puslapio hero nuotraukoje ant silosų matomą ELKON ženklinimą; modelis, maišyklė ir našumas viešai nenurodyti. Tiksli mazgo lokacija paimta iš naudotojo pateiktos Google Maps nuorodos; vietovė patikslinta pagal OpenStreetMap. Įmonės kodas patvirtintas Registrų centro viešame juridinio asmens pranešime.</t>
+          <t>Adresas, įmonės kodas ir betono gamyba patvirtinti oficialioje svetainėje bei viešame gamybos kontrolės sertifikate. Koordinatės paimtos iš oficialioje svetainėje pateiktos Google Maps nuorodos. Maišyklės tūris 3 m³, realus našumas 60 m³/val. ir silosai 3x65 t įrašyti pagal naudotojo pateiktą informaciją. Gamintojas Liebherr nurodytas kaip tikėtinas pagal oficialios galerijos nuotraukas; viešo gamintojo ženklinimo ant paties mazgo nerasta.</t>
         </is>
       </c>
       <c r="Z67" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>pabrades-betonas-pabrade</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>306177188</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>UAB Pabradės betonas</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>Pabradės betonas</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>Konkurentas</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>Pabradė</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>Švenčionių r. sav.</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>Vilniaus g. 161, Pabradė, LT-18177 Švenčionių r.</t>
-        </is>
-      </c>
-      <c r="I68" s="3" t="n">
-        <v>54.9758768</v>
-      </c>
-      <c r="J68" s="3" t="n">
-        <v>25.7373849</v>
-      </c>
-      <c r="K68" s="2" t="inlineStr">
-        <is>
-          <t>Tikslus oficialioje svetainėje pateiktos Google Maps nuorodos taškas</t>
-        </is>
-      </c>
-      <c r="L68" s="2" t="inlineStr">
-        <is>
-          <t>Oficiali Pabradės betono Google Maps nuoroda</t>
-        </is>
-      </c>
-      <c r="M68" s="2" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/TQBCVR8DczDRvQaeA</t>
-        </is>
-      </c>
-      <c r="N68" s="2" t="inlineStr">
-        <is>
-          <t>ready_mix_concrete</t>
-        </is>
-      </c>
-      <c r="O68" s="2" t="inlineStr">
-        <is>
-          <t>Betono mišiniai</t>
-        </is>
-      </c>
-      <c r="P68" s="2" t="inlineStr">
-        <is>
-          <t>Liebherr (tikėtina)</t>
-        </is>
-      </c>
-      <c r="Q68" s="2" t="inlineStr">
-        <is>
-          <t>3 m³</t>
-        </is>
-      </c>
-      <c r="R68" s="2" t="inlineStr">
-        <is>
-          <t>60 m³/val.</t>
-        </is>
-      </c>
-      <c r="S68" s="4" t="inlineStr">
-        <is>
-          <t>3x65 t</t>
-        </is>
-      </c>
-      <c r="T68" s="2" t="inlineStr">
-        <is>
-          <t>UAB Pabradės betonas Vilniaus g. 161, Pabradėje, gamina sertifikuotą normalųjį betoną ir oficialiai nurodo dirbanti 50 km spinduliu aplink Pabradę. Oficialios galerijos nuotraukose matoma stacionari gamybos bazė su trimis cemento silosais. Mazgo gamintojas tikėtinai Liebherr pagal oficialiose nuotraukose matomą Liebherr įrangą ir gamyklos konstrukcijos vizualinius požymius; gamintojo lentelė viešai neparodyta.</t>
-        </is>
-      </c>
-      <c r="U68" s="5" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="V68" s="2" t="inlineStr">
-        <is>
-          <t>https://www.pabradesbetonas.lt/</t>
-        </is>
-      </c>
-      <c r="W68" s="2" t="inlineStr">
-        <is>
-          <t>https://www.pabradesbetonas.lt/</t>
-        </is>
-      </c>
-      <c r="X68" s="2" t="inlineStr">
-        <is>
-          <t>https://www.pabradesbetonas.lt/galerija/</t>
-        </is>
-      </c>
-      <c r="Y68" s="2" t="inlineStr">
-        <is>
-          <t>Adresas, įmonės kodas ir betono gamyba patvirtinti oficialioje svetainėje bei viešame gamybos kontrolės sertifikate. Koordinatės paimtos iš oficialioje svetainėje pateiktos Google Maps nuorodos. Maišyklės tūris 3 m³, realus našumas 60 m³/val. ir silosai 3x65 t įrašyti pagal naudotojo pateiktą informaciją. Gamintojas Liebherr nurodytas kaip tikėtinas pagal oficialios galerijos nuotraukas; viešo gamintojo ženklinimo ant paties mazgo nerasta.</t>
-        </is>
-      </c>
-      <c r="Z68" s="2" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z68"/>
+  <autoFilter ref="A1:Z67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8451,7 +8341,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-23T15:17:04.691715+00:00</t>
+          <t>2026-09-23T15:24:19.634207+00:00</t>
         </is>
       </c>
     </row>
@@ -8506,7 +8396,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-23T15:17:04.691715+00:00</t>
+          <t>2026-09-23T15:24:19.635205+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8520,7 +8410,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Prideti Alkesta ir Gevalda betono mazgus
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z67" headerRowCount="1">
-  <autoFilter ref="A1:Z67"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z70" headerRowCount="1">
+  <autoFilter ref="A1:Z70"/>
   <tableColumns count="26">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z67"/>
+  <dimension ref="A1:Z70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -8251,8 +8251,382 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>alkesta-marijampole-vasaros</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>249672710</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>UAB Alkesta</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Alkesta</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Konkurentas</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Marijampolė</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Marijampolės sav.</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Vasaros g. 14, Marijampolė, LT-68111</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="n">
+        <v>54.5686121</v>
+      </c>
+      <c r="J68" s="3" t="n">
+        <v>23.3895157</v>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>Naudotojo pateikta Google Maps lokacija</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>Elba</t>
+        </is>
+      </c>
+      <c r="Q68" s="2" t="inlineStr">
+        <is>
+          <t>0,5 m³</t>
+        </is>
+      </c>
+      <c r="R68" s="2" t="inlineStr">
+        <is>
+          <t>10 m³/val.</t>
+        </is>
+      </c>
+      <c r="S68" s="4" t="inlineStr"/>
+      <c r="T68" s="2" t="inlineStr">
+        <is>
+          <t>UAB Alkesta Marijampolės betono mazgas Vasaros g. 14. Mazgo gamintojas Elba, maišyklė 0,5 m³, našumas 10 m³/val.</t>
+        </is>
+      </c>
+      <c r="U68" s="5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="V68" s="2" t="inlineStr">
+        <is>
+          <t>https://alkesta.lt/</t>
+        </is>
+      </c>
+      <c r="W68" s="2" t="inlineStr">
+        <is>
+          <t>https://spsc.lt/registrai/regsapp/ser_produktai_view.php?editid1=13061</t>
+        </is>
+      </c>
+      <c r="X68" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
+        </is>
+      </c>
+      <c r="Y68" s="2" t="inlineStr">
+        <is>
+          <t>Oficialus SPSC sertifikatų registras patvirtina UAB Alkesta betono gamybą ir gamybos vietą Vasaros g. 14, Marijampolėje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris ir našumas įrašyti pagal naudotojo pateiktą informaciją.</t>
+        </is>
+      </c>
+      <c r="Z68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>gevalda-visincia</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>302592895</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>UAB Gevalda</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Gevalda</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Konkurentas</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Visinčia</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Šalčininkų r. sav.</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>Visinčia, Pabarės sen., Šalčininkų r. sav.</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="n">
+        <v>54.4122467</v>
+      </c>
+      <c r="J69" s="3" t="n">
+        <v>25.1449142</v>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>Naudotojo pateikta Google Maps lokacija</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="P69" s="2" t="inlineStr">
+        <is>
+          <t>Elkon</t>
+        </is>
+      </c>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>3 m³</t>
+        </is>
+      </c>
+      <c r="R69" s="2" t="inlineStr">
+        <is>
+          <t>60 m³/val.</t>
+        </is>
+      </c>
+      <c r="S69" s="4" t="inlineStr">
+        <is>
+          <t>2x85 t</t>
+        </is>
+      </c>
+      <c r="T69" s="2" t="inlineStr">
+        <is>
+          <t>UAB Gevalda mobilus betono mazgas Visinčioje. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
+        </is>
+      </c>
+      <c r="U69" s="5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="V69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gevalda.lt/</t>
+        </is>
+      </c>
+      <c r="W69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gevalda.lt/paslaugos/gamyba</t>
+        </is>
+      </c>
+      <c r="X69" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
+        </is>
+      </c>
+      <c r="Y69" s="2" t="inlineStr">
+        <is>
+          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris, našumas ir silosai įrašyti pagal naudotojo pateiktą informaciją.</t>
+        </is>
+      </c>
+      <c r="Z69" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>gevalda-kaunas-palemonas</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>302592895</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>UAB Gevalda</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Gevalda</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Konkurentas</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Kaunas</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Kauno m. sav.</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Kražantės g., Palemonas, Kaunas</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="n">
+        <v>54.918</v>
+      </c>
+      <c r="J70" s="3" t="n">
+        <v>24.063</v>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>Naudotojo pateikta Google Maps lokacija</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="P70" s="2" t="inlineStr">
+        <is>
+          <t>Elkon</t>
+        </is>
+      </c>
+      <c r="Q70" s="2" t="inlineStr">
+        <is>
+          <t>3 m³</t>
+        </is>
+      </c>
+      <c r="R70" s="2" t="inlineStr">
+        <is>
+          <t>60 m³/val.</t>
+        </is>
+      </c>
+      <c r="S70" s="4" t="inlineStr">
+        <is>
+          <t>2x85 t</t>
+        </is>
+      </c>
+      <c r="T70" s="2" t="inlineStr">
+        <is>
+          <t>UAB Gevalda mobilus betono mazgas Palemone, Kaune. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
+        </is>
+      </c>
+      <c r="U70" s="5" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="V70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gevalda.lt/</t>
+        </is>
+      </c>
+      <c r="W70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gevalda.lt/paslaugos/gamyba</t>
+        </is>
+      </c>
+      <c r="X70" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
+        </is>
+      </c>
+      <c r="Y70" s="2" t="inlineStr">
+        <is>
+          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija ir analogiški techniniai duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
+        </is>
+      </c>
+      <c r="Z70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z67"/>
+  <autoFilter ref="A1:Z70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8341,7 +8715,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-23T15:24:19.634207+00:00</t>
+          <t>2026-09-23T15:50:11.921774+00:00</t>
         </is>
       </c>
     </row>
@@ -8396,7 +8770,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-23T15:24:19.635205+00:00</t>
+          <t>2026-09-23T15:50:11.921774+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8410,7 +8784,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Pasalinti Beton Eura taska
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z70" headerRowCount="1">
-  <autoFilter ref="A1:Z70"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z69" headerRowCount="1">
+  <autoFilter ref="A1:Z69"/>
   <tableColumns count="26">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z70"/>
+  <dimension ref="A1:Z69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -6802,22 +6802,22 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>beton-eura-dovainonys</t>
+          <t>silutes-betonas-silute</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>302745280</t>
+          <t>177392928</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>UAB Beton Eura</t>
+          <t>UAB Šilutės betonas</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Beton Eura</t>
+          <t>Šilutės betonas</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -6827,24 +6827,24 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Dovainonys</t>
+          <t>Šilutė</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Kaišiadorių r. sav.</t>
+          <t>Šilutės r. sav.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Žilvičių g. 2, Dovainonys, Kaišiadorių r.</t>
+          <t>Ramučių g. 1, Šilutė</t>
         </is>
       </c>
       <c r="I56" s="3" t="n">
-        <v>54.8395918</v>
+        <v>55.3538641</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>24.2360193</v>
+        <v>21.4796635</v>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>Beton Eura betono gamyba</t>
+          <t>Šilutės betono gamyba</t>
         </is>
       </c>
       <c r="Q56" s="2" t="inlineStr"/>
@@ -6887,24 +6887,20 @@
       <c r="U56" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V56" s="2" t="inlineStr">
-        <is>
-          <t>https://www.betoneura.lt/</t>
-        </is>
-      </c>
+      <c r="V56" s="2" t="inlineStr"/>
       <c r="W56" s="2" t="inlineStr">
         <is>
-          <t>https://www.betoneura.lt/kontaktai/</t>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
       <c r="X56" s="2" t="inlineStr">
         <is>
-          <t>https://www.betoneura.lt/kontaktai/</t>
+          <t>https://fsaskaita.lt/imone/uzdaroji-akcine-bendrove-silutes-betonas-177392928</t>
         </is>
       </c>
       <c r="Y56" s="2" t="inlineStr">
         <is>
-          <t>Oficialus Beton Eura kontaktų puslapis patvirtina Žilvičių g. 2 adresą ir rekvizitus.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z56" s="2" t="inlineStr">
@@ -6916,22 +6912,22 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>silutes-betonas-silute</t>
+          <t>kruszbet-lithuania-jure</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>177392928</t>
+          <t>305173596</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>UAB Šilutės betonas</t>
+          <t>UAB KRUSZBET Lithuania</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Šilutės betonas</t>
+          <t>KRUSZBET Lithuania</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -6941,24 +6937,24 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Šilutė</t>
+          <t>Jūrė</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Šilutės r. sav.</t>
+          <t>Kazlų Rūdos sav.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Ramučių g. 1, Šilutė</t>
+          <t>Medelyno g. 30A, Jūrė, Kazlų Rūdos sav.</t>
         </is>
       </c>
       <c r="I57" s="3" t="n">
-        <v>55.3538641</v>
+        <v>54.7706307</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>21.4796635</v>
+        <v>23.4998409</v>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
@@ -6987,7 +6983,7 @@
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
-          <t>Šilutės betono gamyba</t>
+          <t>KRUSZBET Lithuania betono gamyba</t>
         </is>
       </c>
       <c r="Q57" s="2" t="inlineStr"/>
@@ -7007,11 +7003,7 @@
           <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
-      <c r="X57" s="2" t="inlineStr">
-        <is>
-          <t>https://fsaskaita.lt/imone/uzdaroji-akcine-bendrove-silutes-betonas-177392928</t>
-        </is>
-      </c>
+      <c r="X57" s="2" t="inlineStr"/>
       <c r="Y57" s="2" t="inlineStr">
         <is>
           <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
@@ -7026,49 +7018,49 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>kruszbet-lithuania-jure</t>
+          <t>telsiu-keliai-telsiai</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>305173596</t>
+          <t>180200843</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>UAB KRUSZBET Lithuania</t>
+          <t>UAB Telšių keliai</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>KRUSZBET Lithuania</t>
+          <t>Telšių keliai</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta EVRK 23.63</t>
+          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Jūrė</t>
+          <t>Telšiai</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Kazlų Rūdos sav.</t>
+          <t>Telšių r. sav.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Medelyno g. 30A, Jūrė, Kazlų Rūdos sav.</t>
+          <t>Mažeikių g. 18, Telšiai</t>
         </is>
       </c>
       <c r="I58" s="3" t="n">
-        <v>54.7706307</v>
+        <v>56.0004158</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>23.4998409</v>
+        <v>22.2581129</v>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
@@ -7097,57 +7089,67 @@
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>KRUSZBET Lithuania betono gamyba</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q58" s="2" t="inlineStr"/>
       <c r="R58" s="2" t="inlineStr"/>
-      <c r="S58" s="4" t="inlineStr"/>
+      <c r="S58" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T58" s="2" t="inlineStr">
         <is>
-          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai.</t>
         </is>
       </c>
       <c r="U58" s="5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="V58" s="2" t="inlineStr"/>
+        <v>0.86</v>
+      </c>
+      <c r="V58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/</t>
+        </is>
+      </c>
       <c r="W58" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X58" s="2" t="inlineStr"/>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+        </is>
+      </c>
+      <c r="X58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+        </is>
+      </c>
       <c r="Y58" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
         </is>
       </c>
       <c r="Z58" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>telsiu-keliai-telsiai</t>
+          <t>vpa-laistai</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>180200843</t>
+          <t>110185819</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>UAB Telšių keliai</t>
+          <t>UAB V. Paulius &amp; Associates</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Telšių keliai</t>
+          <t>VPA</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -7157,38 +7159,38 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Telšiai</t>
+          <t>Laistai</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Telšių r. sav.</t>
+          <t>Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Mažeikių g. 18, Telšiai</t>
+          <t>Stariškės g. 9, Laistų k., Dovilų sen., Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="I59" s="3" t="n">
-        <v>56.0004158</v>
+        <v>55.636908</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>22.2581129</v>
+        <v>21.209254</v>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Naudotojo pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>Google Maps nuoroda</t>
         </is>
       </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
         </is>
       </c>
       <c r="N59" s="2" t="inlineStr">
@@ -7203,108 +7205,116 @@
       </c>
       <c r="P59" s="2" t="inlineStr">
         <is>
-          <t>Elkon</t>
-        </is>
-      </c>
-      <c r="Q59" s="2" t="inlineStr"/>
-      <c r="R59" s="2" t="inlineStr"/>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="Q59" s="2" t="inlineStr">
+        <is>
+          <t>3 m³</t>
+        </is>
+      </c>
+      <c r="R59" s="2" t="inlineStr">
+        <is>
+          <t>60-80 m³/h</t>
+        </is>
+      </c>
       <c r="S59" s="4" t="n">
         <v>2</v>
       </c>
       <c r="T59" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai.</t>
+          <t>VPA betono mazgas Klaipėdos rajone.</t>
         </is>
       </c>
       <c r="U59" s="5" t="n">
-        <v>0.86</v>
+        <v>0.7</v>
       </c>
       <c r="V59" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/</t>
+          <t>https://www.vpa.lt/</t>
         </is>
       </c>
       <c r="W59" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+          <t>https://www.vpa.lt/?Kontaktai=</t>
         </is>
       </c>
       <c r="X59" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
         </is>
       </c>
       <c r="Y59" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
+          <t>Vieta nustatyta pagal naudotojo pateiktą Google Maps nuorodą. VPA kontaktų puslapis nurodo Stariškės g. 9, Laistų k. adresą. Techniniai mazgo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z59" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>vpa-laistai</t>
+          <t>c3-beton-baisogala</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>110185819</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>UAB V. Paulius &amp; Associates</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>VPA</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
+          <t>Konkurentas</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Laistai</t>
+          <t>Baisogala</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Klaipėdos r. sav.</t>
+          <t>Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Stariškės g. 9, Laistų k., Dovilų sen., Klaipėdos r. sav.</t>
+          <t>Dvaro g., Baisogala, Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="I60" s="3" t="n">
-        <v>55.636908</v>
+        <v>55.6372</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>21.209254</v>
+        <v>23.7183</v>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>Naudotojo pateiktos Google Maps nuorodos taškas</t>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>Google Maps nuoroda</t>
+          <t>C3 Betonas oficialus puslapis</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
@@ -7319,60 +7329,62 @@
       </c>
       <c r="P60" s="2" t="inlineStr">
         <is>
-          <t>Liebherr</t>
+          <t>Baisiogala Plant</t>
         </is>
       </c>
       <c r="Q60" s="2" t="inlineStr">
         <is>
-          <t>3 m³</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="R60" s="2" t="inlineStr">
         <is>
-          <t>60-80 m³/h</t>
-        </is>
-      </c>
-      <c r="S60" s="4" t="n">
-        <v>2</v>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="S60" s="4" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
       </c>
       <c r="T60" s="2" t="inlineStr">
         <is>
-          <t>VPA betono mazgas Klaipėdos rajone.</t>
+          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
         </is>
       </c>
       <c r="U60" s="5" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="V60" s="2" t="inlineStr">
         <is>
-          <t>https://www.vpa.lt/</t>
+          <t>https://c3beton.com/</t>
         </is>
       </c>
       <c r="W60" s="2" t="inlineStr">
         <is>
-          <t>https://www.vpa.lt/?Kontaktai=</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="X60" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="Y60" s="2" t="inlineStr">
         <is>
-          <t>Vieta nustatyta pagal naudotojo pateiktą Google Maps nuorodą. VPA kontaktų puslapis nurodo Stariškės g. 9, Laistų k. adresą. Techniniai mazgo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
         </is>
       </c>
       <c r="Z60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-baisogala</t>
+          <t>c3-beton-martiniskis</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -7397,24 +7409,24 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Baisogala</t>
+          <t>Martiniškis</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Radviliškio r. sav.</t>
+          <t>Jonavos r. sav.</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Dvaro g., Baisogala, Radviliškio r. sav.</t>
+          <t>Vanagiškiai, Kulvos sen., Jonavos r. sav.</t>
         </is>
       </c>
       <c r="I61" s="3" t="n">
-        <v>55.6372</v>
+        <v>55.1441659</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>23.7183</v>
+        <v>24.1869636</v>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
@@ -7443,27 +7455,27 @@
       </c>
       <c r="P61" s="2" t="inlineStr">
         <is>
-          <t>Baisiogala Plant</t>
+          <t>Martiniškis Plant</t>
         </is>
       </c>
       <c r="Q61" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>Ammann Elba Euromix C120, 3 m³</t>
         </is>
       </c>
       <c r="R61" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>60–80 m³/val.</t>
         </is>
       </c>
       <c r="S61" s="4" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>2x85 t</t>
         </is>
       </c>
       <c r="T61" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
+          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U61" s="5" t="n">
@@ -7486,7 +7498,7 @@
       </c>
       <c r="Y61" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z61" s="2" t="inlineStr">
@@ -7498,7 +7510,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-martiniskis</t>
+          <t>c3-beton-stasenai</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -7523,38 +7535,38 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Martiniškis</t>
+          <t>Vilnius</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Jonavos r. sav.</t>
+          <t>Vilniaus m. sav.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Vanagiškiai, Kulvos sen., Jonavos r. sav.</t>
+          <t>Ušos g. 21, Vilnius, 02121 Vilniaus m. sav.</t>
         </is>
       </c>
       <c r="I62" s="3" t="n">
-        <v>55.1441659</v>
+        <v>54.6493094</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>24.1869636</v>
+        <v>25.3107972</v>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
+          <t>Tikslus adreso taškas pagal geokodavimą</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas oficialus puslapis</t>
+          <t>ArcGIS geokodavimas pagal naudotojo pateiktą adresą</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://geocode.arcgis.com/arcgis/rest/services/World/GeocodeServer/findAddressCandidates</t>
         </is>
       </c>
       <c r="N62" s="2" t="inlineStr">
@@ -7569,12 +7581,12 @@
       </c>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t>Martiniškis Plant</t>
+          <t>Vilnius Ušos g. Plant</t>
         </is>
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>Ammann Elba Euromix C120, 3 m³</t>
+          <t>Nissbau Euromix C120, 3 m³</t>
         </is>
       </c>
       <c r="R62" s="2" t="inlineStr">
@@ -7589,7 +7601,7 @@
       </c>
       <c r="T62" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
+          <t>Betono mazgas Nissbau Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U62" s="5" t="n">
@@ -7612,7 +7624,7 @@
       </c>
       <c r="Y62" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Perkelta iš Stašėnų lokacijos į Ušos g. 21, Vilnius pagal naudotojo pateiktą informaciją. Maišyklė pervadinta į Nissbau Euromix C120, 3 m³. Koordinatės geokoduotos pagal naują adresą.</t>
         </is>
       </c>
       <c r="Z62" s="2" t="inlineStr">
@@ -7624,7 +7636,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-stasenai</t>
+          <t>c3-beton-runeikiai</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -7649,38 +7661,38 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Vilnius</t>
+          <t>Runeikiai</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus m. sav.</t>
+          <t>Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Ušos g. 21, Vilnius, 02121 Vilniaus m. sav.</t>
+          <t>Paguiriai, Šėtos sen., Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="I63" s="3" t="n">
-        <v>54.6493094</v>
+        <v>55.3327393</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>25.3107972</v>
+        <v>24.3501308</v>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas pagal geokodavimą</t>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>ArcGIS geokodavimas pagal naudotojo pateiktą adresą</t>
+          <t>C3 Betonas oficialus puslapis</t>
         </is>
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>https://geocode.arcgis.com/arcgis/rest/services/World/GeocodeServer/findAddressCandidates</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="N63" s="2" t="inlineStr">
@@ -7695,12 +7707,12 @@
       </c>
       <c r="P63" s="2" t="inlineStr">
         <is>
-          <t>Vilnius Ušos g. Plant</t>
+          <t>Runeikiai Plant</t>
         </is>
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>Nissbau Euromix C120, 3 m³</t>
+          <t>Ammann Elba Euromix C120, 3 m³</t>
         </is>
       </c>
       <c r="R63" s="2" t="inlineStr">
@@ -7715,7 +7727,7 @@
       </c>
       <c r="T63" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgas Nissbau Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
+          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U63" s="5" t="n">
@@ -7738,7 +7750,7 @@
       </c>
       <c r="Y63" s="2" t="inlineStr">
         <is>
-          <t>Perkelta iš Stašėnų lokacijos į Ušos g. 21, Vilnius pagal naudotojo pateiktą informaciją. Maišyklė pervadinta į Nissbau Euromix C120, 3 m³. Koordinatės geokoduotos pagal naują adresą.</t>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z63" s="2" t="inlineStr">
@@ -7750,22 +7762,22 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-runeikiai</t>
+          <t>reljef-rukla</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>301731961</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas</t>
+          <t>UAB Reljef</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas</t>
+          <t>Reljef</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -7775,38 +7787,38 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Runeikiai</t>
+          <t>Rukla</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Kėdainių r. sav.</t>
+          <t>Jonavos r. sav.</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Paguiriai, Šėtos sen., Kėdainių r. sav.</t>
+          <t>Rukla, Jonavos r. sav.</t>
         </is>
       </c>
       <c r="I64" s="3" t="n">
-        <v>55.3327393</v>
+        <v>55.05225</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>24.3501308</v>
+        <v>24.4064167</v>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
+          <t>Tikslus naudotojo pateiktas taškas; adresas artimiausias pagal OpenStreetMap</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas oficialus puslapis</t>
+          <t>Naudotojo pateiktos koordinatės</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
@@ -7821,77 +7833,77 @@
       </c>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>Runeikiai Plant</t>
+          <t>Ammann Elba</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>Ammann Elba Euromix C120, 3 m³</t>
+          <t>Nenustatyta</t>
         </is>
       </c>
       <c r="R64" s="2" t="inlineStr">
         <is>
-          <t>60–80 m³/val.</t>
+          <t>Nenustatytas</t>
         </is>
       </c>
       <c r="S64" s="4" t="inlineStr">
         <is>
-          <t>2x85 t</t>
+          <t>2x65 t</t>
         </is>
       </c>
       <c r="T64" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
+          <t>Rukloje veikiantis UAB Reljef betono mazgas: Ammann Elba, 2x65 t silosai. Maišyklė ir našumas nenustatyti.</t>
         </is>
       </c>
       <c r="U64" s="5" t="n">
-        <v>0.9</v>
+        <v>0.82</v>
       </c>
       <c r="V64" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/</t>
+          <t>https://www.reljef.lt/</t>
         </is>
       </c>
       <c r="W64" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.reljef.lt/</t>
         </is>
       </c>
       <c r="X64" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
         </is>
       </c>
       <c r="Y64" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Įmonės rekvizitai paimti iš oficialaus UAB Reljef puslapio. Betono mazgo gamintojas, silosai ir lokacija įrašyti pagal naudotojo pateiktą informaciją. Artimiausias viešai geokoduotas adresas nustatytas pagal OpenStreetMap.</t>
         </is>
       </c>
       <c r="Z64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>reljef-rukla</t>
+          <t>ponas-betonas-paraudondvariai</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>301731961</t>
+          <t>306676006</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>UAB Reljef</t>
+          <t>UAB Ponas betonas</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Reljef</t>
+          <t>Ponas betonas</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -7901,38 +7913,38 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Rukla</t>
+          <t>Paraudondvariai</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Jonavos r. sav.</t>
+          <t>Vilniaus r. sav.</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Rukla, Jonavos r. sav.</t>
+          <t>Vilniaus g., Paraudondvariai, Riešės sen., Vilniaus r. sav.</t>
         </is>
       </c>
       <c r="I65" s="3" t="n">
-        <v>55.05225</v>
+        <v>54.8321418</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>24.4064167</v>
+        <v>25.2755596</v>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>Tikslus naudotojo pateiktas taškas; adresas artimiausias pagal OpenStreetMap</t>
+          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>Naudotojo pateiktos koordinatės</t>
+          <t>Naudotojo pateikta Google Maps lokacija</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
+          <t>https://maps.app.goo.gl/NxQohpnzv1q9DA6CA?g_st=ac</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
@@ -7947,77 +7959,77 @@
       </c>
       <c r="P65" s="2" t="inlineStr">
         <is>
-          <t>Ammann Elba</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>Nenustatyta</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr">
         <is>
-          <t>Nenustatytas</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="S65" s="4" t="inlineStr">
         <is>
-          <t>2x65 t</t>
+          <t>2 matomi oficialioje nuotraukoje</t>
         </is>
       </c>
       <c r="T65" s="2" t="inlineStr">
         <is>
-          <t>Rukloje veikiantis UAB Reljef betono mazgas: Ammann Elba, 2x65 t silosai. Maišyklė ir našumas nenustatyti.</t>
+          <t>Oficialiame UAB Ponas betonas puslapyje nurodoma, kad įmonė turi nuosavą betono mazgą, gamina prekinį betoną ir jį pristato. Puslapio hero nuotraukoje ant silosų matomas ELKON ženklinimas, todėl mazgo gamintojas identifikuotas kaip Elkon. Konkretus modelis, maišyklė ir našumas viešai nenurodyti; oficialioje nuotraukoje matomi 2 silosai.</t>
         </is>
       </c>
       <c r="U65" s="5" t="n">
-        <v>0.82</v>
+        <v>0.98</v>
       </c>
       <c r="V65" s="2" t="inlineStr">
         <is>
-          <t>https://www.reljef.lt/</t>
+          <t>https://www.ponasbetonas.lt/</t>
         </is>
       </c>
       <c r="W65" s="2" t="inlineStr">
         <is>
-          <t>https://www.reljef.lt/</t>
+          <t>https://www.ponasbetonas.lt/#Apiemus</t>
         </is>
       </c>
       <c r="X65" s="2" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
+          <t>https://www.ponasbetonas.lt/</t>
         </is>
       </c>
       <c r="Y65" s="2" t="inlineStr">
         <is>
-          <t>Įmonės rekvizitai paimti iš oficialaus UAB Reljef puslapio. Betono mazgo gamintojas, silosai ir lokacija įrašyti pagal naudotojo pateiktą informaciją. Artimiausias viešai geokoduotas adresas nustatytas pagal OpenStreetMap.</t>
+          <t>Nuosavas betono mazgas ir prekinio betono gamyba patvirtinti oficialiame įmonės puslapyje. Mazgo gamintojas nustatytas pagal oficialaus puslapio hero nuotraukoje ant silosų matomą ELKON ženklinimą; modelis, maišyklė ir našumas viešai nenurodyti. Tiksli mazgo lokacija paimta iš naudotojo pateiktos Google Maps nuorodos; vietovė patikslinta pagal OpenStreetMap. Įmonės kodas patvirtintas Registrų centro viešame juridinio asmens pranešime.</t>
         </is>
       </c>
       <c r="Z65" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>ponas-betonas-paraudondvariai</t>
+          <t>pabrades-betonas-pabrade</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>306676006</t>
+          <t>306177188</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>UAB Ponas betonas</t>
+          <t>UAB Pabradės betonas</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Ponas betonas</t>
+          <t>Pabradės betonas</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -8027,38 +8039,38 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Paraudondvariai</t>
+          <t>Pabradė</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus r. sav.</t>
+          <t>Švenčionių r. sav.</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus g., Paraudondvariai, Riešės sen., Vilniaus r. sav.</t>
+          <t>Vilniaus g. 161, Pabradė, LT-18177 Švenčionių r.</t>
         </is>
       </c>
       <c r="I66" s="3" t="n">
-        <v>54.8321418</v>
+        <v>54.9758768</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>25.2755596</v>
+        <v>25.7373849</v>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
+          <t>Tikslus oficialioje svetainėje pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>Naudotojo pateikta Google Maps lokacija</t>
+          <t>Oficiali Pabradės betono Google Maps nuoroda</t>
         </is>
       </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/NxQohpnzv1q9DA6CA?g_st=ac</t>
+          <t>https://maps.app.goo.gl/TQBCVR8DczDRvQaeA</t>
         </is>
       </c>
       <c r="N66" s="2" t="inlineStr">
@@ -8073,77 +8085,77 @@
       </c>
       <c r="P66" s="2" t="inlineStr">
         <is>
-          <t>Elkon</t>
+          <t>Liebherr (tikėtina)</t>
         </is>
       </c>
       <c r="Q66" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>3 m³</t>
         </is>
       </c>
       <c r="R66" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>60 m³/val.</t>
         </is>
       </c>
       <c r="S66" s="4" t="inlineStr">
         <is>
-          <t>2 matomi oficialioje nuotraukoje</t>
+          <t>3x65 t</t>
         </is>
       </c>
       <c r="T66" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame UAB Ponas betonas puslapyje nurodoma, kad įmonė turi nuosavą betono mazgą, gamina prekinį betoną ir jį pristato. Puslapio hero nuotraukoje ant silosų matomas ELKON ženklinimas, todėl mazgo gamintojas identifikuotas kaip Elkon. Konkretus modelis, maišyklė ir našumas viešai nenurodyti; oficialioje nuotraukoje matomi 2 silosai.</t>
+          <t>UAB Pabradės betonas Vilniaus g. 161, Pabradėje, gamina sertifikuotą normalųjį betoną ir oficialiai nurodo dirbanti 50 km spinduliu aplink Pabradę. Oficialios galerijos nuotraukose matoma stacionari gamybos bazė su trimis cemento silosais. Mazgo gamintojas tikėtinai Liebherr pagal oficialiose nuotraukose matomą Liebherr įrangą ir gamyklos konstrukcijos vizualinius požymius; gamintojo lentelė viešai neparodyta.</t>
         </is>
       </c>
       <c r="U66" s="5" t="n">
-        <v>0.98</v>
+        <v>0.72</v>
       </c>
       <c r="V66" s="2" t="inlineStr">
         <is>
-          <t>https://www.ponasbetonas.lt/</t>
+          <t>https://www.pabradesbetonas.lt/</t>
         </is>
       </c>
       <c r="W66" s="2" t="inlineStr">
         <is>
-          <t>https://www.ponasbetonas.lt/#Apiemus</t>
+          <t>https://www.pabradesbetonas.lt/</t>
         </is>
       </c>
       <c r="X66" s="2" t="inlineStr">
         <is>
-          <t>https://www.ponasbetonas.lt/</t>
+          <t>https://www.pabradesbetonas.lt/galerija/</t>
         </is>
       </c>
       <c r="Y66" s="2" t="inlineStr">
         <is>
-          <t>Nuosavas betono mazgas ir prekinio betono gamyba patvirtinti oficialiame įmonės puslapyje. Mazgo gamintojas nustatytas pagal oficialaus puslapio hero nuotraukoje ant silosų matomą ELKON ženklinimą; modelis, maišyklė ir našumas viešai nenurodyti. Tiksli mazgo lokacija paimta iš naudotojo pateiktos Google Maps nuorodos; vietovė patikslinta pagal OpenStreetMap. Įmonės kodas patvirtintas Registrų centro viešame juridinio asmens pranešime.</t>
+          <t>Adresas, įmonės kodas ir betono gamyba patvirtinti oficialioje svetainėje bei viešame gamybos kontrolės sertifikate. Koordinatės paimtos iš oficialioje svetainėje pateiktos Google Maps nuorodos. Maišyklės tūris 3 m³, realus našumas 60 m³/val. ir silosai 3x65 t įrašyti pagal naudotojo pateiktą informaciją. Gamintojas Liebherr nurodytas kaip tikėtinas pagal oficialios galerijos nuotraukas; viešo gamintojo ženklinimo ant paties mazgo nerasta.</t>
         </is>
       </c>
       <c r="Z66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>pabrades-betonas-pabrade</t>
+          <t>alkesta-marijampole-vasaros</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>306177188</t>
+          <t>249672710</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>UAB Pabradės betonas</t>
+          <t>UAB Alkesta</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Pabradės betonas</t>
+          <t>Alkesta</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -8153,38 +8165,38 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Pabradė</t>
+          <t>Marijampolė</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Švenčionių r. sav.</t>
+          <t>Marijampolės sav.</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus g. 161, Pabradė, LT-18177 Švenčionių r.</t>
+          <t>Vasaros g. 14, Marijampolė, LT-68111</t>
         </is>
       </c>
       <c r="I67" s="3" t="n">
-        <v>54.9758768</v>
+        <v>54.5686121</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>25.7373849</v>
+        <v>23.3895157</v>
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>Tikslus oficialioje svetainėje pateiktos Google Maps nuorodos taškas</t>
+          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>Oficiali Pabradės betono Google Maps nuoroda</t>
+          <t>Naudotojo pateikta Google Maps lokacija</t>
         </is>
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/TQBCVR8DczDRvQaeA</t>
+          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
         </is>
       </c>
       <c r="N67" s="2" t="inlineStr">
@@ -8199,50 +8211,46 @@
       </c>
       <c r="P67" s="2" t="inlineStr">
         <is>
-          <t>Liebherr (tikėtina)</t>
+          <t>Elba</t>
         </is>
       </c>
       <c r="Q67" s="2" t="inlineStr">
         <is>
-          <t>3 m³</t>
+          <t>0,5 m³</t>
         </is>
       </c>
       <c r="R67" s="2" t="inlineStr">
         <is>
-          <t>60 m³/val.</t>
-        </is>
-      </c>
-      <c r="S67" s="4" t="inlineStr">
-        <is>
-          <t>3x65 t</t>
-        </is>
-      </c>
+          <t>10 m³/val.</t>
+        </is>
+      </c>
+      <c r="S67" s="4" t="inlineStr"/>
       <c r="T67" s="2" t="inlineStr">
         <is>
-          <t>UAB Pabradės betonas Vilniaus g. 161, Pabradėje, gamina sertifikuotą normalųjį betoną ir oficialiai nurodo dirbanti 50 km spinduliu aplink Pabradę. Oficialios galerijos nuotraukose matoma stacionari gamybos bazė su trimis cemento silosais. Mazgo gamintojas tikėtinai Liebherr pagal oficialiose nuotraukose matomą Liebherr įrangą ir gamyklos konstrukcijos vizualinius požymius; gamintojo lentelė viešai neparodyta.</t>
+          <t>UAB Alkesta Marijampolės betono mazgas Vasaros g. 14. Mazgo gamintojas Elba, maišyklė 0,5 m³, našumas 10 m³/val.</t>
         </is>
       </c>
       <c r="U67" s="5" t="n">
-        <v>0.72</v>
+        <v>0.95</v>
       </c>
       <c r="V67" s="2" t="inlineStr">
         <is>
-          <t>https://www.pabradesbetonas.lt/</t>
+          <t>https://alkesta.lt/</t>
         </is>
       </c>
       <c r="W67" s="2" t="inlineStr">
         <is>
-          <t>https://www.pabradesbetonas.lt/</t>
+          <t>https://spsc.lt/registrai/regsapp/ser_produktai_view.php?editid1=13061</t>
         </is>
       </c>
       <c r="X67" s="2" t="inlineStr">
         <is>
-          <t>https://www.pabradesbetonas.lt/galerija/</t>
+          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
         </is>
       </c>
       <c r="Y67" s="2" t="inlineStr">
         <is>
-          <t>Adresas, įmonės kodas ir betono gamyba patvirtinti oficialioje svetainėje bei viešame gamybos kontrolės sertifikate. Koordinatės paimtos iš oficialioje svetainėje pateiktos Google Maps nuorodos. Maišyklės tūris 3 m³, realus našumas 60 m³/val. ir silosai 3x65 t įrašyti pagal naudotojo pateiktą informaciją. Gamintojas Liebherr nurodytas kaip tikėtinas pagal oficialios galerijos nuotraukas; viešo gamintojo ženklinimo ant paties mazgo nerasta.</t>
+          <t>Oficialus SPSC sertifikatų registras patvirtina UAB Alkesta betono gamybą ir gamybos vietą Vasaros g. 14, Marijampolėje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris ir našumas įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z67" s="2" t="inlineStr">
@@ -8254,22 +8262,22 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>alkesta-marijampole-vasaros</t>
+          <t>gevalda-visincia</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>249672710</t>
+          <t>302592895</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>UAB Alkesta</t>
+          <t>UAB Gevalda</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Alkesta</t>
+          <t>Gevalda</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -8279,24 +8287,24 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Marijampolė</t>
+          <t>Visinčia</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Marijampolės sav.</t>
+          <t>Šalčininkų r. sav.</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>Vasaros g. 14, Marijampolė, LT-68111</t>
+          <t>Visinčia, Pabarės sen., Šalčininkų r. sav.</t>
         </is>
       </c>
       <c r="I68" s="3" t="n">
-        <v>54.5686121</v>
+        <v>54.4122467</v>
       </c>
       <c r="J68" s="3" t="n">
-        <v>23.3895157</v>
+        <v>25.1449142</v>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
@@ -8310,7 +8318,7 @@
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
+          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
         </is>
       </c>
       <c r="N68" s="2" t="inlineStr">
@@ -8325,23 +8333,27 @@
       </c>
       <c r="P68" s="2" t="inlineStr">
         <is>
-          <t>Elba</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t>0,5 m³</t>
+          <t>3 m³</t>
         </is>
       </c>
       <c r="R68" s="2" t="inlineStr">
         <is>
-          <t>10 m³/val.</t>
-        </is>
-      </c>
-      <c r="S68" s="4" t="inlineStr"/>
+          <t>60 m³/val.</t>
+        </is>
+      </c>
+      <c r="S68" s="4" t="inlineStr">
+        <is>
+          <t>2x85 t</t>
+        </is>
+      </c>
       <c r="T68" s="2" t="inlineStr">
         <is>
-          <t>UAB Alkesta Marijampolės betono mazgas Vasaros g. 14. Mazgo gamintojas Elba, maišyklė 0,5 m³, našumas 10 m³/val.</t>
+          <t>UAB Gevalda mobilus betono mazgas Visinčioje. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U68" s="5" t="n">
@@ -8349,22 +8361,22 @@
       </c>
       <c r="V68" s="2" t="inlineStr">
         <is>
-          <t>https://alkesta.lt/</t>
+          <t>https://www.gevalda.lt/</t>
         </is>
       </c>
       <c r="W68" s="2" t="inlineStr">
         <is>
-          <t>https://spsc.lt/registrai/regsapp/ser_produktai_view.php?editid1=13061</t>
+          <t>https://www.gevalda.lt/paslaugos/gamyba</t>
         </is>
       </c>
       <c r="X68" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
+          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
         </is>
       </c>
       <c r="Y68" s="2" t="inlineStr">
         <is>
-          <t>Oficialus SPSC sertifikatų registras patvirtina UAB Alkesta betono gamybą ir gamybos vietą Vasaros g. 14, Marijampolėje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris ir našumas įrašyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris, našumas ir silosai įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z68" s="2" t="inlineStr">
@@ -8376,7 +8388,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>gevalda-visincia</t>
+          <t>gevalda-kaunas-palemonas</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -8401,24 +8413,24 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Visinčia</t>
+          <t>Kaunas</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Šalčininkų r. sav.</t>
+          <t>Kauno m. sav.</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>Visinčia, Pabarės sen., Šalčininkų r. sav.</t>
+          <t>Kražantės g., Palemonas, Kaunas</t>
         </is>
       </c>
       <c r="I69" s="3" t="n">
-        <v>54.4122467</v>
+        <v>54.918</v>
       </c>
       <c r="J69" s="3" t="n">
-        <v>25.1449142</v>
+        <v>24.063</v>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
@@ -8432,7 +8444,7 @@
       </c>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
+          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
         </is>
       </c>
       <c r="N69" s="2" t="inlineStr">
@@ -8467,7 +8479,7 @@
       </c>
       <c r="T69" s="2" t="inlineStr">
         <is>
-          <t>UAB Gevalda mobilus betono mazgas Visinčioje. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
+          <t>UAB Gevalda mobilus betono mazgas Palemone, Kaune. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U69" s="5" t="n">
@@ -8485,148 +8497,22 @@
       </c>
       <c r="X69" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
+          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
         </is>
       </c>
       <c r="Y69" s="2" t="inlineStr">
         <is>
-          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris, našumas ir silosai įrašyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija ir analogiški techniniai duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z69" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>gevalda-kaunas-palemonas</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>302592895</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>UAB Gevalda</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>Gevalda</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>Konkurentas</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>Kaunas</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>Kauno m. sav.</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>Kražantės g., Palemonas, Kaunas</t>
-        </is>
-      </c>
-      <c r="I70" s="3" t="n">
-        <v>54.918</v>
-      </c>
-      <c r="J70" s="3" t="n">
-        <v>24.063</v>
-      </c>
-      <c r="K70" s="2" t="inlineStr">
-        <is>
-          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
-        </is>
-      </c>
-      <c r="L70" s="2" t="inlineStr">
-        <is>
-          <t>Naudotojo pateikta Google Maps lokacija</t>
-        </is>
-      </c>
-      <c r="M70" s="2" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
-        </is>
-      </c>
-      <c r="N70" s="2" t="inlineStr">
-        <is>
-          <t>ready_mix_concrete</t>
-        </is>
-      </c>
-      <c r="O70" s="2" t="inlineStr">
-        <is>
-          <t>Betono mišiniai</t>
-        </is>
-      </c>
-      <c r="P70" s="2" t="inlineStr">
-        <is>
-          <t>Elkon</t>
-        </is>
-      </c>
-      <c r="Q70" s="2" t="inlineStr">
-        <is>
-          <t>3 m³</t>
-        </is>
-      </c>
-      <c r="R70" s="2" t="inlineStr">
-        <is>
-          <t>60 m³/val.</t>
-        </is>
-      </c>
-      <c r="S70" s="4" t="inlineStr">
-        <is>
-          <t>2x85 t</t>
-        </is>
-      </c>
-      <c r="T70" s="2" t="inlineStr">
-        <is>
-          <t>UAB Gevalda mobilus betono mazgas Palemone, Kaune. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
-        </is>
-      </c>
-      <c r="U70" s="5" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="V70" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gevalda.lt/</t>
-        </is>
-      </c>
-      <c r="W70" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gevalda.lt/paslaugos/gamyba</t>
-        </is>
-      </c>
-      <c r="X70" s="2" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
-        </is>
-      </c>
-      <c r="Y70" s="2" t="inlineStr">
-        <is>
-          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija ir analogiški techniniai duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
-        </is>
-      </c>
-      <c r="Z70" s="2" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z70"/>
+  <autoFilter ref="A1:Z69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8715,7 +8601,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-23T15:50:11.921774+00:00</t>
+          <t>2026-09-23T15:57:21.399333+00:00</t>
         </is>
       </c>
     </row>
@@ -8770,7 +8656,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-23T15:50:11.921774+00:00</t>
+          <t>2026-09-23T15:57:21.399333+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8784,7 +8670,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Papildyti Betono bazes techninius duomenis
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -4112,16 +4112,28 @@
           <t>Betono bazė</t>
         </is>
       </c>
-      <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="inlineStr"/>
-      <c r="S31" s="4" t="inlineStr"/>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>1 m³</t>
+        </is>
+      </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>20-30 m³/val.</t>
+        </is>
+      </c>
+      <c r="S31" s="4" t="inlineStr">
+        <is>
+          <t>2x50 t (horizontalūs)</t>
+        </is>
+      </c>
       <c r="T31" s="2" t="inlineStr">
         <is>
-          <t>Viešuose šaltiniuose minima betono mišinių veikla; tikslų mazgo adresą reikia patikslinti.</t>
+          <t>UAB Betono bazė betono mazgas Elektrinės g. 11, Drūkšinių k. Maišyklė 1 m³, našumas 20-30 m³/val., du horizontalūs po 50 t silosai.</t>
         </is>
       </c>
       <c r="U31" s="5" t="n">
-        <v>0.65</v>
+        <v>0.95</v>
       </c>
       <c r="V31" s="2" t="inlineStr">
         <is>
@@ -4140,12 +4152,12 @@
       </c>
       <c r="Y31" s="2" t="inlineStr">
         <is>
-          <t>Oficialus kontaktų puslapis patvirtina Elektrinės g. 11 adresą ir betono bazės veiklą.</t>
+          <t>Oficialus kontaktų puslapis patvirtina Elektrinės g. 11 adresą ir betono bazės veiklą. Maišyklės tūris, našumas ir horizontalių silosų skaičius bei talpa įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z31" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8613,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-23T15:57:21.399333+00:00</t>
+          <t>2026-09-24T04:22:17.382218+00:00</t>
         </is>
       </c>
     </row>
@@ -8656,7 +8668,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-23T15:57:21.399333+00:00</t>
+          <t>2026-09-24T04:22:17.383221+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Pasalinti du taskus ir pazymeti Silutes mazga
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$67</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z69" headerRowCount="1">
-  <autoFilter ref="A1:Z69"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z67" headerRowCount="1">
+  <autoFilter ref="A1:Z67"/>
   <tableColumns count="26">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z69"/>
+  <dimension ref="A1:Z67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -4618,18 +4618,18 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>re-betono-konstrukcijos-kretinga</t>
+          <t>silales-statyba-vingininkai</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>UAB RE Betono konstrukcijos</t>
+          <t>UAB Šilalės statyba</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>RE Betono konstrukcijos</t>
+          <t>Šilalės statyba</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -4639,24 +4639,24 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Kretinga</t>
+          <t>Vingininkai</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Kretingos r. sav.</t>
+          <t>Šilalės r. sav.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Tiekėjų g. 27B, Kretinga</t>
+          <t>Lauryno Ivinskio g. 7, Vingininkai, Šilalės r.</t>
         </is>
       </c>
       <c r="I36" s="3" t="n">
-        <v>55.87963</v>
+        <v>55.4808479</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>21.220888</v>
+        <v>22.1937399</v>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
@@ -4685,7 +4685,7 @@
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>RE Betono konstrukcijų gamyba</t>
+          <t>Šilalės statybos betono gaminių gamyba</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr"/>
@@ -4693,26 +4693,30 @@
       <c r="S36" s="4" t="inlineStr"/>
       <c r="T36" s="2" t="inlineStr">
         <is>
-          <t>Viešame kataloge nurodomi betonas, cemento gaminiai, betono siurblys ir pamatų blokai Kretingoje.</t>
+          <t>Viešai skelbiama betono gaminių ir statybinių konstrukcijų veikla Šilalės rajone.</t>
         </is>
       </c>
       <c r="U36" s="5" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="V36" s="2" t="inlineStr"/>
+        <v>0.72</v>
+      </c>
+      <c r="V36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.silalesstatyba.lt/</t>
+        </is>
+      </c>
       <c r="W36" s="2" t="inlineStr">
         <is>
-          <t>https://www.1551.lt/re-betono-konstrukcijos-uab-betonas-cementas-betono-siurblys-pamatu-blokai-kretingoje-104253/</t>
+          <t>https://www.silalesstatyba.lt/</t>
         </is>
       </c>
       <c r="X36" s="2" t="inlineStr">
         <is>
-          <t>https://www.1551.lt/re-betono-konstrukcijos-uab-betonas-cementas-betono-siurblys-pamatu-blokai-kretingoje-104253/</t>
+          <t>https://www.silalesstatyba.lt/</t>
         </is>
       </c>
       <c r="Y36" s="2" t="inlineStr">
         <is>
-          <t>Katalogo šaltinis, reikia patikslinti gamybos apimtį.</t>
+          <t>Reikia patikslinti tikslų gaminių asortimentą.</t>
         </is>
       </c>
       <c r="Z36" s="2" t="inlineStr">
@@ -4724,18 +4728,18 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>silales-statyba-vingininkai</t>
+          <t>panevezio-gelzbetonis-panevezys</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>UAB Šilalės statyba</t>
+          <t>UAB Panevėžio gelžbetonis</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Šilalės statyba</t>
+          <t>Panevėžio gelžbetonis</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -4745,24 +4749,24 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Vingininkai</t>
+          <t>Panevėžys</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Šilalės r. sav.</t>
+          <t>Panevėžio m. sav.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Lauryno Ivinskio g. 7, Vingininkai, Šilalės r.</t>
+          <t>S. Kerbedžio g. 52, Panevėžys</t>
         </is>
       </c>
       <c r="I37" s="3" t="n">
-        <v>55.4808479</v>
+        <v>55.7409491</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>22.1937399</v>
+        <v>24.3803541</v>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
@@ -4786,12 +4790,12 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>Betono gaminiai</t>
+          <t>Gelžbetonis</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>Šilalės statybos betono gaminių gamyba</t>
+          <t>Panevėžio gelžbetonio gamykla</t>
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr"/>
@@ -4799,30 +4803,26 @@
       <c r="S37" s="4" t="inlineStr"/>
       <c r="T37" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono gaminių ir statybinių konstrukcijų veikla Šilalės rajone.</t>
+          <t>Viešame įmonių kataloge nurodomas gelžbetonio gaminių profilis Panevėžyje.</t>
         </is>
       </c>
       <c r="U37" s="5" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="V37" s="2" t="inlineStr">
-        <is>
-          <t>https://www.silalesstatyba.lt/</t>
-        </is>
-      </c>
+        <v>0.78</v>
+      </c>
+      <c r="V37" s="2" t="inlineStr"/>
       <c r="W37" s="2" t="inlineStr">
         <is>
-          <t>https://www.silalesstatyba.lt/</t>
+          <t>https://www.spec.lt/imone/panevezio-gelzbetonis-uab</t>
         </is>
       </c>
       <c r="X37" s="2" t="inlineStr">
         <is>
-          <t>https://www.silalesstatyba.lt/</t>
+          <t>https://www.spec.lt/imone/panevezio-gelzbetonis-uab</t>
         </is>
       </c>
       <c r="Y37" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti tikslų gaminių asortimentą.</t>
+          <t>Reikia patikrinti veiklos aktyvumą ir produkcijos apimtį.</t>
         </is>
       </c>
       <c r="Z37" s="2" t="inlineStr">
@@ -4834,18 +4834,18 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>panevezio-gelzbetonis-panevezys</t>
+          <t>pamatas-telsiai</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr"/>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>UAB Panevėžio gelžbetonis</t>
+          <t>UAB Pamatas</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Panevėžio gelžbetonis</t>
+          <t>Pamatas</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -4855,24 +4855,24 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Panevėžys</t>
+          <t>Telšiai</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Panevėžio m. sav.</t>
+          <t>Telšių r. sav.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>S. Kerbedžio g. 52, Panevėžys</t>
+          <t>Tryškių g. 46, Dimaičių k., Telšių r.</t>
         </is>
       </c>
       <c r="I38" s="3" t="n">
-        <v>55.7409491</v>
+        <v>55.9874536</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>24.3803541</v>
+        <v>22.287162</v>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
@@ -4896,12 +4896,12 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>Gelžbetonis</t>
+          <t>Betono gaminiai</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>Panevėžio gelžbetonio gamykla</t>
+          <t>Pamatas betono gaminių gamyba</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr"/>
@@ -4909,26 +4909,30 @@
       <c r="S38" s="4" t="inlineStr"/>
       <c r="T38" s="2" t="inlineStr">
         <is>
-          <t>Viešame įmonių kataloge nurodomas gelžbetonio gaminių profilis Panevėžyje.</t>
+          <t>Viešai skelbiami pamatų ir kiti betono gaminiai Telšių rajone.</t>
         </is>
       </c>
       <c r="U38" s="5" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="V38" s="2" t="inlineStr"/>
+        <v>0.72</v>
+      </c>
+      <c r="V38" s="2" t="inlineStr">
+        <is>
+          <t>https://pamatas.lt/</t>
+        </is>
+      </c>
       <c r="W38" s="2" t="inlineStr">
         <is>
-          <t>https://www.spec.lt/imone/panevezio-gelzbetonis-uab</t>
+          <t>https://pamatas.lt/</t>
         </is>
       </c>
       <c r="X38" s="2" t="inlineStr">
         <is>
-          <t>https://www.spec.lt/imone/panevezio-gelzbetonis-uab</t>
+          <t>https://pamatas.lt/</t>
         </is>
       </c>
       <c r="Y38" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikrinti veiklos aktyvumą ir produkcijos apimtį.</t>
+          <t>Adresas patikslintas pagal lietuvišką įmonės puslapį; koordinatės nustatytos Lietuvos geolokatoriumi.</t>
         </is>
       </c>
       <c r="Z38" s="2" t="inlineStr">
@@ -4940,18 +4944,18 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>pamatas-telsiai</t>
+          <t>betono-zona-klaipeda</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr"/>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>UAB Pamatas</t>
+          <t>UAB Betono zona</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Pamatas</t>
+          <t>Betono zona</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -4961,24 +4965,24 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Telšiai</t>
+          <t>Klaipėda</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Telšių r. sav.</t>
+          <t>Klaipėdos m. sav.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Tryškių g. 46, Dimaičių k., Telšių r.</t>
+          <t>Dvaro g. 6, Klaipėda</t>
         </is>
       </c>
       <c r="I39" s="3" t="n">
-        <v>55.9874536</v>
+        <v>55.7549809</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>22.287162</v>
+        <v>21.150509</v>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
@@ -5007,7 +5011,7 @@
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>Pamatas betono gaminių gamyba</t>
+          <t>Betono zona</t>
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr"/>
@@ -5015,30 +5019,30 @@
       <c r="S39" s="4" t="inlineStr"/>
       <c r="T39" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiami pamatų ir kiti betono gaminiai Telšių rajone.</t>
+          <t>Viešai skelbiama betono gaminių veikla Klaipėdoje.</t>
         </is>
       </c>
       <c r="U39" s="5" t="n">
-        <v>0.72</v>
+        <v>0.65</v>
       </c>
       <c r="V39" s="2" t="inlineStr">
         <is>
-          <t>https://pamatas.lt/</t>
+          <t>https://betonozona.lt/</t>
         </is>
       </c>
       <c r="W39" s="2" t="inlineStr">
         <is>
-          <t>https://pamatas.lt/</t>
+          <t>https://betonozona.lt/</t>
         </is>
       </c>
       <c r="X39" s="2" t="inlineStr">
         <is>
-          <t>https://pamatas.lt/</t>
+          <t>https://betonozona.lt/</t>
         </is>
       </c>
       <c r="Y39" s="2" t="inlineStr">
         <is>
-          <t>Adresas patikslintas pagal lietuvišką įmonės puslapį; koordinatės nustatytos Lietuvos geolokatoriumi.</t>
+          <t>Patikrinti, ar įmonė pati gamina, ar tik prekiauja betono gaminiais.</t>
         </is>
       </c>
       <c r="Z39" s="2" t="inlineStr">
@@ -5050,18 +5054,22 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>pamario-grupe-kalnuvenai</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr"/>
+          <t>topbeton-panevezys</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>307083610</t>
+        </is>
+      </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>UAB Pamario grupė</t>
+          <t>UAB Topbeton</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Pamario grupė</t>
+          <t>Topbeton</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -5071,24 +5079,24 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Kalnuvėnai</t>
+          <t>Panevėžys</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Klaipėdos r. sav.</t>
+          <t>Panevėžio m. sav.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Kaukėnų g. 12, Kalnuvėnai, Klaipėdos r.</t>
+          <t>Beržų g. 5C, Panevėžys</t>
         </is>
       </c>
       <c r="I40" s="3" t="n">
-        <v>55.7905468</v>
+        <v>55.7168572</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>21.1471136</v>
+        <v>24.3617863</v>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
@@ -5117,7 +5125,7 @@
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>Pamario grupės betono mazgas</t>
+          <t>Topbeton betono mazgas</t>
         </is>
       </c>
       <c r="Q40" s="2" t="inlineStr"/>
@@ -5125,30 +5133,30 @@
       <c r="S40" s="4" t="inlineStr"/>
       <c r="T40" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono mišinių veikla Klaipėdos rajone.</t>
+          <t>Viešai skelbiama betono mišinių gamyba Panevėžyje.</t>
         </is>
       </c>
       <c r="U40" s="5" t="n">
-        <v>0.75</v>
+        <v>0.78</v>
       </c>
       <c r="V40" s="2" t="inlineStr">
         <is>
-          <t>https://pamariogrupe.lt/</t>
+          <t>https://topbeton.lt/</t>
         </is>
       </c>
       <c r="W40" s="2" t="inlineStr">
         <is>
-          <t>https://pamariogrupe.lt/</t>
+          <t>https://www.topbeton.lt/kontaktai/</t>
         </is>
       </c>
       <c r="X40" s="2" t="inlineStr">
         <is>
-          <t>https://pamariogrupe.lt/</t>
+          <t>https://www.topbeton.lt/kontaktai/</t>
         </is>
       </c>
       <c r="Y40" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti našumą ir gamybos režimą.</t>
+          <t>Oficialus kontaktų puslapis patvirtina Beržų g. 5C adresą.</t>
         </is>
       </c>
       <c r="Z40" s="2" t="inlineStr">
@@ -5160,18 +5168,18 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>betono-zona-klaipeda</t>
+          <t>gelzbetonio-gamyba-panevezys</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr"/>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>UAB Betono zona</t>
+          <t>MB Gelžbetonio gamyba</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Betono zona</t>
+          <t>Gelžbetonio gamyba</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -5181,24 +5189,24 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Klaipėda</t>
+          <t>Panevėžys</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Klaipėdos m. sav.</t>
+          <t>Panevėžio m. sav.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Dvaro g. 6, Klaipėda</t>
+          <t>S. Kerbedžio g. 52, Panevėžys</t>
         </is>
       </c>
       <c r="I41" s="3" t="n">
-        <v>55.7549809</v>
+        <v>55.7409491</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>21.150509</v>
+        <v>24.3803541</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
@@ -5222,12 +5230,12 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>Betono gaminiai</t>
+          <t>Gelžbetonis</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>Betono zona</t>
+          <t>Gelžbetonio gamyba Panevėžyje</t>
         </is>
       </c>
       <c r="Q41" s="2" t="inlineStr"/>
@@ -5235,30 +5243,30 @@
       <c r="S41" s="4" t="inlineStr"/>
       <c r="T41" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono gaminių veikla Klaipėdoje.</t>
+          <t>Viešai skelbiama gelžbetonio gaminių gamyba Panevėžyje.</t>
         </is>
       </c>
       <c r="U41" s="5" t="n">
-        <v>0.65</v>
+        <v>0.72</v>
       </c>
       <c r="V41" s="2" t="inlineStr">
         <is>
-          <t>https://betonozona.lt/</t>
+          <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
       <c r="W41" s="2" t="inlineStr">
         <is>
-          <t>https://betonozona.lt/</t>
+          <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
       <c r="X41" s="2" t="inlineStr">
         <is>
-          <t>https://betonozona.lt/</t>
+          <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
       <c r="Y41" s="2" t="inlineStr">
         <is>
-          <t>Patikrinti, ar įmonė pati gamina, ar tik prekiauja betono gaminiais.</t>
+          <t>Reikia patikslinti ryšį su kitomis S. Kerbedžio g. 52 įmonėmis.</t>
         </is>
       </c>
       <c r="Z41" s="2" t="inlineStr">
@@ -5270,22 +5278,18 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>topbeton-panevezys</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>307083610</t>
-        </is>
-      </c>
+          <t>inroma-pakruojis</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>UAB Topbeton</t>
+          <t>UAB Inroma</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Topbeton</t>
+          <t>Inroma</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -5295,24 +5299,24 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Panevėžys</t>
+          <t>Pakruojis</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Panevėžio m. sav.</t>
+          <t>Pakruojo r. sav.</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Beržų g. 5C, Panevėžys</t>
+          <t>Pramonės g. 5B, Pakruojis</t>
         </is>
       </c>
       <c r="I42" s="3" t="n">
-        <v>55.7168572</v>
+        <v>55.9763263</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>24.3617863</v>
+        <v>23.8584712</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -5341,7 +5345,7 @@
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>Topbeton betono mazgas</t>
+          <t>Inroma betono mazgas</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr"/>
@@ -5349,30 +5353,30 @@
       <c r="S42" s="4" t="inlineStr"/>
       <c r="T42" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono mišinių gamyba Panevėžyje.</t>
+          <t>Viešai skelbiama betono mišinių veikla Pakruojyje.</t>
         </is>
       </c>
       <c r="U42" s="5" t="n">
-        <v>0.78</v>
+        <v>0.72</v>
       </c>
       <c r="V42" s="2" t="inlineStr">
         <is>
-          <t>https://topbeton.lt/</t>
+          <t>https://inroma.lt/</t>
         </is>
       </c>
       <c r="W42" s="2" t="inlineStr">
         <is>
-          <t>https://www.topbeton.lt/kontaktai/</t>
+          <t>https://inroma.lt/</t>
         </is>
       </c>
       <c r="X42" s="2" t="inlineStr">
         <is>
-          <t>https://www.topbeton.lt/kontaktai/</t>
+          <t>https://inroma.lt/</t>
         </is>
       </c>
       <c r="Y42" s="2" t="inlineStr">
         <is>
-          <t>Oficialus kontaktų puslapis patvirtina Beržų g. 5C adresą.</t>
+          <t>Reikia patikslinti našumą.</t>
         </is>
       </c>
       <c r="Z42" s="2" t="inlineStr">
@@ -5384,18 +5388,22 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>gelzbetonio-gamyba-panevezys</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr"/>
+          <t>utenos-betonas-utena</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>300904691</t>
+        </is>
+      </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>MB Gelžbetonio gamyba</t>
+          <t>UAB Utenos betonas</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Gelžbetonio gamyba</t>
+          <t>Utenos betonas</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -5405,24 +5413,24 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Panevėžys</t>
+          <t>Utena</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Panevėžio m. sav.</t>
+          <t>Utenos r. sav.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>S. Kerbedžio g. 52, Panevėžys</t>
+          <t>Metalo g. 9B, Utena</t>
         </is>
       </c>
       <c r="I43" s="3" t="n">
-        <v>55.7409491</v>
+        <v>55.4947607</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>24.3803541</v>
+        <v>25.6225075</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
@@ -5441,17 +5449,17 @@
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>precast_concrete</t>
+          <t>ready_mix_concrete</t>
         </is>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>Gelžbetonis</t>
+          <t>Betono mišiniai</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>Gelžbetonio gamyba Panevėžyje</t>
+          <t>Utenos betono mazgas</t>
         </is>
       </c>
       <c r="Q43" s="2" t="inlineStr"/>
@@ -5459,30 +5467,30 @@
       <c r="S43" s="4" t="inlineStr"/>
       <c r="T43" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama gelžbetonio gaminių gamyba Panevėžyje.</t>
+          <t>Viešai skelbiama betono mišinių veikla Utenoje.</t>
         </is>
       </c>
       <c r="U43" s="5" t="n">
-        <v>0.72</v>
+        <v>0.78</v>
       </c>
       <c r="V43" s="2" t="inlineStr">
         <is>
-          <t>https://gelzbetoniogamyba.lt/</t>
+          <t>https://utenosbetonas.lt/</t>
         </is>
       </c>
       <c r="W43" s="2" t="inlineStr">
         <is>
-          <t>https://gelzbetoniogamyba.lt/</t>
+          <t>https://www.utenosbetonas.lt/kontaktai/</t>
         </is>
       </c>
       <c r="X43" s="2" t="inlineStr">
         <is>
-          <t>https://gelzbetoniogamyba.lt/</t>
+          <t>https://www.utenosbetonas.lt/kontaktai/</t>
         </is>
       </c>
       <c r="Y43" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti ryšį su kitomis S. Kerbedžio g. 52 įmonėmis.</t>
+          <t>Oficialus kontaktų puslapis patvirtina Metalo g. 9B adresą.</t>
         </is>
       </c>
       <c r="Z43" s="2" t="inlineStr">
@@ -5494,18 +5502,22 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>inroma-pakruojis</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr"/>
+          <t>sbetonas-jonava</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>300902683</t>
+        </is>
+      </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>UAB Inroma</t>
+          <t>UAB Sbetonas</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Inroma</t>
+          <t>Sbetonas</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -5515,24 +5527,24 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Pakruojis</t>
+          <t>Jonava</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Pakruojo r. sav.</t>
+          <t>Jonavos r. sav.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Pramonės g. 5B, Pakruojis</t>
+          <t>Skarulių g. 58, Jonava</t>
         </is>
       </c>
       <c r="I44" s="3" t="n">
-        <v>55.9763263</v>
+        <v>55.0786452</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>23.8584712</v>
+        <v>24.3199072</v>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
@@ -5561,7 +5573,7 @@
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>Inroma betono mazgas</t>
+          <t>Sbetonas betono mazgas</t>
         </is>
       </c>
       <c r="Q44" s="2" t="inlineStr"/>
@@ -5569,30 +5581,30 @@
       <c r="S44" s="4" t="inlineStr"/>
       <c r="T44" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono mišinių veikla Pakruojyje.</t>
+          <t>Viešai skelbiama prekinio betono gamyba Jonavoje.</t>
         </is>
       </c>
       <c r="U44" s="5" t="n">
-        <v>0.72</v>
+        <v>0.78</v>
       </c>
       <c r="V44" s="2" t="inlineStr">
         <is>
-          <t>https://inroma.lt/</t>
+          <t>https://sbetonas.lt/</t>
         </is>
       </c>
       <c r="W44" s="2" t="inlineStr">
         <is>
-          <t>https://inroma.lt/</t>
+          <t>https://sbetonas.lt/</t>
         </is>
       </c>
       <c r="X44" s="2" t="inlineStr">
         <is>
-          <t>https://inroma.lt/</t>
+          <t>https://sbetonas.lt/</t>
         </is>
       </c>
       <c r="Y44" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti našumą.</t>
+          <t>Papildomai rasta pagal prekinio betono požymį.</t>
         </is>
       </c>
       <c r="Z44" s="2" t="inlineStr">
@@ -5604,22 +5616,18 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>utenos-betonas-utena</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>300904691</t>
-        </is>
-      </c>
+          <t>kalcitas-naujoji-akmene</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr"/>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>UAB Utenos betonas</t>
+          <t>AB Kalcitas</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Utenos betonas</t>
+          <t>Kalcitas</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -5629,24 +5637,24 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Utena</t>
+          <t>Naujoji Akmenė</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Utenos r. sav.</t>
+          <t>Akmenės r. sav.</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Metalo g. 9B, Utena</t>
+          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
         </is>
       </c>
       <c r="I45" s="3" t="n">
-        <v>55.4947607</v>
+        <v>56.3143832</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>25.6225075</v>
+        <v>22.9130704</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -5675,7 +5683,7 @@
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>Utenos betono mazgas</t>
+          <t>Kalcitas betono mišinių gamybos linija</t>
         </is>
       </c>
       <c r="Q45" s="2" t="inlineStr"/>
@@ -5683,30 +5691,26 @@
       <c r="S45" s="4" t="inlineStr"/>
       <c r="T45" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono mišinių veikla Utenoje.</t>
+          <t>Viešame kataloge nurodomi betonas, betono mišiniai ir betono gamybos linija Naujojoje Akmenėje.</t>
         </is>
       </c>
       <c r="U45" s="5" t="n">
         <v>0.78</v>
       </c>
-      <c r="V45" s="2" t="inlineStr">
-        <is>
-          <t>https://utenosbetonas.lt/</t>
-        </is>
-      </c>
+      <c r="V45" s="2" t="inlineStr"/>
       <c r="W45" s="2" t="inlineStr">
         <is>
-          <t>https://www.utenosbetonas.lt/kontaktai/</t>
+          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
         </is>
       </c>
       <c r="X45" s="2" t="inlineStr">
         <is>
-          <t>https://www.utenosbetonas.lt/kontaktai/</t>
+          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
         </is>
       </c>
       <c r="Y45" s="2" t="inlineStr">
         <is>
-          <t>Oficialus kontaktų puslapis patvirtina Metalo g. 9B adresą.</t>
+          <t>Reikia patikslinti, ar veikla yra nuolat aktyvi.</t>
         </is>
       </c>
       <c r="Z45" s="2" t="inlineStr">
@@ -5718,22 +5722,18 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>sbetonas-jonava</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>300902683</t>
-        </is>
-      </c>
+          <t>gelgaudiskio-gelzbetonis-gelgaudiskis</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>UAB Sbetonas</t>
+          <t>UAB Gelgaudiškio gelžbetonis</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Sbetonas</t>
+          <t>Gelgaudiškio gelžbetonis</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -5743,24 +5743,24 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Jonava</t>
+          <t>Gelgaudiškis</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Jonavos r. sav.</t>
+          <t>Šakių r. sav.</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Skarulių g. 58, Jonava</t>
+          <t>Vakarų g. 33 D, 71431, Gelgaudiškis</t>
         </is>
       </c>
       <c r="I46" s="3" t="n">
-        <v>55.0786452</v>
+        <v>55.07067</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>24.3199072</v>
+        <v>22.976723</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
@@ -5769,27 +5769,27 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>GLG kontaktų puslapis</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://glg.lt/kontaktai/</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>ready_mix_concrete</t>
+          <t>precast_concrete</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>Betono mišiniai</t>
+          <t>Betono mišiniai ir gelžbetonis</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>Sbetonas betono mazgas</t>
+          <t>Gelgaudiškio gelžbetonio gamykla</t>
         </is>
       </c>
       <c r="Q46" s="2" t="inlineStr"/>
@@ -5797,30 +5797,30 @@
       <c r="S46" s="4" t="inlineStr"/>
       <c r="T46" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama prekinio betono gamyba Jonavoje.</t>
+          <t>Įmonė gamina gelžbetonio gaminius, prekinį ir hidrotechninį betoną bei smėlbetonio mišinius.</t>
         </is>
       </c>
       <c r="U46" s="5" t="n">
-        <v>0.78</v>
+        <v>0.9</v>
       </c>
       <c r="V46" s="2" t="inlineStr">
         <is>
-          <t>https://sbetonas.lt/</t>
+          <t>https://glg.lt/</t>
         </is>
       </c>
       <c r="W46" s="2" t="inlineStr">
         <is>
-          <t>https://sbetonas.lt/</t>
+          <t>https://glg.lt/kontaktai/</t>
         </is>
       </c>
       <c r="X46" s="2" t="inlineStr">
         <is>
-          <t>https://sbetonas.lt/</t>
+          <t>https://glg.lt/betonas/betono-misiniai/</t>
         </is>
       </c>
       <c r="Y46" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta pagal prekinio betono požymį.</t>
+          <t>Patikslinta pagal oficialų glg.lt kontaktų ir įmonės aprašymo puslapius.</t>
         </is>
       </c>
       <c r="Z46" s="2" t="inlineStr">
@@ -5832,45 +5832,49 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>kalcitas-naujoji-akmene</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr"/>
+          <t>ginfa-kutiskiai</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>302680943</t>
+        </is>
+      </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>AB Kalcitas</t>
+          <t>UAB GinFa</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Kalcitas</t>
+          <t>GinFa</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta</t>
+          <t>Papildomai rasta EVRK 23.63</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Naujoji Akmenė</t>
+          <t>Kutiškiai</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Akmenės r. sav.</t>
+          <t>Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
+          <t>Alyvų g. 8, Kutiškiai, Radviliškio r.</t>
         </is>
       </c>
       <c r="I47" s="3" t="n">
-        <v>56.3143832</v>
+        <v>55.8326273</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>22.9130704</v>
+        <v>23.4995317</v>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
@@ -5899,7 +5903,7 @@
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>Kalcitas betono mišinių gamybos linija</t>
+          <t>GinFa betono gamyba</t>
         </is>
       </c>
       <c r="Q47" s="2" t="inlineStr"/>
@@ -5907,26 +5911,22 @@
       <c r="S47" s="4" t="inlineStr"/>
       <c r="T47" s="2" t="inlineStr">
         <is>
-          <t>Viešame kataloge nurodomi betonas, betono mišiniai ir betono gamybos linija Naujojoje Akmenėje.</t>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
       <c r="U47" s="5" t="n">
-        <v>0.78</v>
+        <v>0.82</v>
       </c>
       <c r="V47" s="2" t="inlineStr"/>
       <c r="W47" s="2" t="inlineStr">
         <is>
-          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
-        </is>
-      </c>
-      <c r="X47" s="2" t="inlineStr">
-        <is>
-          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
-        </is>
-      </c>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="X47" s="2" t="inlineStr"/>
       <c r="Y47" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti, ar veikla yra nuolat aktyvi.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z47" s="2" t="inlineStr">
@@ -5938,45 +5938,49 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>gelgaudiskio-gelzbetonis-gelgaudiskis</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr"/>
+          <t>antano-gribino-imone-prienai</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>170687267</t>
+        </is>
+      </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>UAB Gelgaudiškio gelžbetonis</t>
+          <t>IĮ Antano Gribino gamybos ir komercinės veiklos įmonė</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Gelgaudiškio gelžbetonis</t>
+          <t>Antano Gribino įmonė</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta</t>
+          <t>Papildomai rasta EVRK 23.63</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Gelgaudiškis</t>
+          <t>Prienai</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Šakių r. sav.</t>
+          <t>Prienų r. sav.</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Vakarų g. 33 D, 71431, Gelgaudiškis</t>
+          <t>Kęstučio g. 95A, Prienai</t>
         </is>
       </c>
       <c r="I48" s="3" t="n">
-        <v>55.07067</v>
+        <v>54.6523184</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>22.976723</v>
+        <v>23.9696591</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
@@ -5985,27 +5989,27 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>GLG kontaktų puslapis</t>
+          <t>Lietuvos geolokatorius</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>https://glg.lt/kontaktai/</t>
+          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>precast_concrete</t>
+          <t>ready_mix_concrete</t>
         </is>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>Betono mišiniai ir gelžbetonis</t>
+          <t>Betono mišiniai</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>Gelgaudiškio gelžbetonio gamykla</t>
+          <t>Antano Gribino įmonės betono gamyba</t>
         </is>
       </c>
       <c r="Q48" s="2" t="inlineStr"/>
@@ -6013,30 +6017,22 @@
       <c r="S48" s="4" t="inlineStr"/>
       <c r="T48" s="2" t="inlineStr">
         <is>
-          <t>Įmonė gamina gelžbetonio gaminius, prekinį ir hidrotechninį betoną bei smėlbetonio mišinius.</t>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
       <c r="U48" s="5" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="V48" s="2" t="inlineStr">
-        <is>
-          <t>https://glg.lt/</t>
-        </is>
-      </c>
+        <v>0.82</v>
+      </c>
+      <c r="V48" s="2" t="inlineStr"/>
       <c r="W48" s="2" t="inlineStr">
         <is>
-          <t>https://glg.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="X48" s="2" t="inlineStr">
-        <is>
-          <t>https://glg.lt/betonas/betono-misiniai/</t>
-        </is>
-      </c>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="X48" s="2" t="inlineStr"/>
       <c r="Y48" s="2" t="inlineStr">
         <is>
-          <t>Patikslinta pagal oficialų glg.lt kontaktų ir įmonės aprašymo puslapius.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z48" s="2" t="inlineStr">
@@ -6048,22 +6044,22 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>ginfa-kutiskiai</t>
+          <t>vinido-taurage</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>302680943</t>
+          <t>306258220</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>UAB GinFa</t>
+          <t>UAB Vinido</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>GinFa</t>
+          <t>Vinido</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -6073,24 +6069,24 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Kutiškiai</t>
+          <t>Tauragė</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Radviliškio r. sav.</t>
+          <t>Tauragės r. sav.</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Alyvų g. 8, Kutiškiai, Radviliškio r.</t>
+          <t>Gaurės g. 32, Tauragė</t>
         </is>
       </c>
       <c r="I49" s="3" t="n">
-        <v>55.8326273</v>
+        <v>55.2492204</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>23.4995317</v>
+        <v>22.3185845</v>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
@@ -6119,7 +6115,7 @@
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>GinFa betono gamyba</t>
+          <t>Vinido betono gamyba</t>
         </is>
       </c>
       <c r="Q49" s="2" t="inlineStr"/>
@@ -6133,16 +6129,24 @@
       <c r="U49" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V49" s="2" t="inlineStr"/>
+      <c r="V49" s="2" t="inlineStr">
+        <is>
+          <t>https://betonastaurageje.lt/</t>
+        </is>
+      </c>
       <c r="W49" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X49" s="2" t="inlineStr"/>
+          <t>https://betonastaurageje.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X49" s="2" t="inlineStr">
+        <is>
+          <t>https://betonastaurageje.lt/betonas/</t>
+        </is>
+      </c>
       <c r="Y49" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Oficiali Vinido svetainė patvirtina Gaurės g. 32 adresą, betono gamybą ir betono mazgą.</t>
         </is>
       </c>
       <c r="Z49" s="2" t="inlineStr">
@@ -6154,22 +6158,22 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>antano-gribino-imone-prienai</t>
+          <t>santvara-kedainiai</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>170687267</t>
+          <t>304915297</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>IĮ Antano Gribino gamybos ir komercinės veiklos įmonė</t>
+          <t>UAB Santvara</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Antano Gribino įmonė</t>
+          <t>Santvara</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -6179,24 +6183,24 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Prienai</t>
+          <t>Kėdainiai</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Prienų r. sav.</t>
+          <t>Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Kęstučio g. 95A, Prienai</t>
+          <t>Aruodų g. 34, Kėdainiai</t>
         </is>
       </c>
       <c r="I50" s="3" t="n">
-        <v>54.6523184</v>
+        <v>55.2634747</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>23.9696591</v>
+        <v>23.9440384</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
@@ -6225,7 +6229,7 @@
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>Antano Gribino įmonės betono gamyba</t>
+          <t>Santvara betono gamyba</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr"/>
@@ -6239,16 +6243,24 @@
       <c r="U50" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V50" s="2" t="inlineStr"/>
+      <c r="V50" s="2" t="inlineStr">
+        <is>
+          <t>https://santvara.eu/</t>
+        </is>
+      </c>
       <c r="W50" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X50" s="2" t="inlineStr"/>
+          <t>https://santvara.eu/</t>
+        </is>
+      </c>
+      <c r="X50" s="2" t="inlineStr">
+        <is>
+          <t>https://santvara.eu/</t>
+        </is>
+      </c>
       <c r="Y50" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Oficiali Santvara svetainė patvirtina Aruodų g. 34 adresą ir betono bei birių medžiagų veiklą.</t>
         </is>
       </c>
       <c r="Z50" s="2" t="inlineStr">
@@ -6260,22 +6272,22 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>vinido-taurage</t>
+          <t>medis-ir-betonas-naujoji-akmene</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>306258220</t>
+          <t>153074073</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>UAB Vinido</t>
+          <t>AB Medis ir betonas</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Vinido</t>
+          <t>Medis ir betonas</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -6285,24 +6297,24 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Tauragė</t>
+          <t>Naujoji Akmenė</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Tauragės r. sav.</t>
+          <t>Akmenės r. sav.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Gaurės g. 32, Tauragė</t>
+          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
         </is>
       </c>
       <c r="I51" s="3" t="n">
-        <v>55.2492204</v>
+        <v>56.3143832</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>22.3185845</v>
+        <v>22.9130704</v>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
@@ -6331,7 +6343,7 @@
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
-          <t>Vinido betono gamyba</t>
+          <t>Medis ir betonas gamyba</t>
         </is>
       </c>
       <c r="Q51" s="2" t="inlineStr"/>
@@ -6345,24 +6357,16 @@
       <c r="U51" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V51" s="2" t="inlineStr">
-        <is>
-          <t>https://betonastaurageje.lt/</t>
-        </is>
-      </c>
+      <c r="V51" s="2" t="inlineStr"/>
       <c r="W51" s="2" t="inlineStr">
         <is>
-          <t>https://betonastaurageje.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="X51" s="2" t="inlineStr">
-        <is>
-          <t>https://betonastaurageje.lt/betonas/</t>
-        </is>
-      </c>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="X51" s="2" t="inlineStr"/>
       <c r="Y51" s="2" t="inlineStr">
         <is>
-          <t>Oficiali Vinido svetainė patvirtina Gaurės g. 32 adresą, betono gamybą ir betono mazgą.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z51" s="2" t="inlineStr">
@@ -6374,22 +6378,22 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>santvara-kedainiai</t>
+          <t>ekobetonas-marijampole</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>304915297</t>
+          <t>300636364</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>UAB Santvara</t>
+          <t>UAB Ekobetonas</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Santvara</t>
+          <t>Ekobetonas</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -6399,24 +6403,24 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Kėdainiai</t>
+          <t>Marijampolė</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Kėdainių r. sav.</t>
+          <t>Marijampolės sav.</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Aruodų g. 34, Kėdainiai</t>
+          <t>Gamyklų g. 3, Marijampolė</t>
         </is>
       </c>
       <c r="I52" s="3" t="n">
-        <v>55.2634747</v>
+        <v>54.5750142</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>23.9440384</v>
+        <v>23.3796805</v>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
@@ -6445,7 +6449,7 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>Santvara betono gamyba</t>
+          <t>Ekobetonas betono gamyba</t>
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr"/>
@@ -6461,22 +6465,22 @@
       </c>
       <c r="V52" s="2" t="inlineStr">
         <is>
-          <t>https://santvara.eu/</t>
+          <t>https://ekobetonas.lt/</t>
         </is>
       </c>
       <c r="W52" s="2" t="inlineStr">
         <is>
-          <t>https://santvara.eu/</t>
+          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
         </is>
       </c>
       <c r="X52" s="2" t="inlineStr">
         <is>
-          <t>https://santvara.eu/</t>
+          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
         </is>
       </c>
       <c r="Y52" s="2" t="inlineStr">
         <is>
-          <t>Oficiali Santvara svetainė patvirtina Aruodų g. 34 adresą ir betono bei birių medžiagų veiklą.</t>
+          <t>Oficialus Ekobetonas kontaktų puslapis patvirtina Gamyklų g. 3 adresą ir betono užsakymų kontaktus.</t>
         </is>
       </c>
       <c r="Z52" s="2" t="inlineStr">
@@ -6488,22 +6492,22 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>medis-ir-betonas-naujoji-akmene</t>
+          <t>rokbetonis-rokiskis</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>153074073</t>
+          <t>304184091</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>AB Medis ir betonas</t>
+          <t>MB Rokbetonis</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Medis ir betonas</t>
+          <t>Rokbetonis</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -6513,24 +6517,24 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Naujoji Akmenė</t>
+          <t>Rokiškis</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Akmenės r. sav.</t>
+          <t>Rokiškio r. sav.</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
+          <t>Vydūno g. 12A, Parokiškė, Rokiškio r.</t>
         </is>
       </c>
       <c r="I53" s="3" t="n">
-        <v>56.3143832</v>
+        <v>55.9525796</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>22.9130704</v>
+        <v>25.5624197</v>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
@@ -6559,7 +6563,7 @@
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>Medis ir betonas gamyba</t>
+          <t>Rokbetonis betono gamyba</t>
         </is>
       </c>
       <c r="Q53" s="2" t="inlineStr"/>
@@ -6571,7 +6575,7 @@
         </is>
       </c>
       <c r="U53" s="5" t="n">
-        <v>0.82</v>
+        <v>0.72</v>
       </c>
       <c r="V53" s="2" t="inlineStr"/>
       <c r="W53" s="2" t="inlineStr">
@@ -6582,7 +6586,7 @@
       <c r="X53" s="2" t="inlineStr"/>
       <c r="Y53" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Rokiškio miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
         </is>
       </c>
       <c r="Z53" s="2" t="inlineStr">
@@ -6594,22 +6598,22 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>ekobetonas-marijampole</t>
+          <t>silutes-betonas-silute</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>300636364</t>
+          <t>177392928</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>UAB Ekobetonas</t>
+          <t>UAB Šilutės betonas</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Ekobetonas</t>
+          <t>Šilutės betonas</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -6619,24 +6623,24 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Marijampolė</t>
+          <t>Šilutė</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Marijampolės sav.</t>
+          <t>Šilutės r. sav.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Gamyklų g. 3, Marijampolė</t>
+          <t>Ramučių g. 1, Šilutė</t>
         </is>
       </c>
       <c r="I54" s="3" t="n">
-        <v>54.5750142</v>
+        <v>55.3538641</v>
       </c>
       <c r="J54" s="3" t="n">
-        <v>23.3796805</v>
+        <v>21.4796635</v>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
@@ -6665,7 +6669,7 @@
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>Ekobetonas betono gamyba</t>
+          <t>Šilutės betono gamyba (Nebeaktyvus mazgas)</t>
         </is>
       </c>
       <c r="Q54" s="2" t="inlineStr"/>
@@ -6673,57 +6677,53 @@
       <c r="S54" s="4" t="inlineStr"/>
       <c r="T54" s="2" t="inlineStr">
         <is>
-          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+          <t>Nebeaktyvus mazgas. Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
       <c r="U54" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V54" s="2" t="inlineStr">
-        <is>
-          <t>https://ekobetonas.lt/</t>
-        </is>
-      </c>
+      <c r="V54" s="2" t="inlineStr"/>
       <c r="W54" s="2" t="inlineStr">
         <is>
-          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
         </is>
       </c>
       <c r="X54" s="2" t="inlineStr">
         <is>
-          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
+          <t>https://fsaskaita.lt/imone/uzdaroji-akcine-bendrove-silutes-betonas-177392928</t>
         </is>
       </c>
       <c r="Y54" s="2" t="inlineStr">
         <is>
-          <t>Oficialus Ekobetonas kontaktų puslapis patvirtina Gamyklų g. 3 adresą ir betono užsakymų kontaktus.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą. Mazgas pažymėtas nebeaktyviu pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z54" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>rokbetonis-rokiskis</t>
+          <t>kruszbet-lithuania-jure</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>304184091</t>
+          <t>305173596</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>MB Rokbetonis</t>
+          <t>UAB KRUSZBET Lithuania</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Rokbetonis</t>
+          <t>KRUSZBET Lithuania</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -6733,24 +6733,24 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Rokiškis</t>
+          <t>Jūrė</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Rokiškio r. sav.</t>
+          <t>Kazlų Rūdos sav.</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Vydūno g. 12A, Parokiškė, Rokiškio r.</t>
+          <t>Medelyno g. 30A, Jūrė, Kazlų Rūdos sav.</t>
         </is>
       </c>
       <c r="I55" s="3" t="n">
-        <v>55.9525796</v>
+        <v>54.7706307</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>25.5624197</v>
+        <v>23.4998409</v>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
@@ -6779,7 +6779,7 @@
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>Rokbetonis betono gamyba</t>
+          <t>KRUSZBET Lithuania betono gamyba</t>
         </is>
       </c>
       <c r="Q55" s="2" t="inlineStr"/>
@@ -6791,7 +6791,7 @@
         </is>
       </c>
       <c r="U55" s="5" t="n">
-        <v>0.72</v>
+        <v>0.82</v>
       </c>
       <c r="V55" s="2" t="inlineStr"/>
       <c r="W55" s="2" t="inlineStr">
@@ -6802,7 +6802,7 @@
       <c r="X55" s="2" t="inlineStr"/>
       <c r="Y55" s="2" t="inlineStr">
         <is>
-          <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Rokiškio miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z55" s="2" t="inlineStr">
@@ -6814,49 +6814,49 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>silutes-betonas-silute</t>
+          <t>telsiu-keliai-telsiai</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>177392928</t>
+          <t>180200843</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>UAB Šilutės betonas</t>
+          <t>UAB Telšių keliai</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Šilutės betonas</t>
+          <t>Telšių keliai</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta EVRK 23.63</t>
+          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Šilutė</t>
+          <t>Telšiai</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Šilutės r. sav.</t>
+          <t>Telšių r. sav.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Ramučių g. 1, Šilutė</t>
+          <t>Mažeikių g. 18, Telšiai</t>
         </is>
       </c>
       <c r="I56" s="3" t="n">
-        <v>55.3538641</v>
+        <v>56.0004158</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>21.4796635</v>
+        <v>22.2581129</v>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
@@ -6885,102 +6885,108 @@
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>Šilutės betono gamyba</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q56" s="2" t="inlineStr"/>
       <c r="R56" s="2" t="inlineStr"/>
-      <c r="S56" s="4" t="inlineStr"/>
+      <c r="S56" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T56" s="2" t="inlineStr">
         <is>
-          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai.</t>
         </is>
       </c>
       <c r="U56" s="5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="V56" s="2" t="inlineStr"/>
+        <v>0.86</v>
+      </c>
+      <c r="V56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/</t>
+        </is>
+      </c>
       <c r="W56" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
         </is>
       </c>
       <c r="X56" s="2" t="inlineStr">
         <is>
-          <t>https://fsaskaita.lt/imone/uzdaroji-akcine-bendrove-silutes-betonas-177392928</t>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
         </is>
       </c>
       <c r="Y56" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
         </is>
       </c>
       <c r="Z56" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>kruszbet-lithuania-jure</t>
+          <t>vpa-laistai</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>305173596</t>
+          <t>110185819</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>UAB KRUSZBET Lithuania</t>
+          <t>UAB V. Paulius &amp; Associates</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>KRUSZBET Lithuania</t>
+          <t>VPA</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta EVRK 23.63</t>
+          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Jūrė</t>
+          <t>Laistai</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Kazlų Rūdos sav.</t>
+          <t>Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Medelyno g. 30A, Jūrė, Kazlų Rūdos sav.</t>
+          <t>Stariškės g. 9, Laistų k., Dovilų sen., Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="I57" s="3" t="n">
-        <v>54.7706307</v>
+        <v>55.636908</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>23.4998409</v>
+        <v>21.209254</v>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Naudotojo pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>Google Maps nuoroda</t>
         </is>
       </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
         </is>
       </c>
       <c r="N57" s="2" t="inlineStr">
@@ -6995,98 +7001,116 @@
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
-          <t>KRUSZBET Lithuania betono gamyba</t>
-        </is>
-      </c>
-      <c r="Q57" s="2" t="inlineStr"/>
-      <c r="R57" s="2" t="inlineStr"/>
-      <c r="S57" s="4" t="inlineStr"/>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="Q57" s="2" t="inlineStr">
+        <is>
+          <t>3 m³</t>
+        </is>
+      </c>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t>60-80 m³/h</t>
+        </is>
+      </c>
+      <c r="S57" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T57" s="2" t="inlineStr">
         <is>
-          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+          <t>VPA betono mazgas Klaipėdos rajone.</t>
         </is>
       </c>
       <c r="U57" s="5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="V57" s="2" t="inlineStr"/>
+        <v>0.7</v>
+      </c>
+      <c r="V57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vpa.lt/</t>
+        </is>
+      </c>
       <c r="W57" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X57" s="2" t="inlineStr"/>
+          <t>https://www.vpa.lt/?Kontaktai=</t>
+        </is>
+      </c>
+      <c r="X57" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+        </is>
+      </c>
       <c r="Y57" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Vieta nustatyta pagal naudotojo pateiktą Google Maps nuorodą. VPA kontaktų puslapis nurodo Stariškės g. 9, Laistų k. adresą. Techniniai mazgo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z57" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>telsiu-keliai-telsiai</t>
+          <t>c3-beton-baisogala</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>180200843</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>UAB Telšių keliai</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Telšių keliai</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
+          <t>Konkurentas</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Telšiai</t>
+          <t>Baisogala</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Telšių r. sav.</t>
+          <t>Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Mažeikių g. 18, Telšiai</t>
+          <t>Dvaro g., Baisogala, Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="I58" s="3" t="n">
-        <v>56.0004158</v>
+        <v>55.6372</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>22.2581129</v>
+        <v>23.7183</v>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>C3 Betonas oficialus puslapis</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
@@ -7101,108 +7125,118 @@
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>Elkon</t>
-        </is>
-      </c>
-      <c r="Q58" s="2" t="inlineStr"/>
-      <c r="R58" s="2" t="inlineStr"/>
-      <c r="S58" s="4" t="n">
-        <v>2</v>
+          <t>Baisiogala Plant</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="S58" s="4" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
       </c>
       <c r="T58" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai.</t>
+          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
         </is>
       </c>
       <c r="U58" s="5" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="V58" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/</t>
+          <t>https://c3beton.com/</t>
         </is>
       </c>
       <c r="W58" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="X58" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="Y58" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
         </is>
       </c>
       <c r="Z58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>vpa-laistai</t>
+          <t>c3-beton-martiniskis</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>110185819</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>UAB V. Paulius &amp; Associates</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>VPA</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
+          <t>Konkurentas</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Laistai</t>
+          <t>Martiniškis</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Klaipėdos r. sav.</t>
+          <t>Jonavos r. sav.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Stariškės g. 9, Laistų k., Dovilų sen., Klaipėdos r. sav.</t>
+          <t>Vanagiškiai, Kulvos sen., Jonavos r. sav.</t>
         </is>
       </c>
       <c r="I59" s="3" t="n">
-        <v>55.636908</v>
+        <v>55.1441659</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>21.209254</v>
+        <v>24.1869636</v>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Naudotojo pateiktos Google Maps nuorodos taškas</t>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>Google Maps nuoroda</t>
+          <t>C3 Betonas oficialus puslapis</t>
         </is>
       </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="N59" s="2" t="inlineStr">
@@ -7217,60 +7251,62 @@
       </c>
       <c r="P59" s="2" t="inlineStr">
         <is>
-          <t>Liebherr</t>
+          <t>Martiniškis Plant</t>
         </is>
       </c>
       <c r="Q59" s="2" t="inlineStr">
         <is>
-          <t>3 m³</t>
+          <t>Ammann Elba Euromix C120, 3 m³</t>
         </is>
       </c>
       <c r="R59" s="2" t="inlineStr">
         <is>
-          <t>60-80 m³/h</t>
-        </is>
-      </c>
-      <c r="S59" s="4" t="n">
-        <v>2</v>
+          <t>60–80 m³/val.</t>
+        </is>
+      </c>
+      <c r="S59" s="4" t="inlineStr">
+        <is>
+          <t>2x85 t</t>
+        </is>
       </c>
       <c r="T59" s="2" t="inlineStr">
         <is>
-          <t>VPA betono mazgas Klaipėdos rajone.</t>
+          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U59" s="5" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="V59" s="2" t="inlineStr">
         <is>
-          <t>https://www.vpa.lt/</t>
+          <t>https://c3beton.com/</t>
         </is>
       </c>
       <c r="W59" s="2" t="inlineStr">
         <is>
-          <t>https://www.vpa.lt/?Kontaktai=</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="X59" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="Y59" s="2" t="inlineStr">
         <is>
-          <t>Vieta nustatyta pagal naudotojo pateiktą Google Maps nuorodą. VPA kontaktų puslapis nurodo Stariškės g. 9, Laistų k. adresą. Techniniai mazgo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z59" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-baisogala</t>
+          <t>c3-beton-stasenai</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -7295,38 +7331,38 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Baisogala</t>
+          <t>Vilnius</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Radviliškio r. sav.</t>
+          <t>Vilniaus m. sav.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Dvaro g., Baisogala, Radviliškio r. sav.</t>
+          <t>Ušos g. 21, Vilnius, 02121 Vilniaus m. sav.</t>
         </is>
       </c>
       <c r="I60" s="3" t="n">
-        <v>55.6372</v>
+        <v>54.6493094</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>23.7183</v>
+        <v>25.3107972</v>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
+          <t>Tikslus adreso taškas pagal geokodavimą</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas oficialus puslapis</t>
+          <t>ArcGIS geokodavimas pagal naudotojo pateiktą adresą</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://geocode.arcgis.com/arcgis/rest/services/World/GeocodeServer/findAddressCandidates</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
@@ -7341,27 +7377,27 @@
       </c>
       <c r="P60" s="2" t="inlineStr">
         <is>
-          <t>Baisiogala Plant</t>
+          <t>Vilnius Ušos g. Plant</t>
         </is>
       </c>
       <c r="Q60" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>Nissbau Euromix C120, 3 m³</t>
         </is>
       </c>
       <c r="R60" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>60–80 m³/val.</t>
         </is>
       </c>
       <c r="S60" s="4" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>2x85 t</t>
         </is>
       </c>
       <c r="T60" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
+          <t>Betono mazgas Nissbau Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U60" s="5" t="n">
@@ -7384,7 +7420,7 @@
       </c>
       <c r="Y60" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
+          <t>Perkelta iš Stašėnų lokacijos į Ušos g. 21, Vilnius pagal naudotojo pateiktą informaciją. Maišyklė pervadinta į Nissbau Euromix C120, 3 m³. Koordinatės geokoduotos pagal naują adresą.</t>
         </is>
       </c>
       <c r="Z60" s="2" t="inlineStr">
@@ -7396,7 +7432,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-martiniskis</t>
+          <t>c3-beton-runeikiai</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -7421,24 +7457,24 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Martiniškis</t>
+          <t>Runeikiai</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Jonavos r. sav.</t>
+          <t>Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Vanagiškiai, Kulvos sen., Jonavos r. sav.</t>
+          <t>Paguiriai, Šėtos sen., Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="I61" s="3" t="n">
-        <v>55.1441659</v>
+        <v>55.3327393</v>
       </c>
       <c r="J61" s="3" t="n">
-        <v>24.1869636</v>
+        <v>24.3501308</v>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
@@ -7467,7 +7503,7 @@
       </c>
       <c r="P61" s="2" t="inlineStr">
         <is>
-          <t>Martiniškis Plant</t>
+          <t>Runeikiai Plant</t>
         </is>
       </c>
       <c r="Q61" s="2" t="inlineStr">
@@ -7522,22 +7558,22 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-stasenai</t>
+          <t>reljef-rukla</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>301731961</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas</t>
+          <t>UAB Reljef</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas</t>
+          <t>Reljef</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -7547,38 +7583,38 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Vilnius</t>
+          <t>Rukla</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus m. sav.</t>
+          <t>Jonavos r. sav.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Ušos g. 21, Vilnius, 02121 Vilniaus m. sav.</t>
+          <t>Rukla, Jonavos r. sav.</t>
         </is>
       </c>
       <c r="I62" s="3" t="n">
-        <v>54.6493094</v>
+        <v>55.05225</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>25.3107972</v>
+        <v>24.4064167</v>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas pagal geokodavimą</t>
+          <t>Tikslus naudotojo pateiktas taškas; adresas artimiausias pagal OpenStreetMap</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>ArcGIS geokodavimas pagal naudotojo pateiktą adresą</t>
+          <t>Naudotojo pateiktos koordinatės</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>https://geocode.arcgis.com/arcgis/rest/services/World/GeocodeServer/findAddressCandidates</t>
+          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
         </is>
       </c>
       <c r="N62" s="2" t="inlineStr">
@@ -7593,203 +7629,203 @@
       </c>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t>Vilnius Ušos g. Plant</t>
+          <t>Ammann Elba</t>
         </is>
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>Nissbau Euromix C120, 3 m³</t>
+          <t>Nenustatyta</t>
         </is>
       </c>
       <c r="R62" s="2" t="inlineStr">
         <is>
-          <t>60–80 m³/val.</t>
+          <t>Nenustatytas</t>
         </is>
       </c>
       <c r="S62" s="4" t="inlineStr">
         <is>
-          <t>2x85 t</t>
+          <t>2x65 t</t>
         </is>
       </c>
       <c r="T62" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgas Nissbau Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
+          <t>Rukloje veikiantis UAB Reljef betono mazgas: Ammann Elba, 2x65 t silosai. Maišyklė ir našumas nenustatyti.</t>
         </is>
       </c>
       <c r="U62" s="5" t="n">
-        <v>0.9</v>
+        <v>0.82</v>
       </c>
       <c r="V62" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/</t>
+          <t>https://www.reljef.lt/</t>
         </is>
       </c>
       <c r="W62" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.reljef.lt/</t>
         </is>
       </c>
       <c r="X62" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
         </is>
       </c>
       <c r="Y62" s="2" t="inlineStr">
         <is>
-          <t>Perkelta iš Stašėnų lokacijos į Ušos g. 21, Vilnius pagal naudotojo pateiktą informaciją. Maišyklė pervadinta į Nissbau Euromix C120, 3 m³. Koordinatės geokoduotos pagal naują adresą.</t>
+          <t>Įmonės rekvizitai paimti iš oficialaus UAB Reljef puslapio. Betono mazgo gamintojas, silosai ir lokacija įrašyti pagal naudotojo pateiktą informaciją. Artimiausias viešai geokoduotas adresas nustatytas pagal OpenStreetMap.</t>
         </is>
       </c>
       <c r="Z62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-runeikiai</t>
+          <t>ponas-betonas-paraudondvariai</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
+          <t>306676006</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>UAB Ponas betonas</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Ponas betonas</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Konkurentas</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Paraudondvariai</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Vilniaus r. sav.</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Vilniaus g., Paraudondvariai, Riešės sen., Vilniaus r. sav.</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="n">
+        <v>54.8321418</v>
+      </c>
+      <c r="J63" s="3" t="n">
+        <v>25.2755596</v>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>Naudotojo pateikta Google Maps lokacija</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/NxQohpnzv1q9DA6CA?g_st=ac</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr">
+        <is>
+          <t>Elkon</t>
+        </is>
+      </c>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
           <t>Nenurodyta viešai</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>C3 Betonas</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>C3 Betonas</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>Konkurentas</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>Runeikiai</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="inlineStr">
-        <is>
-          <t>Kėdainių r. sav.</t>
-        </is>
-      </c>
-      <c r="H63" s="2" t="inlineStr">
-        <is>
-          <t>Paguiriai, Šėtos sen., Kėdainių r. sav.</t>
-        </is>
-      </c>
-      <c r="I63" s="3" t="n">
-        <v>55.3327393</v>
-      </c>
-      <c r="J63" s="3" t="n">
-        <v>24.3501308</v>
-      </c>
-      <c r="K63" s="2" t="inlineStr">
-        <is>
-          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
-        </is>
-      </c>
-      <c r="L63" s="2" t="inlineStr">
-        <is>
-          <t>C3 Betonas oficialus puslapis</t>
-        </is>
-      </c>
-      <c r="M63" s="2" t="inlineStr">
-        <is>
-          <t>https://c3beton.com/lt/betonas</t>
-        </is>
-      </c>
-      <c r="N63" s="2" t="inlineStr">
-        <is>
-          <t>ready_mix_concrete</t>
-        </is>
-      </c>
-      <c r="O63" s="2" t="inlineStr">
-        <is>
-          <t>Betono mišiniai</t>
-        </is>
-      </c>
-      <c r="P63" s="2" t="inlineStr">
-        <is>
-          <t>Runeikiai Plant</t>
-        </is>
-      </c>
-      <c r="Q63" s="2" t="inlineStr">
-        <is>
-          <t>Ammann Elba Euromix C120, 3 m³</t>
-        </is>
-      </c>
       <c r="R63" s="2" t="inlineStr">
         <is>
-          <t>60–80 m³/val.</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="S63" s="4" t="inlineStr">
         <is>
-          <t>2x85 t</t>
+          <t>2 matomi oficialioje nuotraukoje</t>
         </is>
       </c>
       <c r="T63" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
+          <t>Oficialiame UAB Ponas betonas puslapyje nurodoma, kad įmonė turi nuosavą betono mazgą, gamina prekinį betoną ir jį pristato. Puslapio hero nuotraukoje ant silosų matomas ELKON ženklinimas, todėl mazgo gamintojas identifikuotas kaip Elkon. Konkretus modelis, maišyklė ir našumas viešai nenurodyti; oficialioje nuotraukoje matomi 2 silosai.</t>
         </is>
       </c>
       <c r="U63" s="5" t="n">
-        <v>0.9</v>
+        <v>0.98</v>
       </c>
       <c r="V63" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/</t>
+          <t>https://www.ponasbetonas.lt/</t>
         </is>
       </c>
       <c r="W63" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.ponasbetonas.lt/#Apiemus</t>
         </is>
       </c>
       <c r="X63" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.ponasbetonas.lt/</t>
         </is>
       </c>
       <c r="Y63" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Nuosavas betono mazgas ir prekinio betono gamyba patvirtinti oficialiame įmonės puslapyje. Mazgo gamintojas nustatytas pagal oficialaus puslapio hero nuotraukoje ant silosų matomą ELKON ženklinimą; modelis, maišyklė ir našumas viešai nenurodyti. Tiksli mazgo lokacija paimta iš naudotojo pateiktos Google Maps nuorodos; vietovė patikslinta pagal OpenStreetMap. Įmonės kodas patvirtintas Registrų centro viešame juridinio asmens pranešime.</t>
         </is>
       </c>
       <c r="Z63" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>reljef-rukla</t>
+          <t>pabrades-betonas-pabrade</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>301731961</t>
+          <t>306177188</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>UAB Reljef</t>
+          <t>UAB Pabradės betonas</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Reljef</t>
+          <t>Pabradės betonas</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -7799,38 +7835,38 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Rukla</t>
+          <t>Pabradė</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Jonavos r. sav.</t>
+          <t>Švenčionių r. sav.</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Rukla, Jonavos r. sav.</t>
+          <t>Vilniaus g. 161, Pabradė, LT-18177 Švenčionių r.</t>
         </is>
       </c>
       <c r="I64" s="3" t="n">
-        <v>55.05225</v>
+        <v>54.9758768</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>24.4064167</v>
+        <v>25.7373849</v>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Tikslus naudotojo pateiktas taškas; adresas artimiausias pagal OpenStreetMap</t>
+          <t>Tikslus oficialioje svetainėje pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>Naudotojo pateiktos koordinatės</t>
+          <t>Oficiali Pabradės betono Google Maps nuoroda</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
+          <t>https://maps.app.goo.gl/TQBCVR8DczDRvQaeA</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
@@ -7845,77 +7881,77 @@
       </c>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>Ammann Elba</t>
+          <t>Liebherr (tikėtina)</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>Nenustatyta</t>
+          <t>3 m³</t>
         </is>
       </c>
       <c r="R64" s="2" t="inlineStr">
         <is>
-          <t>Nenustatytas</t>
+          <t>60 m³/val.</t>
         </is>
       </c>
       <c r="S64" s="4" t="inlineStr">
         <is>
-          <t>2x65 t</t>
+          <t>3x65 t</t>
         </is>
       </c>
       <c r="T64" s="2" t="inlineStr">
         <is>
-          <t>Rukloje veikiantis UAB Reljef betono mazgas: Ammann Elba, 2x65 t silosai. Maišyklė ir našumas nenustatyti.</t>
+          <t>UAB Pabradės betonas Vilniaus g. 161, Pabradėje, gamina sertifikuotą normalųjį betoną ir oficialiai nurodo dirbanti 50 km spinduliu aplink Pabradę. Oficialios galerijos nuotraukose matoma stacionari gamybos bazė su trimis cemento silosais. Mazgo gamintojas tikėtinai Liebherr pagal oficialiose nuotraukose matomą Liebherr įrangą ir gamyklos konstrukcijos vizualinius požymius; gamintojo lentelė viešai neparodyta.</t>
         </is>
       </c>
       <c r="U64" s="5" t="n">
-        <v>0.82</v>
+        <v>0.72</v>
       </c>
       <c r="V64" s="2" t="inlineStr">
         <is>
-          <t>https://www.reljef.lt/</t>
+          <t>https://www.pabradesbetonas.lt/</t>
         </is>
       </c>
       <c r="W64" s="2" t="inlineStr">
         <is>
-          <t>https://www.reljef.lt/</t>
+          <t>https://www.pabradesbetonas.lt/</t>
         </is>
       </c>
       <c r="X64" s="2" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
+          <t>https://www.pabradesbetonas.lt/galerija/</t>
         </is>
       </c>
       <c r="Y64" s="2" t="inlineStr">
         <is>
-          <t>Įmonės rekvizitai paimti iš oficialaus UAB Reljef puslapio. Betono mazgo gamintojas, silosai ir lokacija įrašyti pagal naudotojo pateiktą informaciją. Artimiausias viešai geokoduotas adresas nustatytas pagal OpenStreetMap.</t>
+          <t>Adresas, įmonės kodas ir betono gamyba patvirtinti oficialioje svetainėje bei viešame gamybos kontrolės sertifikate. Koordinatės paimtos iš oficialioje svetainėje pateiktos Google Maps nuorodos. Maišyklės tūris 3 m³, realus našumas 60 m³/val. ir silosai 3x65 t įrašyti pagal naudotojo pateiktą informaciją. Gamintojas Liebherr nurodytas kaip tikėtinas pagal oficialios galerijos nuotraukas; viešo gamintojo ženklinimo ant paties mazgo nerasta.</t>
         </is>
       </c>
       <c r="Z64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>ponas-betonas-paraudondvariai</t>
+          <t>alkesta-marijampole-vasaros</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>306676006</t>
+          <t>249672710</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>UAB Ponas betonas</t>
+          <t>UAB Alkesta</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Ponas betonas</t>
+          <t>Alkesta</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -7925,24 +7961,24 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Paraudondvariai</t>
+          <t>Marijampolė</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus r. sav.</t>
+          <t>Marijampolės sav.</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus g., Paraudondvariai, Riešės sen., Vilniaus r. sav.</t>
+          <t>Vasaros g. 14, Marijampolė, LT-68111</t>
         </is>
       </c>
       <c r="I65" s="3" t="n">
-        <v>54.8321418</v>
+        <v>54.5686121</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>25.2755596</v>
+        <v>23.3895157</v>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
@@ -7956,7 +7992,7 @@
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/NxQohpnzv1q9DA6CA?g_st=ac</t>
+          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
@@ -7971,77 +8007,73 @@
       </c>
       <c r="P65" s="2" t="inlineStr">
         <is>
-          <t>Elkon</t>
+          <t>Elba</t>
         </is>
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>0,5 m³</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
-        </is>
-      </c>
-      <c r="S65" s="4" t="inlineStr">
-        <is>
-          <t>2 matomi oficialioje nuotraukoje</t>
-        </is>
-      </c>
+          <t>10 m³/val.</t>
+        </is>
+      </c>
+      <c r="S65" s="4" t="inlineStr"/>
       <c r="T65" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame UAB Ponas betonas puslapyje nurodoma, kad įmonė turi nuosavą betono mazgą, gamina prekinį betoną ir jį pristato. Puslapio hero nuotraukoje ant silosų matomas ELKON ženklinimas, todėl mazgo gamintojas identifikuotas kaip Elkon. Konkretus modelis, maišyklė ir našumas viešai nenurodyti; oficialioje nuotraukoje matomi 2 silosai.</t>
+          <t>UAB Alkesta Marijampolės betono mazgas Vasaros g. 14. Mazgo gamintojas Elba, maišyklė 0,5 m³, našumas 10 m³/val.</t>
         </is>
       </c>
       <c r="U65" s="5" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="V65" s="2" t="inlineStr">
         <is>
-          <t>https://www.ponasbetonas.lt/</t>
+          <t>https://alkesta.lt/</t>
         </is>
       </c>
       <c r="W65" s="2" t="inlineStr">
         <is>
-          <t>https://www.ponasbetonas.lt/#Apiemus</t>
+          <t>https://spsc.lt/registrai/regsapp/ser_produktai_view.php?editid1=13061</t>
         </is>
       </c>
       <c r="X65" s="2" t="inlineStr">
         <is>
-          <t>https://www.ponasbetonas.lt/</t>
+          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
         </is>
       </c>
       <c r="Y65" s="2" t="inlineStr">
         <is>
-          <t>Nuosavas betono mazgas ir prekinio betono gamyba patvirtinti oficialiame įmonės puslapyje. Mazgo gamintojas nustatytas pagal oficialaus puslapio hero nuotraukoje ant silosų matomą ELKON ženklinimą; modelis, maišyklė ir našumas viešai nenurodyti. Tiksli mazgo lokacija paimta iš naudotojo pateiktos Google Maps nuorodos; vietovė patikslinta pagal OpenStreetMap. Įmonės kodas patvirtintas Registrų centro viešame juridinio asmens pranešime.</t>
+          <t>Oficialus SPSC sertifikatų registras patvirtina UAB Alkesta betono gamybą ir gamybos vietą Vasaros g. 14, Marijampolėje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris ir našumas įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>pabrades-betonas-pabrade</t>
+          <t>gevalda-visincia</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>306177188</t>
+          <t>302592895</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>UAB Pabradės betonas</t>
+          <t>UAB Gevalda</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Pabradės betonas</t>
+          <t>Gevalda</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -8051,38 +8083,38 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Pabradė</t>
+          <t>Visinčia</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Švenčionių r. sav.</t>
+          <t>Šalčininkų r. sav.</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus g. 161, Pabradė, LT-18177 Švenčionių r.</t>
+          <t>Visinčia, Pabarės sen., Šalčininkų r. sav.</t>
         </is>
       </c>
       <c r="I66" s="3" t="n">
-        <v>54.9758768</v>
+        <v>54.4122467</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>25.7373849</v>
+        <v>25.1449142</v>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>Tikslus oficialioje svetainėje pateiktos Google Maps nuorodos taškas</t>
+          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>Oficiali Pabradės betono Google Maps nuoroda</t>
+          <t>Naudotojo pateikta Google Maps lokacija</t>
         </is>
       </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/TQBCVR8DczDRvQaeA</t>
+          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
         </is>
       </c>
       <c r="N66" s="2" t="inlineStr">
@@ -8097,7 +8129,7 @@
       </c>
       <c r="P66" s="2" t="inlineStr">
         <is>
-          <t>Liebherr (tikėtina)</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q66" s="2" t="inlineStr">
@@ -8112,35 +8144,35 @@
       </c>
       <c r="S66" s="4" t="inlineStr">
         <is>
-          <t>3x65 t</t>
+          <t>2x85 t</t>
         </is>
       </c>
       <c r="T66" s="2" t="inlineStr">
         <is>
-          <t>UAB Pabradės betonas Vilniaus g. 161, Pabradėje, gamina sertifikuotą normalųjį betoną ir oficialiai nurodo dirbanti 50 km spinduliu aplink Pabradę. Oficialios galerijos nuotraukose matoma stacionari gamybos bazė su trimis cemento silosais. Mazgo gamintojas tikėtinai Liebherr pagal oficialiose nuotraukose matomą Liebherr įrangą ir gamyklos konstrukcijos vizualinius požymius; gamintojo lentelė viešai neparodyta.</t>
+          <t>UAB Gevalda mobilus betono mazgas Visinčioje. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U66" s="5" t="n">
-        <v>0.72</v>
+        <v>0.95</v>
       </c>
       <c r="V66" s="2" t="inlineStr">
         <is>
-          <t>https://www.pabradesbetonas.lt/</t>
+          <t>https://www.gevalda.lt/</t>
         </is>
       </c>
       <c r="W66" s="2" t="inlineStr">
         <is>
-          <t>https://www.pabradesbetonas.lt/</t>
+          <t>https://www.gevalda.lt/paslaugos/gamyba</t>
         </is>
       </c>
       <c r="X66" s="2" t="inlineStr">
         <is>
-          <t>https://www.pabradesbetonas.lt/galerija/</t>
+          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
         </is>
       </c>
       <c r="Y66" s="2" t="inlineStr">
         <is>
-          <t>Adresas, įmonės kodas ir betono gamyba patvirtinti oficialioje svetainėje bei viešame gamybos kontrolės sertifikate. Koordinatės paimtos iš oficialioje svetainėje pateiktos Google Maps nuorodos. Maišyklės tūris 3 m³, realus našumas 60 m³/val. ir silosai 3x65 t įrašyti pagal naudotojo pateiktą informaciją. Gamintojas Liebherr nurodytas kaip tikėtinas pagal oficialios galerijos nuotraukas; viešo gamintojo ženklinimo ant paties mazgo nerasta.</t>
+          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris, našumas ir silosai įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z66" s="2" t="inlineStr">
@@ -8152,22 +8184,22 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>alkesta-marijampole-vasaros</t>
+          <t>gevalda-kaunas-palemonas</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>249672710</t>
+          <t>302592895</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>UAB Alkesta</t>
+          <t>UAB Gevalda</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>Alkesta</t>
+          <t>Gevalda</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -8177,24 +8209,24 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Marijampolė</t>
+          <t>Kaunas</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Marijampolės sav.</t>
+          <t>Kauno m. sav.</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>Vasaros g. 14, Marijampolė, LT-68111</t>
+          <t>Kražantės g., Palemonas, Kaunas</t>
         </is>
       </c>
       <c r="I67" s="3" t="n">
-        <v>54.5686121</v>
+        <v>54.918</v>
       </c>
       <c r="J67" s="3" t="n">
-        <v>23.3895157</v>
+        <v>24.063</v>
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
@@ -8208,7 +8240,7 @@
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
+          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
         </is>
       </c>
       <c r="N67" s="2" t="inlineStr">
@@ -8223,23 +8255,27 @@
       </c>
       <c r="P67" s="2" t="inlineStr">
         <is>
-          <t>Elba</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q67" s="2" t="inlineStr">
         <is>
-          <t>0,5 m³</t>
+          <t>3 m³</t>
         </is>
       </c>
       <c r="R67" s="2" t="inlineStr">
         <is>
-          <t>10 m³/val.</t>
-        </is>
-      </c>
-      <c r="S67" s="4" t="inlineStr"/>
+          <t>60 m³/val.</t>
+        </is>
+      </c>
+      <c r="S67" s="4" t="inlineStr">
+        <is>
+          <t>2x85 t</t>
+        </is>
+      </c>
       <c r="T67" s="2" t="inlineStr">
         <is>
-          <t>UAB Alkesta Marijampolės betono mazgas Vasaros g. 14. Mazgo gamintojas Elba, maišyklė 0,5 m³, našumas 10 m³/val.</t>
+          <t>UAB Gevalda mobilus betono mazgas Palemone, Kaune. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U67" s="5" t="n">
@@ -8247,284 +8283,32 @@
       </c>
       <c r="V67" s="2" t="inlineStr">
         <is>
-          <t>https://alkesta.lt/</t>
+          <t>https://www.gevalda.lt/</t>
         </is>
       </c>
       <c r="W67" s="2" t="inlineStr">
         <is>
-          <t>https://spsc.lt/registrai/regsapp/ser_produktai_view.php?editid1=13061</t>
+          <t>https://www.gevalda.lt/paslaugos/gamyba</t>
         </is>
       </c>
       <c r="X67" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
+          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
         </is>
       </c>
       <c r="Y67" s="2" t="inlineStr">
         <is>
-          <t>Oficialus SPSC sertifikatų registras patvirtina UAB Alkesta betono gamybą ir gamybos vietą Vasaros g. 14, Marijampolėje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris ir našumas įrašyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija ir analogiški techniniai duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z67" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>gevalda-visincia</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>302592895</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>UAB Gevalda</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>Gevalda</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>Konkurentas</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>Visinčia</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>Šalčininkų r. sav.</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>Visinčia, Pabarės sen., Šalčininkų r. sav.</t>
-        </is>
-      </c>
-      <c r="I68" s="3" t="n">
-        <v>54.4122467</v>
-      </c>
-      <c r="J68" s="3" t="n">
-        <v>25.1449142</v>
-      </c>
-      <c r="K68" s="2" t="inlineStr">
-        <is>
-          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
-        </is>
-      </c>
-      <c r="L68" s="2" t="inlineStr">
-        <is>
-          <t>Naudotojo pateikta Google Maps lokacija</t>
-        </is>
-      </c>
-      <c r="M68" s="2" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
-        </is>
-      </c>
-      <c r="N68" s="2" t="inlineStr">
-        <is>
-          <t>ready_mix_concrete</t>
-        </is>
-      </c>
-      <c r="O68" s="2" t="inlineStr">
-        <is>
-          <t>Betono mišiniai</t>
-        </is>
-      </c>
-      <c r="P68" s="2" t="inlineStr">
-        <is>
-          <t>Elkon</t>
-        </is>
-      </c>
-      <c r="Q68" s="2" t="inlineStr">
-        <is>
-          <t>3 m³</t>
-        </is>
-      </c>
-      <c r="R68" s="2" t="inlineStr">
-        <is>
-          <t>60 m³/val.</t>
-        </is>
-      </c>
-      <c r="S68" s="4" t="inlineStr">
-        <is>
-          <t>2x85 t</t>
-        </is>
-      </c>
-      <c r="T68" s="2" t="inlineStr">
-        <is>
-          <t>UAB Gevalda mobilus betono mazgas Visinčioje. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
-        </is>
-      </c>
-      <c r="U68" s="5" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="V68" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gevalda.lt/</t>
-        </is>
-      </c>
-      <c r="W68" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gevalda.lt/paslaugos/gamyba</t>
-        </is>
-      </c>
-      <c r="X68" s="2" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
-        </is>
-      </c>
-      <c r="Y68" s="2" t="inlineStr">
-        <is>
-          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris, našumas ir silosai įrašyti pagal naudotojo pateiktą informaciją.</t>
-        </is>
-      </c>
-      <c r="Z68" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>gevalda-kaunas-palemonas</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>302592895</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>UAB Gevalda</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>Gevalda</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>Konkurentas</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>Kaunas</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="inlineStr">
-        <is>
-          <t>Kauno m. sav.</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>Kražantės g., Palemonas, Kaunas</t>
-        </is>
-      </c>
-      <c r="I69" s="3" t="n">
-        <v>54.918</v>
-      </c>
-      <c r="J69" s="3" t="n">
-        <v>24.063</v>
-      </c>
-      <c r="K69" s="2" t="inlineStr">
-        <is>
-          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
-        </is>
-      </c>
-      <c r="L69" s="2" t="inlineStr">
-        <is>
-          <t>Naudotojo pateikta Google Maps lokacija</t>
-        </is>
-      </c>
-      <c r="M69" s="2" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
-        </is>
-      </c>
-      <c r="N69" s="2" t="inlineStr">
-        <is>
-          <t>ready_mix_concrete</t>
-        </is>
-      </c>
-      <c r="O69" s="2" t="inlineStr">
-        <is>
-          <t>Betono mišiniai</t>
-        </is>
-      </c>
-      <c r="P69" s="2" t="inlineStr">
-        <is>
-          <t>Elkon</t>
-        </is>
-      </c>
-      <c r="Q69" s="2" t="inlineStr">
-        <is>
-          <t>3 m³</t>
-        </is>
-      </c>
-      <c r="R69" s="2" t="inlineStr">
-        <is>
-          <t>60 m³/val.</t>
-        </is>
-      </c>
-      <c r="S69" s="4" t="inlineStr">
-        <is>
-          <t>2x85 t</t>
-        </is>
-      </c>
-      <c r="T69" s="2" t="inlineStr">
-        <is>
-          <t>UAB Gevalda mobilus betono mazgas Palemone, Kaune. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
-        </is>
-      </c>
-      <c r="U69" s="5" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="V69" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gevalda.lt/</t>
-        </is>
-      </c>
-      <c r="W69" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gevalda.lt/paslaugos/gamyba</t>
-        </is>
-      </c>
-      <c r="X69" s="2" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
-        </is>
-      </c>
-      <c r="Y69" s="2" t="inlineStr">
-        <is>
-          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija ir analogiški techniniai duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
-        </is>
-      </c>
-      <c r="Z69" s="2" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z69"/>
+  <autoFilter ref="A1:Z67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8613,7 +8397,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-24T04:22:17.382218+00:00</t>
+          <t>2026-09-24T04:42:42.583222+00:00</t>
         </is>
       </c>
     </row>
@@ -8668,7 +8452,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-24T04:22:17.383221+00:00</t>
+          <t>2026-09-24T04:42:42.583222+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8682,7 +8466,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atnaujinti Betonika Senuju Traku gamyklos duomenis
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -3472,18 +3472,22 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>inhus-senieji-trakai</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr"/>
+          <t>betonika-senieji-trakai</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>135551936</t>
+        </is>
+      </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>UAB INHUS Lietuva</t>
+          <t>Betonika UAB</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>INHUS</t>
+          <t>Betonika</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -3503,7 +3507,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Plačioji g. 27, Senieji Trakai</t>
+          <t>Plačioji g. 27, Senųjų Trakų km., LT-21146</t>
         </is>
       </c>
       <c r="I26" s="3" t="n">
@@ -3539,7 +3543,7 @@
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>INHUS gelžbetonio gamykla</t>
+          <t>Betonika Trakų gelžbetonio gamykla</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr"/>
@@ -3547,31 +3551,35 @@
       <c r="S26" s="4" t="inlineStr"/>
       <c r="T26" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiamas surenkamojo gelžbetonio konstrukcijų gamintojas.</t>
+          <t>Surenkamojo gelžbetonio gamykla. Gaminamos perdangos plokštės, kolonos, sijos, sienų elementai, laiptų ir stogo plokštės; įmonė nurodo, kad prekinio betono neparduoda.</t>
         </is>
       </c>
       <c r="U26" s="5" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="V26" s="2" t="inlineStr">
         <is>
-          <t>https://inhus.eu/</t>
+          <t>https://betonika.lt/</t>
         </is>
       </c>
       <c r="W26" s="2" t="inlineStr">
         <is>
-          <t>https://inhus.eu/</t>
+          <t>https://betonika.lt/kontaktai/</t>
         </is>
       </c>
       <c r="X26" s="2" t="inlineStr">
         <is>
-          <t>https://inhus.eu/</t>
-        </is>
-      </c>
-      <c r="Y26" s="2" t="inlineStr"/>
+          <t>https://betonika.lt/apie-mus/</t>
+        </is>
+      </c>
+      <c r="Y26" s="2" t="inlineStr">
+        <is>
+          <t>Oficialiame kontaktų puslapyje ši vieta įvardyta kaip Trakų gamykla; nurodyta „BETONO NEPARDUODAME“.</t>
+        </is>
+      </c>
       <c r="Z26" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-09-25</t>
         </is>
       </c>
     </row>
@@ -8397,7 +8405,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-24T04:42:42.583222+00:00</t>
+          <t>2026-09-25T06:01:50.565312+00:00</t>
         </is>
       </c>
     </row>
@@ -8452,7 +8460,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-24T04:42:42.583222+00:00</t>
+          <t>2026-09-25T06:01:50.565312+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Atnaujinti Klaipedos, Telsiu ir Vinido duomenis, pasalinti du taskus
</commit_message>
<xml_diff>
--- a/data/companies.xlsx
+++ b/data/companies.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Įmonės" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metaduomenys" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importo žurnalas" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Įmonės'!$A$1:$Z$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -169,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z67" headerRowCount="1">
-  <autoFilter ref="A1:Z67"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImonesTable" displayName="ImonesTable" ref="A1:Z66" headerRowCount="1">
+  <autoFilter ref="A1:Z66"/>
   <tableColumns count="26">
     <tableColumn id="1" name="Įrašo ID"/>
     <tableColumn id="2" name="Įmonės kodas"/>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z67"/>
+  <dimension ref="A1:Z66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
@@ -509,10 +509,10 @@
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="42" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="41" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
-    <col width="32" customWidth="1" min="17" max="17"/>
-    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="33" customWidth="1" min="17" max="17"/>
+    <col width="42" customWidth="1" min="18" max="18"/>
     <col width="34" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="29" customWidth="1" min="21" max="21"/>
@@ -1470,7 +1470,11 @@
           <t>60 m³/h</t>
         </is>
       </c>
-      <c r="S8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>4 vnt. (2×120 t, 2×60 t)</t>
+        </is>
+      </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
           <t>Viešai skelbiamas Betono centro betono mazgas Klaipėdoje.</t>
@@ -1496,12 +1500,12 @@
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame Betono centro kontaktų puslapyje patvirtintas Klaipėdos padalinys. Mazgo techniniai duomenys patikslinti pagal naudotojo pateiktą informaciją.</t>
+          <t>Oficialiame Betono centro kontaktų puslapyje patvirtintas Klaipėdos padalinys. Mazgo techniniai duomenys patikslinti pagal naudotojo pateiktą informaciją. Silosai: 4 vnt. (2×120 t, 2×60 t), pagal naudotojo 2026-10-14 pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -4952,18 +4956,22 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>betono-zona-klaipeda</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr"/>
+          <t>topbeton-panevezys</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>307083610</t>
+        </is>
+      </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>UAB Betono zona</t>
+          <t>UAB Topbeton</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Betono zona</t>
+          <t>Topbeton</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -4973,24 +4981,24 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Klaipėda</t>
+          <t>Panevėžys</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Klaipėdos m. sav.</t>
+          <t>Panevėžio m. sav.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Dvaro g. 6, Klaipėda</t>
+          <t>Beržų g. 5C, Panevėžys</t>
         </is>
       </c>
       <c r="I39" s="3" t="n">
-        <v>55.7549809</v>
+        <v>55.7168572</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>21.150509</v>
+        <v>24.3617863</v>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
@@ -5009,17 +5017,17 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>precast_concrete</t>
+          <t>ready_mix_concrete</t>
         </is>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>Betono gaminiai</t>
+          <t>Betono mišiniai</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>Betono zona</t>
+          <t>Topbeton betono mazgas</t>
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr"/>
@@ -5027,30 +5035,30 @@
       <c r="S39" s="4" t="inlineStr"/>
       <c r="T39" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono gaminių veikla Klaipėdoje.</t>
+          <t>Viešai skelbiama betono mišinių gamyba Panevėžyje.</t>
         </is>
       </c>
       <c r="U39" s="5" t="n">
-        <v>0.65</v>
+        <v>0.78</v>
       </c>
       <c r="V39" s="2" t="inlineStr">
         <is>
-          <t>https://betonozona.lt/</t>
+          <t>https://topbeton.lt/</t>
         </is>
       </c>
       <c r="W39" s="2" t="inlineStr">
         <is>
-          <t>https://betonozona.lt/</t>
+          <t>https://www.topbeton.lt/kontaktai/</t>
         </is>
       </c>
       <c r="X39" s="2" t="inlineStr">
         <is>
-          <t>https://betonozona.lt/</t>
+          <t>https://www.topbeton.lt/kontaktai/</t>
         </is>
       </c>
       <c r="Y39" s="2" t="inlineStr">
         <is>
-          <t>Patikrinti, ar įmonė pati gamina, ar tik prekiauja betono gaminiais.</t>
+          <t>Oficialus kontaktų puslapis patvirtina Beržų g. 5C adresą.</t>
         </is>
       </c>
       <c r="Z39" s="2" t="inlineStr">
@@ -5062,22 +5070,18 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>topbeton-panevezys</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>307083610</t>
-        </is>
-      </c>
+          <t>gelzbetonio-gamyba-panevezys</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>UAB Topbeton</t>
+          <t>MB Gelžbetonio gamyba</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Topbeton</t>
+          <t>Gelžbetonio gamyba</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -5097,14 +5101,14 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Beržų g. 5C, Panevėžys</t>
+          <t>S. Kerbedžio g. 52, Panevėžys</t>
         </is>
       </c>
       <c r="I40" s="3" t="n">
-        <v>55.7168572</v>
+        <v>55.7409491</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>24.3617863</v>
+        <v>24.3803541</v>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
@@ -5123,17 +5127,17 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>ready_mix_concrete</t>
+          <t>precast_concrete</t>
         </is>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>Betono mišiniai</t>
+          <t>Gelžbetonis</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>Topbeton betono mazgas</t>
+          <t>Gelžbetonio gamyba Panevėžyje</t>
         </is>
       </c>
       <c r="Q40" s="2" t="inlineStr"/>
@@ -5141,30 +5145,30 @@
       <c r="S40" s="4" t="inlineStr"/>
       <c r="T40" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono mišinių gamyba Panevėžyje.</t>
+          <t>Viešai skelbiama gelžbetonio gaminių gamyba Panevėžyje.</t>
         </is>
       </c>
       <c r="U40" s="5" t="n">
-        <v>0.78</v>
+        <v>0.72</v>
       </c>
       <c r="V40" s="2" t="inlineStr">
         <is>
-          <t>https://topbeton.lt/</t>
+          <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
       <c r="W40" s="2" t="inlineStr">
         <is>
-          <t>https://www.topbeton.lt/kontaktai/</t>
+          <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
       <c r="X40" s="2" t="inlineStr">
         <is>
-          <t>https://www.topbeton.lt/kontaktai/</t>
+          <t>https://gelzbetoniogamyba.lt/</t>
         </is>
       </c>
       <c r="Y40" s="2" t="inlineStr">
         <is>
-          <t>Oficialus kontaktų puslapis patvirtina Beržų g. 5C adresą.</t>
+          <t>Reikia patikslinti ryšį su kitomis S. Kerbedžio g. 52 įmonėmis.</t>
         </is>
       </c>
       <c r="Z40" s="2" t="inlineStr">
@@ -5176,18 +5180,18 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>gelzbetonio-gamyba-panevezys</t>
+          <t>inroma-pakruojis</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr"/>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>MB Gelžbetonio gamyba</t>
+          <t>UAB Inroma</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Gelžbetonio gamyba</t>
+          <t>Inroma</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -5197,24 +5201,24 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Panevėžys</t>
+          <t>Pakruojis</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Panevėžio m. sav.</t>
+          <t>Pakruojo r. sav.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>S. Kerbedžio g. 52, Panevėžys</t>
+          <t>Pramonės g. 5B, Pakruojis</t>
         </is>
       </c>
       <c r="I41" s="3" t="n">
-        <v>55.7409491</v>
+        <v>55.9763263</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>24.3803541</v>
+        <v>23.8584712</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
@@ -5233,17 +5237,17 @@
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>precast_concrete</t>
+          <t>ready_mix_concrete</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>Gelžbetonis</t>
+          <t>Betono mišiniai</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>Gelžbetonio gamyba Panevėžyje</t>
+          <t>Inroma betono mazgas</t>
         </is>
       </c>
       <c r="Q41" s="2" t="inlineStr"/>
@@ -5251,7 +5255,7 @@
       <c r="S41" s="4" t="inlineStr"/>
       <c r="T41" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama gelžbetonio gaminių gamyba Panevėžyje.</t>
+          <t>Viešai skelbiama betono mišinių veikla Pakruojyje.</t>
         </is>
       </c>
       <c r="U41" s="5" t="n">
@@ -5259,22 +5263,22 @@
       </c>
       <c r="V41" s="2" t="inlineStr">
         <is>
-          <t>https://gelzbetoniogamyba.lt/</t>
+          <t>https://inroma.lt/</t>
         </is>
       </c>
       <c r="W41" s="2" t="inlineStr">
         <is>
-          <t>https://gelzbetoniogamyba.lt/</t>
+          <t>https://inroma.lt/</t>
         </is>
       </c>
       <c r="X41" s="2" t="inlineStr">
         <is>
-          <t>https://gelzbetoniogamyba.lt/</t>
+          <t>https://inroma.lt/</t>
         </is>
       </c>
       <c r="Y41" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti ryšį su kitomis S. Kerbedžio g. 52 įmonėmis.</t>
+          <t>Reikia patikslinti našumą.</t>
         </is>
       </c>
       <c r="Z41" s="2" t="inlineStr">
@@ -5286,18 +5290,22 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>inroma-pakruojis</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr"/>
+          <t>utenos-betonas-utena</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>300904691</t>
+        </is>
+      </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>UAB Inroma</t>
+          <t>UAB Utenos betonas</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Inroma</t>
+          <t>Utenos betonas</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -5307,24 +5315,24 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Pakruojis</t>
+          <t>Utena</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Pakruojo r. sav.</t>
+          <t>Utenos r. sav.</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Pramonės g. 5B, Pakruojis</t>
+          <t>Metalo g. 9B, Utena</t>
         </is>
       </c>
       <c r="I42" s="3" t="n">
-        <v>55.9763263</v>
+        <v>55.4947607</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>23.8584712</v>
+        <v>25.6225075</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -5353,7 +5361,7 @@
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>Inroma betono mazgas</t>
+          <t>Utenos betono mazgas</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr"/>
@@ -5361,30 +5369,30 @@
       <c r="S42" s="4" t="inlineStr"/>
       <c r="T42" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono mišinių veikla Pakruojyje.</t>
+          <t>Viešai skelbiama betono mišinių veikla Utenoje.</t>
         </is>
       </c>
       <c r="U42" s="5" t="n">
-        <v>0.72</v>
+        <v>0.78</v>
       </c>
       <c r="V42" s="2" t="inlineStr">
         <is>
-          <t>https://inroma.lt/</t>
+          <t>https://utenosbetonas.lt/</t>
         </is>
       </c>
       <c r="W42" s="2" t="inlineStr">
         <is>
-          <t>https://inroma.lt/</t>
+          <t>https://www.utenosbetonas.lt/kontaktai/</t>
         </is>
       </c>
       <c r="X42" s="2" t="inlineStr">
         <is>
-          <t>https://inroma.lt/</t>
+          <t>https://www.utenosbetonas.lt/kontaktai/</t>
         </is>
       </c>
       <c r="Y42" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti našumą.</t>
+          <t>Oficialus kontaktų puslapis patvirtina Metalo g. 9B adresą.</t>
         </is>
       </c>
       <c r="Z42" s="2" t="inlineStr">
@@ -5396,22 +5404,22 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>utenos-betonas-utena</t>
+          <t>sbetonas-jonava</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>300904691</t>
+          <t>300902683</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>UAB Utenos betonas</t>
+          <t>UAB Sbetonas</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Utenos betonas</t>
+          <t>Sbetonas</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -5421,24 +5429,24 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Utena</t>
+          <t>Jonava</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Utenos r. sav.</t>
+          <t>Jonavos r. sav.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Metalo g. 9B, Utena</t>
+          <t>Skarulių g. 58, Jonava</t>
         </is>
       </c>
       <c r="I43" s="3" t="n">
-        <v>55.4947607</v>
+        <v>55.0786452</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>25.6225075</v>
+        <v>24.3199072</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5475,7 @@
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>Utenos betono mazgas</t>
+          <t>Sbetonas betono mazgas</t>
         </is>
       </c>
       <c r="Q43" s="2" t="inlineStr"/>
@@ -5475,7 +5483,7 @@
       <c r="S43" s="4" t="inlineStr"/>
       <c r="T43" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama betono mišinių veikla Utenoje.</t>
+          <t>Viešai skelbiama prekinio betono gamyba Jonavoje.</t>
         </is>
       </c>
       <c r="U43" s="5" t="n">
@@ -5483,22 +5491,22 @@
       </c>
       <c r="V43" s="2" t="inlineStr">
         <is>
-          <t>https://utenosbetonas.lt/</t>
+          <t>https://sbetonas.lt/</t>
         </is>
       </c>
       <c r="W43" s="2" t="inlineStr">
         <is>
-          <t>https://www.utenosbetonas.lt/kontaktai/</t>
+          <t>https://sbetonas.lt/</t>
         </is>
       </c>
       <c r="X43" s="2" t="inlineStr">
         <is>
-          <t>https://www.utenosbetonas.lt/kontaktai/</t>
+          <t>https://sbetonas.lt/</t>
         </is>
       </c>
       <c r="Y43" s="2" t="inlineStr">
         <is>
-          <t>Oficialus kontaktų puslapis patvirtina Metalo g. 9B adresą.</t>
+          <t>Papildomai rasta pagal prekinio betono požymį.</t>
         </is>
       </c>
       <c r="Z43" s="2" t="inlineStr">
@@ -5510,22 +5518,18 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>sbetonas-jonava</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>300902683</t>
-        </is>
-      </c>
+          <t>kalcitas-naujoji-akmene</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>UAB Sbetonas</t>
+          <t>AB Kalcitas</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Sbetonas</t>
+          <t>Kalcitas</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -5535,24 +5539,24 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Jonava</t>
+          <t>Naujoji Akmenė</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Jonavos r. sav.</t>
+          <t>Akmenės r. sav.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Skarulių g. 58, Jonava</t>
+          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
         </is>
       </c>
       <c r="I44" s="3" t="n">
-        <v>55.0786452</v>
+        <v>56.3143832</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>24.3199072</v>
+        <v>22.9130704</v>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
@@ -5581,7 +5585,7 @@
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>Sbetonas betono mazgas</t>
+          <t>Kalcitas betono mišinių gamybos linija</t>
         </is>
       </c>
       <c r="Q44" s="2" t="inlineStr"/>
@@ -5589,30 +5593,26 @@
       <c r="S44" s="4" t="inlineStr"/>
       <c r="T44" s="2" t="inlineStr">
         <is>
-          <t>Viešai skelbiama prekinio betono gamyba Jonavoje.</t>
+          <t>Viešame kataloge nurodomi betonas, betono mišiniai ir betono gamybos linija Naujojoje Akmenėje.</t>
         </is>
       </c>
       <c r="U44" s="5" t="n">
         <v>0.78</v>
       </c>
-      <c r="V44" s="2" t="inlineStr">
-        <is>
-          <t>https://sbetonas.lt/</t>
-        </is>
-      </c>
+      <c r="V44" s="2" t="inlineStr"/>
       <c r="W44" s="2" t="inlineStr">
         <is>
-          <t>https://sbetonas.lt/</t>
+          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
         </is>
       </c>
       <c r="X44" s="2" t="inlineStr">
         <is>
-          <t>https://sbetonas.lt/</t>
+          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
         </is>
       </c>
       <c r="Y44" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta pagal prekinio betono požymį.</t>
+          <t>Reikia patikslinti, ar veikla yra nuolat aktyvi.</t>
         </is>
       </c>
       <c r="Z44" s="2" t="inlineStr">
@@ -5624,18 +5624,18 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>kalcitas-naujoji-akmene</t>
+          <t>gelgaudiskio-gelzbetonis-gelgaudiskis</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr"/>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>AB Kalcitas</t>
+          <t>UAB Gelgaudiškio gelžbetonis</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Kalcitas</t>
+          <t>Gelgaudiškio gelžbetonis</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -5645,24 +5645,24 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Naujoji Akmenė</t>
+          <t>Gelgaudiškis</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Akmenės r. sav.</t>
+          <t>Šakių r. sav.</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
+          <t>Vakarų g. 33 D, 71431, Gelgaudiškis</t>
         </is>
       </c>
       <c r="I45" s="3" t="n">
-        <v>56.3143832</v>
+        <v>55.07067</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>22.9130704</v>
+        <v>22.976723</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -5671,27 +5671,27 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>GLG kontaktų puslapis</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://glg.lt/kontaktai/</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>ready_mix_concrete</t>
+          <t>precast_concrete</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>Betono mišiniai</t>
+          <t>Betono mišiniai ir gelžbetonis</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>Kalcitas betono mišinių gamybos linija</t>
+          <t>Gelgaudiškio gelžbetonio gamykla</t>
         </is>
       </c>
       <c r="Q45" s="2" t="inlineStr"/>
@@ -5699,26 +5699,30 @@
       <c r="S45" s="4" t="inlineStr"/>
       <c r="T45" s="2" t="inlineStr">
         <is>
-          <t>Viešame kataloge nurodomi betonas, betono mišiniai ir betono gamybos linija Naujojoje Akmenėje.</t>
+          <t>Įmonė gamina gelžbetonio gaminius, prekinį ir hidrotechninį betoną bei smėlbetonio mišinius.</t>
         </is>
       </c>
       <c r="U45" s="5" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="V45" s="2" t="inlineStr"/>
+        <v>0.9</v>
+      </c>
+      <c r="V45" s="2" t="inlineStr">
+        <is>
+          <t>https://glg.lt/</t>
+        </is>
+      </c>
       <c r="W45" s="2" t="inlineStr">
         <is>
-          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
+          <t>https://glg.lt/kontaktai/</t>
         </is>
       </c>
       <c r="X45" s="2" t="inlineStr">
         <is>
-          <t>https://www.1551.lt/kalcitas-ab-betonas-betono-misiniai-betono-gamybos-linija-technikos-nuoma-naujojoje-akmeneje-59982/</t>
+          <t>https://glg.lt/betonas/betono-misiniai/</t>
         </is>
       </c>
       <c r="Y45" s="2" t="inlineStr">
         <is>
-          <t>Reikia patikslinti, ar veikla yra nuolat aktyvi.</t>
+          <t>Patikslinta pagal oficialų glg.lt kontaktų ir įmonės aprašymo puslapius.</t>
         </is>
       </c>
       <c r="Z45" s="2" t="inlineStr">
@@ -5730,45 +5734,49 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>gelgaudiskio-gelzbetonis-gelgaudiskis</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr"/>
+          <t>ginfa-kutiskiai</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>302680943</t>
+        </is>
+      </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>UAB Gelgaudiškio gelžbetonis</t>
+          <t>UAB GinFa</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Gelgaudiškio gelžbetonis</t>
+          <t>GinFa</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta</t>
+          <t>Papildomai rasta EVRK 23.63</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Gelgaudiškis</t>
+          <t>Kutiškiai</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Šakių r. sav.</t>
+          <t>Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Vakarų g. 33 D, 71431, Gelgaudiškis</t>
+          <t>Alyvų g. 8, Kutiškiai, Radviliškio r.</t>
         </is>
       </c>
       <c r="I46" s="3" t="n">
-        <v>55.07067</v>
+        <v>55.8326273</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>22.976723</v>
+        <v>23.4995317</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
@@ -5777,27 +5785,27 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>GLG kontaktų puslapis</t>
+          <t>Lietuvos geolokatorius</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>https://glg.lt/kontaktai/</t>
+          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>precast_concrete</t>
+          <t>ready_mix_concrete</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>Betono mišiniai ir gelžbetonis</t>
+          <t>Betono mišiniai</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>Gelgaudiškio gelžbetonio gamykla</t>
+          <t>GinFa betono gamyba</t>
         </is>
       </c>
       <c r="Q46" s="2" t="inlineStr"/>
@@ -5805,30 +5813,22 @@
       <c r="S46" s="4" t="inlineStr"/>
       <c r="T46" s="2" t="inlineStr">
         <is>
-          <t>Įmonė gamina gelžbetonio gaminius, prekinį ir hidrotechninį betoną bei smėlbetonio mišinius.</t>
+          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
         </is>
       </c>
       <c r="U46" s="5" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="V46" s="2" t="inlineStr">
-        <is>
-          <t>https://glg.lt/</t>
-        </is>
-      </c>
+        <v>0.82</v>
+      </c>
+      <c r="V46" s="2" t="inlineStr"/>
       <c r="W46" s="2" t="inlineStr">
         <is>
-          <t>https://glg.lt/kontaktai/</t>
-        </is>
-      </c>
-      <c r="X46" s="2" t="inlineStr">
-        <is>
-          <t>https://glg.lt/betonas/betono-misiniai/</t>
-        </is>
-      </c>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="X46" s="2" t="inlineStr"/>
       <c r="Y46" s="2" t="inlineStr">
         <is>
-          <t>Patikslinta pagal oficialų glg.lt kontaktų ir įmonės aprašymo puslapius.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z46" s="2" t="inlineStr">
@@ -5840,22 +5840,22 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>ginfa-kutiskiai</t>
+          <t>antano-gribino-imone-prienai</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>302680943</t>
+          <t>170687267</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>UAB GinFa</t>
+          <t>IĮ Antano Gribino gamybos ir komercinės veiklos įmonė</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>GinFa</t>
+          <t>Antano Gribino įmonė</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -5865,24 +5865,24 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Kutiškiai</t>
+          <t>Prienai</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Radviliškio r. sav.</t>
+          <t>Prienų r. sav.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Alyvų g. 8, Kutiškiai, Radviliškio r.</t>
+          <t>Kęstučio g. 95A, Prienai</t>
         </is>
       </c>
       <c r="I47" s="3" t="n">
-        <v>55.8326273</v>
+        <v>54.6523184</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>23.4995317</v>
+        <v>23.9696591</v>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
@@ -5911,7 +5911,7 @@
       </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>GinFa betono gamyba</t>
+          <t>Antano Gribino įmonės betono gamyba</t>
         </is>
       </c>
       <c r="Q47" s="2" t="inlineStr"/>
@@ -5946,22 +5946,22 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>antano-gribino-imone-prienai</t>
+          <t>vinido-taurage</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>170687267</t>
+          <t>306258220</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>IĮ Antano Gribino gamybos ir komercinės veiklos įmonė</t>
+          <t>UAB Vinido</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Antano Gribino įmonė</t>
+          <t>Vinido</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -5971,24 +5971,24 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Prienai</t>
+          <t>Tauragė</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Prienų r. sav.</t>
+          <t>Tauragės r. sav.</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Kęstučio g. 95A, Prienai</t>
+          <t>Gaurės g. 32, Tauragė</t>
         </is>
       </c>
       <c r="I48" s="3" t="n">
-        <v>54.6523184</v>
+        <v>55.2492204</v>
       </c>
       <c r="J48" s="3" t="n">
-        <v>23.9696591</v>
+        <v>22.3185845</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
@@ -6015,59 +6015,67 @@
           <t>Betono mišiniai</t>
         </is>
       </c>
-      <c r="P48" s="2" t="inlineStr">
-        <is>
-          <t>Antano Gribino įmonės betono gamyba</t>
-        </is>
-      </c>
+      <c r="P48" s="2" t="inlineStr"/>
       <c r="Q48" s="2" t="inlineStr"/>
-      <c r="R48" s="2" t="inlineStr"/>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>200–250 m³/dieną (gamyba ir pristatymas)</t>
+        </is>
+      </c>
       <c r="S48" s="4" t="inlineStr"/>
       <c r="T48" s="2" t="inlineStr">
         <is>
-          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+          <t>Nuosavas betono mazgas Tauragėje. Įmonė skelbia galinti pagaminti ir pristatyti iki 200–250 m³ betono per dieną; užsakius nuo 50 m³ dirba ir savaitgaliais. Teikia betono gamybos ir tiekimo, betono siurblio nuomos bei betono gaminių gamybos paslaugas.</t>
         </is>
       </c>
       <c r="U48" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V48" s="2" t="inlineStr"/>
+      <c r="V48" s="2" t="inlineStr">
+        <is>
+          <t>https://betonastaurageje.lt/</t>
+        </is>
+      </c>
       <c r="W48" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X48" s="2" t="inlineStr"/>
+          <t>https://betonastaurageje.lt/kontaktai/</t>
+        </is>
+      </c>
+      <c r="X48" s="2" t="inlineStr">
+        <is>
+          <t>https://betonastaurageje.lt/uab-vinido-betonas/</t>
+        </is>
+      </c>
       <c r="Y48" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Oficiali svetainė patvirtina įmonės kodą 306258220, Gaurės g. 32 adresą ir nuosavą betono mazgą. Kontaktai: +370 644 45799, info@uabvinido.lt. 200–250 m³/dieną yra skelbiama gamybos ir pristatymo apimtis, ne valandinis mazgo našumas. Mazgo gamintojas, maišyklė ir silosai viešai nenurodyti.</t>
         </is>
       </c>
       <c r="Z48" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>vinido-taurage</t>
+          <t>santvara-kedainiai</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>306258220</t>
+          <t>304915297</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>UAB Vinido</t>
+          <t>UAB Santvara</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Vinido</t>
+          <t>Santvara</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -6077,24 +6085,24 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Tauragė</t>
+          <t>Kėdainiai</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Tauragės r. sav.</t>
+          <t>Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Gaurės g. 32, Tauragė</t>
+          <t>Aruodų g. 34, Kėdainiai</t>
         </is>
       </c>
       <c r="I49" s="3" t="n">
-        <v>55.2492204</v>
+        <v>55.2634747</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>22.3185845</v>
+        <v>23.9440384</v>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
@@ -6123,7 +6131,7 @@
       </c>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>Vinido betono gamyba</t>
+          <t>Santvara betono gamyba</t>
         </is>
       </c>
       <c r="Q49" s="2" t="inlineStr"/>
@@ -6139,22 +6147,22 @@
       </c>
       <c r="V49" s="2" t="inlineStr">
         <is>
-          <t>https://betonastaurageje.lt/</t>
+          <t>https://santvara.eu/</t>
         </is>
       </c>
       <c r="W49" s="2" t="inlineStr">
         <is>
-          <t>https://betonastaurageje.lt/kontaktai/</t>
+          <t>https://santvara.eu/</t>
         </is>
       </c>
       <c r="X49" s="2" t="inlineStr">
         <is>
-          <t>https://betonastaurageje.lt/betonas/</t>
+          <t>https://santvara.eu/</t>
         </is>
       </c>
       <c r="Y49" s="2" t="inlineStr">
         <is>
-          <t>Oficiali Vinido svetainė patvirtina Gaurės g. 32 adresą, betono gamybą ir betono mazgą.</t>
+          <t>Oficiali Santvara svetainė patvirtina Aruodų g. 34 adresą ir betono bei birių medžiagų veiklą.</t>
         </is>
       </c>
       <c r="Z49" s="2" t="inlineStr">
@@ -6166,22 +6174,22 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>santvara-kedainiai</t>
+          <t>medis-ir-betonas-naujoji-akmene</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>304915297</t>
+          <t>153074073</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>UAB Santvara</t>
+          <t>AB Medis ir betonas</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Santvara</t>
+          <t>Medis ir betonas</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -6191,24 +6199,24 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Kėdainiai</t>
+          <t>Naujoji Akmenė</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Kėdainių r. sav.</t>
+          <t>Akmenės r. sav.</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Aruodų g. 34, Kėdainiai</t>
+          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
         </is>
       </c>
       <c r="I50" s="3" t="n">
-        <v>55.2634747</v>
+        <v>56.3143832</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>23.9440384</v>
+        <v>22.9130704</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
@@ -6237,7 +6245,7 @@
       </c>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>Santvara betono gamyba</t>
+          <t>Medis ir betonas gamyba</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr"/>
@@ -6251,24 +6259,16 @@
       <c r="U50" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V50" s="2" t="inlineStr">
-        <is>
-          <t>https://santvara.eu/</t>
-        </is>
-      </c>
+      <c r="V50" s="2" t="inlineStr"/>
       <c r="W50" s="2" t="inlineStr">
         <is>
-          <t>https://santvara.eu/</t>
-        </is>
-      </c>
-      <c r="X50" s="2" t="inlineStr">
-        <is>
-          <t>https://santvara.eu/</t>
-        </is>
-      </c>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="X50" s="2" t="inlineStr"/>
       <c r="Y50" s="2" t="inlineStr">
         <is>
-          <t>Oficiali Santvara svetainė patvirtina Aruodų g. 34 adresą ir betono bei birių medžiagų veiklą.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z50" s="2" t="inlineStr">
@@ -6280,22 +6280,22 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>medis-ir-betonas-naujoji-akmene</t>
+          <t>ekobetonas-marijampole</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>153074073</t>
+          <t>300636364</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>AB Medis ir betonas</t>
+          <t>UAB Ekobetonas</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Medis ir betonas</t>
+          <t>Ekobetonas</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -6305,24 +6305,24 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Naujoji Akmenė</t>
+          <t>Marijampolė</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Akmenės r. sav.</t>
+          <t>Marijampolės sav.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>J. Dalinkevičiaus g. 2, Naujoji Akmenė</t>
+          <t>Gamyklų g. 3, Marijampolė</t>
         </is>
       </c>
       <c r="I51" s="3" t="n">
-        <v>56.3143832</v>
+        <v>54.5750142</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>22.9130704</v>
+        <v>23.3796805</v>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
@@ -6351,7 +6351,7 @@
       </c>
       <c r="P51" s="2" t="inlineStr">
         <is>
-          <t>Medis ir betonas gamyba</t>
+          <t>Ekobetonas betono gamyba</t>
         </is>
       </c>
       <c r="Q51" s="2" t="inlineStr"/>
@@ -6365,16 +6365,24 @@
       <c r="U51" s="5" t="n">
         <v>0.82</v>
       </c>
-      <c r="V51" s="2" t="inlineStr"/>
+      <c r="V51" s="2" t="inlineStr">
+        <is>
+          <t>https://ekobetonas.lt/</t>
+        </is>
+      </c>
       <c r="W51" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X51" s="2" t="inlineStr"/>
+          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
+        </is>
+      </c>
+      <c r="X51" s="2" t="inlineStr">
+        <is>
+          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
+        </is>
+      </c>
       <c r="Y51" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Oficialus Ekobetonas kontaktų puslapis patvirtina Gamyklų g. 3 adresą ir betono užsakymų kontaktus.</t>
         </is>
       </c>
       <c r="Z51" s="2" t="inlineStr">
@@ -6386,22 +6394,22 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>ekobetonas-marijampole</t>
+          <t>rokbetonis-rokiskis</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>300636364</t>
+          <t>304184091</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>UAB Ekobetonas</t>
+          <t>MB Rokbetonis</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Ekobetonas</t>
+          <t>Rokbetonis</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -6411,24 +6419,24 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Marijampolė</t>
+          <t>Rokiškis</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Marijampolės sav.</t>
+          <t>Rokiškio r. sav.</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Gamyklų g. 3, Marijampolė</t>
+          <t>Vydūno g. 12A, Parokiškė, Rokiškio r.</t>
         </is>
       </c>
       <c r="I52" s="3" t="n">
-        <v>54.5750142</v>
+        <v>55.9525796</v>
       </c>
       <c r="J52" s="3" t="n">
-        <v>23.3796805</v>
+        <v>25.5624197</v>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
@@ -6457,7 +6465,7 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>Ekobetonas betono gamyba</t>
+          <t>Rokbetonis betono gamyba</t>
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr"/>
@@ -6469,26 +6477,18 @@
         </is>
       </c>
       <c r="U52" s="5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="V52" s="2" t="inlineStr">
-        <is>
-          <t>https://ekobetonas.lt/</t>
-        </is>
-      </c>
+        <v>0.72</v>
+      </c>
+      <c r="V52" s="2" t="inlineStr"/>
       <c r="W52" s="2" t="inlineStr">
         <is>
-          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
-        </is>
-      </c>
-      <c r="X52" s="2" t="inlineStr">
-        <is>
-          <t>https://ekobetonas.lt/kontaktai-betono-gamyba-armaturinis-plienas/</t>
-        </is>
-      </c>
+          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+        </is>
+      </c>
+      <c r="X52" s="2" t="inlineStr"/>
       <c r="Y52" s="2" t="inlineStr">
         <is>
-          <t>Oficialus Ekobetonas kontaktų puslapis patvirtina Gamyklų g. 3 adresą ir betono užsakymų kontaktus.</t>
+          <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Rokiškio miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
         </is>
       </c>
       <c r="Z52" s="2" t="inlineStr">
@@ -6500,22 +6500,22 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>rokbetonis-rokiskis</t>
+          <t>kruszbet-lithuania-jure</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>304184091</t>
+          <t>305173596</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>MB Rokbetonis</t>
+          <t>UAB KRUSZBET Lithuania</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Rokbetonis</t>
+          <t>KRUSZBET Lithuania</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -6525,24 +6525,24 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Rokiškis</t>
+          <t>Jūrė</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Rokiškio r. sav.</t>
+          <t>Kazlų Rūdos sav.</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Vydūno g. 12A, Parokiškė, Rokiškio r.</t>
+          <t>Medelyno g. 30A, Jūrė, Kazlų Rūdos sav.</t>
         </is>
       </c>
       <c r="I53" s="3" t="n">
-        <v>55.9525796</v>
+        <v>54.7706307</v>
       </c>
       <c r="J53" s="3" t="n">
-        <v>25.5624197</v>
+        <v>23.4998409</v>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
@@ -6571,7 +6571,7 @@
       </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>Rokbetonis betono gamyba</t>
+          <t>KRUSZBET Lithuania betono gamyba</t>
         </is>
       </c>
       <c r="Q53" s="2" t="inlineStr"/>
@@ -6583,7 +6583,7 @@
         </is>
       </c>
       <c r="U53" s="5" t="n">
-        <v>0.72</v>
+        <v>0.82</v>
       </c>
       <c r="V53" s="2" t="inlineStr"/>
       <c r="W53" s="2" t="inlineStr">
@@ -6594,7 +6594,7 @@
       <c r="X53" s="2" t="inlineStr"/>
       <c r="Y53" s="2" t="inlineStr">
         <is>
-          <t>Adresas rastas viešuose kataloguose, bet geokoduotas tik iki Rokiškio miesto taško; reikia patikslinti tikslų betono mazgo GPS.</t>
+          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
         </is>
       </c>
       <c r="Z53" s="2" t="inlineStr">
@@ -6606,49 +6606,49 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>silutes-betonas-silute</t>
+          <t>telsiu-keliai-telsiai</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>177392928</t>
+          <t>180200843</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>UAB Šilutės betonas</t>
+          <t>UAB Telšių keliai</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Šilutės betonas</t>
+          <t>Telšių keliai</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta EVRK 23.63</t>
+          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Šilutė</t>
+          <t>Telšiai</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Šilutės r. sav.</t>
+          <t>Telšių r. sav.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Ramučių g. 1, Šilutė</t>
+          <t>Mažeikių g. 18, Telšiai</t>
         </is>
       </c>
       <c r="I54" s="3" t="n">
-        <v>55.3538641</v>
+        <v>56.0004158</v>
       </c>
       <c r="J54" s="3" t="n">
-        <v>21.4796635</v>
+        <v>22.2581129</v>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
@@ -6677,102 +6677,108 @@
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>Šilutės betono gamyba (Nebeaktyvus mazgas)</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q54" s="2" t="inlineStr"/>
       <c r="R54" s="2" t="inlineStr"/>
-      <c r="S54" s="4" t="inlineStr"/>
+      <c r="S54" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T54" s="2" t="inlineStr">
         <is>
-          <t>Nebeaktyvus mazgas. Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai.</t>
         </is>
       </c>
       <c r="U54" s="5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="V54" s="2" t="inlineStr"/>
+        <v>0.86</v>
+      </c>
+      <c r="V54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tkeliai.lt/</t>
+        </is>
+      </c>
       <c r="W54" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
         </is>
       </c>
       <c r="X54" s="2" t="inlineStr">
         <is>
-          <t>https://fsaskaita.lt/imone/uzdaroji-akcine-bendrove-silutes-betonas-177392928</t>
+          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
         </is>
       </c>
       <c r="Y54" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą. Mazgas pažymėtas nebeaktyviu pagal naudotojo pateiktą informaciją.</t>
+          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
         </is>
       </c>
       <c r="Z54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>kruszbet-lithuania-jure</t>
+          <t>vpa-laistai</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>305173596</t>
+          <t>110185819</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>UAB KRUSZBET Lithuania</t>
+          <t>UAB V. Paulius &amp; Associates</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>KRUSZBET Lithuania</t>
+          <t>VPA</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Papildomai rasta EVRK 23.63</t>
+          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Jūrė</t>
+          <t>Laistai</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Kazlų Rūdos sav.</t>
+          <t>Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Medelyno g. 30A, Jūrė, Kazlų Rūdos sav.</t>
+          <t>Stariškės g. 9, Laistų k., Dovilų sen., Klaipėdos r. sav.</t>
         </is>
       </c>
       <c r="I55" s="3" t="n">
-        <v>54.7706307</v>
+        <v>55.636908</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>23.4998409</v>
+        <v>21.209254</v>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Naudotojo pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>Google Maps nuoroda</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
         </is>
       </c>
       <c r="N55" s="2" t="inlineStr">
@@ -6787,98 +6793,116 @@
       </c>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>KRUSZBET Lithuania betono gamyba</t>
-        </is>
-      </c>
-      <c r="Q55" s="2" t="inlineStr"/>
-      <c r="R55" s="2" t="inlineStr"/>
-      <c r="S55" s="4" t="inlineStr"/>
+          <t>Liebherr</t>
+        </is>
+      </c>
+      <c r="Q55" s="2" t="inlineStr">
+        <is>
+          <t>3 m³</t>
+        </is>
+      </c>
+      <c r="R55" s="2" t="inlineStr">
+        <is>
+          <t>60-80 m³/h</t>
+        </is>
+      </c>
+      <c r="S55" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="T55" s="2" t="inlineStr">
         <is>
-          <t>Registrų centro/VDA atviruose duomenyse pagrindinė veikla nurodyta kaip prekinio betono mišinio gamyba (EVRK 23.63).</t>
+          <t>VPA betono mazgas Klaipėdos rajone.</t>
         </is>
       </c>
       <c r="U55" s="5" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="V55" s="2" t="inlineStr"/>
+        <v>0.7</v>
+      </c>
+      <c r="V55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vpa.lt/</t>
+        </is>
+      </c>
       <c r="W55" s="2" t="inlineStr">
         <is>
-          <t>https://data.gov.lt/dataset/juridiniu-asmenu-ekonomines-veiklos-rusys-ir-instituciniai-sektoriai/</t>
-        </is>
-      </c>
-      <c r="X55" s="2" t="inlineStr"/>
+          <t>https://www.vpa.lt/?Kontaktai=</t>
+        </is>
+      </c>
+      <c r="X55" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+        </is>
+      </c>
       <c r="Y55" s="2" t="inlineStr">
         <is>
-          <t>Adresas geokoduotas pagal viešai randamą įmonės adresą; betono mazgo vietą verta patikslinti atskiru šaltiniu.</t>
+          <t>Vieta nustatyta pagal naudotojo pateiktą Google Maps nuorodą. VPA kontaktų puslapis nurodo Stariškės g. 9, Laistų k. adresą. Techniniai mazgo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z55" s="2" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>telsiu-keliai-telsiai</t>
+          <t>c3-beton-baisogala</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>180200843</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>UAB Telšių keliai</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Telšių keliai</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
+          <t>Konkurentas</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Telšiai</t>
+          <t>Baisogala</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Telšių r. sav.</t>
+          <t>Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Mažeikių g. 18, Telšiai</t>
+          <t>Dvaro g., Baisogala, Radviliškio r. sav.</t>
         </is>
       </c>
       <c r="I56" s="3" t="n">
-        <v>56.0004158</v>
+        <v>55.6372</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>22.2581129</v>
+        <v>23.7183</v>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas</t>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>Lietuvos geolokatorius</t>
+          <t>C3 Betonas oficialus puslapis</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>https://hub.arcgis.com/content/b9e27b4266524b39bc651d6a26480b87</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="N56" s="2" t="inlineStr">
@@ -6893,108 +6917,118 @@
       </c>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>Elkon</t>
-        </is>
-      </c>
-      <c r="Q56" s="2" t="inlineStr"/>
-      <c r="R56" s="2" t="inlineStr"/>
-      <c r="S56" s="4" t="n">
-        <v>2</v>
+          <t>Baisiogala Plant</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
+      </c>
+      <c r="S56" s="4" t="inlineStr">
+        <is>
+          <t>Nenurodyta viešai</t>
+        </is>
       </c>
       <c r="T56" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame įmonės puslapyje skelbiama betono mišinių gamyba ir prekyba. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai.</t>
+          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
         </is>
       </c>
       <c r="U56" s="5" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="V56" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/</t>
+          <t>https://c3beton.com/</t>
         </is>
       </c>
       <c r="W56" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="X56" s="2" t="inlineStr">
         <is>
-          <t>https://www.tkeliai.lt/kitos-paslaugos/</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="Y56" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal naudotojo informaciją; veikla patvirtinta oficialiame lietuviškame įmonės puslapyje. Naudotojo duomenimis, betono mazgas vadinasi Elkon, yra 2 silosai. Koordinatės nustatytos Lietuvos geolokatoriumi pagal Mažeikių g. 18 adresą.</t>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
         </is>
       </c>
       <c r="Z56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>vpa-laistai</t>
+          <t>c3-beton-martiniskis</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>110185819</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>UAB V. Paulius &amp; Associates</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>VPA</t>
+          <t>C3 Betonas</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Papildomai įtraukta pagal naudotojo informaciją</t>
+          <t>Konkurentas</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Laistai</t>
+          <t>Martiniškis</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Klaipėdos r. sav.</t>
+          <t>Jonavos r. sav.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Stariškės g. 9, Laistų k., Dovilų sen., Klaipėdos r. sav.</t>
+          <t>Vanagiškiai, Kulvos sen., Jonavos r. sav.</t>
         </is>
       </c>
       <c r="I57" s="3" t="n">
-        <v>55.636908</v>
+        <v>55.1441659</v>
       </c>
       <c r="J57" s="3" t="n">
-        <v>21.209254</v>
+        <v>24.1869636</v>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Naudotojo pateiktos Google Maps nuorodos taškas</t>
+          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>Google Maps nuoroda</t>
+          <t>C3 Betonas oficialus puslapis</t>
         </is>
       </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="N57" s="2" t="inlineStr">
@@ -7009,60 +7043,62 @@
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
-          <t>Liebherr</t>
+          <t>Martiniškis Plant</t>
         </is>
       </c>
       <c r="Q57" s="2" t="inlineStr">
         <is>
-          <t>3 m³</t>
+          <t>Ammann Elba Euromix C120, 3 m³</t>
         </is>
       </c>
       <c r="R57" s="2" t="inlineStr">
         <is>
-          <t>60-80 m³/h</t>
-        </is>
-      </c>
-      <c r="S57" s="4" t="n">
-        <v>2</v>
+          <t>60–80 m³/val.</t>
+        </is>
+      </c>
+      <c r="S57" s="4" t="inlineStr">
+        <is>
+          <t>2x85 t</t>
+        </is>
       </c>
       <c r="T57" s="2" t="inlineStr">
         <is>
-          <t>VPA betono mazgas Klaipėdos rajone.</t>
+          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U57" s="5" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="V57" s="2" t="inlineStr">
         <is>
-          <t>https://www.vpa.lt/</t>
+          <t>https://c3beton.com/</t>
         </is>
       </c>
       <c r="W57" s="2" t="inlineStr">
         <is>
-          <t>https://www.vpa.lt/?Kontaktai=</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="X57" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/2geTBr4zmdrmPY548</t>
+          <t>https://c3beton.com/lt/betonas</t>
         </is>
       </c>
       <c r="Y57" s="2" t="inlineStr">
         <is>
-          <t>Vieta nustatyta pagal naudotojo pateiktą Google Maps nuorodą. VPA kontaktų puslapis nurodo Stariškės g. 9, Laistų k. adresą. Techniniai mazgo duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z57" s="2" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-14</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-baisogala</t>
+          <t>c3-beton-stasenai</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -7087,38 +7123,38 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Baisogala</t>
+          <t>Vilnius</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Radviliškio r. sav.</t>
+          <t>Vilniaus m. sav.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Dvaro g., Baisogala, Radviliškio r. sav.</t>
+          <t>Ušos g. 21, Vilnius, 02121 Vilniaus m. sav.</t>
         </is>
       </c>
       <c r="I58" s="3" t="n">
-        <v>55.6372</v>
+        <v>54.6493094</v>
       </c>
       <c r="J58" s="3" t="n">
-        <v>23.7183</v>
+        <v>25.3107972</v>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
+          <t>Tikslus adreso taškas pagal geokodavimą</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas oficialus puslapis</t>
+          <t>ArcGIS geokodavimas pagal naudotojo pateiktą adresą</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://geocode.arcgis.com/arcgis/rest/services/World/GeocodeServer/findAddressCandidates</t>
         </is>
       </c>
       <c r="N58" s="2" t="inlineStr">
@@ -7133,27 +7169,27 @@
       </c>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>Baisiogala Plant</t>
+          <t>Vilnius Ušos g. Plant</t>
         </is>
       </c>
       <c r="Q58" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>Nissbau Euromix C120, 3 m³</t>
         </is>
       </c>
       <c r="R58" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>60–80 m³/val.</t>
         </is>
       </c>
       <c r="S58" s="4" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>2x85 t</t>
         </is>
       </c>
       <c r="T58" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame C3 Betonas puslapyje ši vieta rodoma kaip C3 betono gamykla Lietuvos tinkle. C3 nurodo, kad aplink gamyklas taikomas 50 km pristatymo spindulys.</t>
+          <t>Betono mazgas Nissbau Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U58" s="5" t="n">
@@ -7176,7 +7212,7 @@
       </c>
       <c r="Y58" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Įmonės kodas ir techniniai mazgo duomenys viešai nenurodyti.</t>
+          <t>Perkelta iš Stašėnų lokacijos į Ušos g. 21, Vilnius pagal naudotojo pateiktą informaciją. Maišyklė pervadinta į Nissbau Euromix C120, 3 m³. Koordinatės geokoduotos pagal naują adresą.</t>
         </is>
       </c>
       <c r="Z58" s="2" t="inlineStr">
@@ -7188,7 +7224,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-martiniskis</t>
+          <t>c3-beton-runeikiai</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -7213,24 +7249,24 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Martiniškis</t>
+          <t>Runeikiai</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Jonavos r. sav.</t>
+          <t>Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Vanagiškiai, Kulvos sen., Jonavos r. sav.</t>
+          <t>Paguiriai, Šėtos sen., Kėdainių r. sav.</t>
         </is>
       </c>
       <c r="I59" s="3" t="n">
-        <v>55.1441659</v>
+        <v>55.3327393</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>24.1869636</v>
+        <v>24.3501308</v>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
@@ -7259,7 +7295,7 @@
       </c>
       <c r="P59" s="2" t="inlineStr">
         <is>
-          <t>Martiniškis Plant</t>
+          <t>Runeikiai Plant</t>
         </is>
       </c>
       <c r="Q59" s="2" t="inlineStr">
@@ -7314,22 +7350,22 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-stasenai</t>
+          <t>reljef-rukla</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>301731961</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas</t>
+          <t>UAB Reljef</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>C3 Betonas</t>
+          <t>Reljef</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -7339,38 +7375,38 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Vilnius</t>
+          <t>Rukla</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus m. sav.</t>
+          <t>Jonavos r. sav.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Ušos g. 21, Vilnius, 02121 Vilniaus m. sav.</t>
+          <t>Rukla, Jonavos r. sav.</t>
         </is>
       </c>
       <c r="I60" s="3" t="n">
-        <v>54.6493094</v>
+        <v>55.05225</v>
       </c>
       <c r="J60" s="3" t="n">
-        <v>25.3107972</v>
+        <v>24.4064167</v>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>Tikslus adreso taškas pagal geokodavimą</t>
+          <t>Tikslus naudotojo pateiktas taškas; adresas artimiausias pagal OpenStreetMap</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>ArcGIS geokodavimas pagal naudotojo pateiktą adresą</t>
+          <t>Naudotojo pateiktos koordinatės</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>https://geocode.arcgis.com/arcgis/rest/services/World/GeocodeServer/findAddressCandidates</t>
+          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
@@ -7385,203 +7421,203 @@
       </c>
       <c r="P60" s="2" t="inlineStr">
         <is>
-          <t>Vilnius Ušos g. Plant</t>
+          <t>Ammann Elba</t>
         </is>
       </c>
       <c r="Q60" s="2" t="inlineStr">
         <is>
-          <t>Nissbau Euromix C120, 3 m³</t>
+          <t>Nenustatyta</t>
         </is>
       </c>
       <c r="R60" s="2" t="inlineStr">
         <is>
-          <t>60–80 m³/val.</t>
+          <t>Nenustatytas</t>
         </is>
       </c>
       <c r="S60" s="4" t="inlineStr">
         <is>
-          <t>2x85 t</t>
+          <t>2x65 t</t>
         </is>
       </c>
       <c r="T60" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgas Nissbau Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
+          <t>Rukloje veikiantis UAB Reljef betono mazgas: Ammann Elba, 2x65 t silosai. Maišyklė ir našumas nenustatyti.</t>
         </is>
       </c>
       <c r="U60" s="5" t="n">
-        <v>0.9</v>
+        <v>0.82</v>
       </c>
       <c r="V60" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/</t>
+          <t>https://www.reljef.lt/</t>
         </is>
       </c>
       <c r="W60" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.reljef.lt/</t>
         </is>
       </c>
       <c r="X60" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
         </is>
       </c>
       <c r="Y60" s="2" t="inlineStr">
         <is>
-          <t>Perkelta iš Stašėnų lokacijos į Ušos g. 21, Vilnius pagal naudotojo pateiktą informaciją. Maišyklė pervadinta į Nissbau Euromix C120, 3 m³. Koordinatės geokoduotos pagal naują adresą.</t>
+          <t>Įmonės rekvizitai paimti iš oficialaus UAB Reljef puslapio. Betono mazgo gamintojas, silosai ir lokacija įrašyti pagal naudotojo pateiktą informaciją. Artimiausias viešai geokoduotas adresas nustatytas pagal OpenStreetMap.</t>
         </is>
       </c>
       <c r="Z60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>c3-beton-runeikiai</t>
+          <t>ponas-betonas-paraudondvariai</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
+          <t>306676006</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>UAB Ponas betonas</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Ponas betonas</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Konkurentas</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Paraudondvariai</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Vilniaus r. sav.</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Vilniaus g., Paraudondvariai, Riešės sen., Vilniaus r. sav.</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="n">
+        <v>54.8321418</v>
+      </c>
+      <c r="J61" s="3" t="n">
+        <v>25.2755596</v>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>Naudotojo pateikta Google Maps lokacija</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>https://maps.app.goo.gl/NxQohpnzv1q9DA6CA?g_st=ac</t>
+        </is>
+      </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>ready_mix_concrete</t>
+        </is>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>Betono mišiniai</t>
+        </is>
+      </c>
+      <c r="P61" s="2" t="inlineStr">
+        <is>
+          <t>Elkon</t>
+        </is>
+      </c>
+      <c r="Q61" s="2" t="inlineStr">
+        <is>
           <t>Nenurodyta viešai</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>C3 Betonas</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>C3 Betonas</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>Konkurentas</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>Runeikiai</t>
-        </is>
-      </c>
-      <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t>Kėdainių r. sav.</t>
-        </is>
-      </c>
-      <c r="H61" s="2" t="inlineStr">
-        <is>
-          <t>Paguiriai, Šėtos sen., Kėdainių r. sav.</t>
-        </is>
-      </c>
-      <c r="I61" s="3" t="n">
-        <v>55.3327393</v>
-      </c>
-      <c r="J61" s="3" t="n">
-        <v>24.3501308</v>
-      </c>
-      <c r="K61" s="2" t="inlineStr">
-        <is>
-          <t>Oficialiame puslapyje pateiktas gamyklos taškas</t>
-        </is>
-      </c>
-      <c r="L61" s="2" t="inlineStr">
-        <is>
-          <t>C3 Betonas oficialus puslapis</t>
-        </is>
-      </c>
-      <c r="M61" s="2" t="inlineStr">
-        <is>
-          <t>https://c3beton.com/lt/betonas</t>
-        </is>
-      </c>
-      <c r="N61" s="2" t="inlineStr">
-        <is>
-          <t>ready_mix_concrete</t>
-        </is>
-      </c>
-      <c r="O61" s="2" t="inlineStr">
-        <is>
-          <t>Betono mišiniai</t>
-        </is>
-      </c>
-      <c r="P61" s="2" t="inlineStr">
-        <is>
-          <t>Runeikiai Plant</t>
-        </is>
-      </c>
-      <c r="Q61" s="2" t="inlineStr">
-        <is>
-          <t>Ammann Elba Euromix C120, 3 m³</t>
-        </is>
-      </c>
       <c r="R61" s="2" t="inlineStr">
         <is>
-          <t>60–80 m³/val.</t>
+          <t>Nenurodyta viešai</t>
         </is>
       </c>
       <c r="S61" s="4" t="inlineStr">
         <is>
-          <t>2x85 t</t>
+          <t>2 matomi oficialioje nuotraukoje</t>
         </is>
       </c>
       <c r="T61" s="2" t="inlineStr">
         <is>
-          <t>Betono mazgas Ammann Elba Euromix C120; maišyklė 3 m³; našumas 60–80 m³/val.; silosai 2x85 t.</t>
+          <t>Oficialiame UAB Ponas betonas puslapyje nurodoma, kad įmonė turi nuosavą betono mazgą, gamina prekinį betoną ir jį pristato. Puslapio hero nuotraukoje ant silosų matomas ELKON ženklinimas, todėl mazgo gamintojas identifikuotas kaip Elkon. Konkretus modelis, maišyklė ir našumas viešai nenurodyti; oficialioje nuotraukoje matomi 2 silosai.</t>
         </is>
       </c>
       <c r="U61" s="5" t="n">
-        <v>0.9</v>
+        <v>0.98</v>
       </c>
       <c r="V61" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/</t>
+          <t>https://www.ponasbetonas.lt/</t>
         </is>
       </c>
       <c r="W61" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.ponasbetonas.lt/#Apiemus</t>
         </is>
       </c>
       <c r="X61" s="2" t="inlineStr">
         <is>
-          <t>https://c3beton.com/lt/betonas</t>
+          <t>https://www.ponasbetonas.lt/</t>
         </is>
       </c>
       <c r="Y61" s="2" t="inlineStr">
         <is>
-          <t>Įtraukta pagal oficialaus C3 Betonas puslapio žemėlapį. Koordinatės paimtos iš oficialaus puslapio programinio kodo; adresas patikslintas pagal koordinates. Techniniai duomenys papildyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Nuosavas betono mazgas ir prekinio betono gamyba patvirtinti oficialiame įmonės puslapyje. Mazgo gamintojas nustatytas pagal oficialaus puslapio hero nuotraukoje ant silosų matomą ELKON ženklinimą; modelis, maišyklė ir našumas viešai nenurodyti. Tiksli mazgo lokacija paimta iš naudotojo pateiktos Google Maps nuorodos; vietovė patikslinta pagal OpenStreetMap. Įmonės kodas patvirtintas Registrų centro viešame juridinio asmens pranešime.</t>
         </is>
       </c>
       <c r="Z61" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>reljef-rukla</t>
+          <t>pabrades-betonas-pabrade</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>301731961</t>
+          <t>306177188</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>UAB Reljef</t>
+          <t>UAB Pabradės betonas</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Reljef</t>
+          <t>Pabradės betonas</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -7591,38 +7627,38 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Rukla</t>
+          <t>Pabradė</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Jonavos r. sav.</t>
+          <t>Švenčionių r. sav.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Rukla, Jonavos r. sav.</t>
+          <t>Vilniaus g. 161, Pabradė, LT-18177 Švenčionių r.</t>
         </is>
       </c>
       <c r="I62" s="3" t="n">
-        <v>55.05225</v>
+        <v>54.9758768</v>
       </c>
       <c r="J62" s="3" t="n">
-        <v>24.4064167</v>
+        <v>25.7373849</v>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Tikslus naudotojo pateiktas taškas; adresas artimiausias pagal OpenStreetMap</t>
+          <t>Tikslus oficialioje svetainėje pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>Naudotojo pateiktos koordinatės</t>
+          <t>Oficiali Pabradės betono Google Maps nuoroda</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
+          <t>https://maps.app.goo.gl/TQBCVR8DczDRvQaeA</t>
         </is>
       </c>
       <c r="N62" s="2" t="inlineStr">
@@ -7637,77 +7673,77 @@
       </c>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t>Ammann Elba</t>
+          <t>Liebherr (tikėtina)</t>
         </is>
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>Nenustatyta</t>
+          <t>3 m³</t>
         </is>
       </c>
       <c r="R62" s="2" t="inlineStr">
         <is>
-          <t>Nenustatytas</t>
+          <t>60 m³/val.</t>
         </is>
       </c>
       <c r="S62" s="4" t="inlineStr">
         <is>
-          <t>2x65 t</t>
+          <t>3x65 t</t>
         </is>
       </c>
       <c r="T62" s="2" t="inlineStr">
         <is>
-          <t>Rukloje veikiantis UAB Reljef betono mazgas: Ammann Elba, 2x65 t silosai. Maišyklė ir našumas nenustatyti.</t>
+          <t>UAB Pabradės betonas Vilniaus g. 161, Pabradėje, gamina sertifikuotą normalųjį betoną ir oficialiai nurodo dirbanti 50 km spinduliu aplink Pabradę. Oficialios galerijos nuotraukose matoma stacionari gamybos bazė su trimis cemento silosais. Mazgo gamintojas tikėtinai Liebherr pagal oficialiose nuotraukose matomą Liebherr įrangą ir gamyklos konstrukcijos vizualinius požymius; gamintojo lentelė viešai neparodyta.</t>
         </is>
       </c>
       <c r="U62" s="5" t="n">
-        <v>0.82</v>
+        <v>0.72</v>
       </c>
       <c r="V62" s="2" t="inlineStr">
         <is>
-          <t>https://www.reljef.lt/</t>
+          <t>https://www.pabradesbetonas.lt/</t>
         </is>
       </c>
       <c r="W62" s="2" t="inlineStr">
         <is>
-          <t>https://www.reljef.lt/</t>
+          <t>https://www.pabradesbetonas.lt/</t>
         </is>
       </c>
       <c r="X62" s="2" t="inlineStr">
         <is>
-          <t>https://www.openstreetmap.org/?mlat=55.05225&amp;mlon=24.4064167#map=18/55.05225/24.4064167</t>
+          <t>https://www.pabradesbetonas.lt/galerija/</t>
         </is>
       </c>
       <c r="Y62" s="2" t="inlineStr">
         <is>
-          <t>Įmonės rekvizitai paimti iš oficialaus UAB Reljef puslapio. Betono mazgo gamintojas, silosai ir lokacija įrašyti pagal naudotojo pateiktą informaciją. Artimiausias viešai geokoduotas adresas nustatytas pagal OpenStreetMap.</t>
+          <t>Adresas, įmonės kodas ir betono gamyba patvirtinti oficialioje svetainėje bei viešame gamybos kontrolės sertifikate. Koordinatės paimtos iš oficialioje svetainėje pateiktos Google Maps nuorodos. Maišyklės tūris 3 m³, realus našumas 60 m³/val. ir silosai 3x65 t įrašyti pagal naudotojo pateiktą informaciją. Gamintojas Liebherr nurodytas kaip tikėtinas pagal oficialios galerijos nuotraukas; viešo gamintojo ženklinimo ant paties mazgo nerasta.</t>
         </is>
       </c>
       <c r="Z62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>ponas-betonas-paraudondvariai</t>
+          <t>alkesta-marijampole-vasaros</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>306676006</t>
+          <t>249672710</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>UAB Ponas betonas</t>
+          <t>UAB Alkesta</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Ponas betonas</t>
+          <t>Alkesta</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -7717,24 +7753,24 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Paraudondvariai</t>
+          <t>Marijampolė</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus r. sav.</t>
+          <t>Marijampolės sav.</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus g., Paraudondvariai, Riešės sen., Vilniaus r. sav.</t>
+          <t>Vasaros g. 14, Marijampolė, LT-68111</t>
         </is>
       </c>
       <c r="I63" s="3" t="n">
-        <v>54.8321418</v>
+        <v>54.5686121</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>25.2755596</v>
+        <v>23.3895157</v>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
@@ -7748,7 +7784,7 @@
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/NxQohpnzv1q9DA6CA?g_st=ac</t>
+          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
         </is>
       </c>
       <c r="N63" s="2" t="inlineStr">
@@ -7763,77 +7799,73 @@
       </c>
       <c r="P63" s="2" t="inlineStr">
         <is>
-          <t>Elkon</t>
+          <t>Elba</t>
         </is>
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
+          <t>0,5 m³</t>
         </is>
       </c>
       <c r="R63" s="2" t="inlineStr">
         <is>
-          <t>Nenurodyta viešai</t>
-        </is>
-      </c>
-      <c r="S63" s="4" t="inlineStr">
-        <is>
-          <t>2 matomi oficialioje nuotraukoje</t>
-        </is>
-      </c>
+          <t>10 m³/val.</t>
+        </is>
+      </c>
+      <c r="S63" s="4" t="inlineStr"/>
       <c r="T63" s="2" t="inlineStr">
         <is>
-          <t>Oficialiame UAB Ponas betonas puslapyje nurodoma, kad įmonė turi nuosavą betono mazgą, gamina prekinį betoną ir jį pristato. Puslapio hero nuotraukoje ant silosų matomas ELKON ženklinimas, todėl mazgo gamintojas identifikuotas kaip Elkon. Konkretus modelis, maišyklė ir našumas viešai nenurodyti; oficialioje nuotraukoje matomi 2 silosai.</t>
+          <t>UAB Alkesta Marijampolės betono mazgas Vasaros g. 14. Mazgo gamintojas Elba, maišyklė 0,5 m³, našumas 10 m³/val.</t>
         </is>
       </c>
       <c r="U63" s="5" t="n">
-        <v>0.98</v>
+        <v>0.95</v>
       </c>
       <c r="V63" s="2" t="inlineStr">
         <is>
-          <t>https://www.ponasbetonas.lt/</t>
+          <t>https://alkesta.lt/</t>
         </is>
       </c>
       <c r="W63" s="2" t="inlineStr">
         <is>
-          <t>https://www.ponasbetonas.lt/#Apiemus</t>
+          <t>https://spsc.lt/registrai/regsapp/ser_produktai_view.php?editid1=13061</t>
         </is>
       </c>
       <c r="X63" s="2" t="inlineStr">
         <is>
-          <t>https://www.ponasbetonas.lt/</t>
+          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
         </is>
       </c>
       <c r="Y63" s="2" t="inlineStr">
         <is>
-          <t>Nuosavas betono mazgas ir prekinio betono gamyba patvirtinti oficialiame įmonės puslapyje. Mazgo gamintojas nustatytas pagal oficialaus puslapio hero nuotraukoje ant silosų matomą ELKON ženklinimą; modelis, maišyklė ir našumas viešai nenurodyti. Tiksli mazgo lokacija paimta iš naudotojo pateiktos Google Maps nuorodos; vietovė patikslinta pagal OpenStreetMap. Įmonės kodas patvirtintas Registrų centro viešame juridinio asmens pranešime.</t>
+          <t>Oficialus SPSC sertifikatų registras patvirtina UAB Alkesta betono gamybą ir gamybos vietą Vasaros g. 14, Marijampolėje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris ir našumas įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-23</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>pabrades-betonas-pabrade</t>
+          <t>gevalda-visincia</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>306177188</t>
+          <t>302592895</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>UAB Pabradės betonas</t>
+          <t>UAB Gevalda</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Pabradės betonas</t>
+          <t>Gevalda</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -7843,38 +7875,38 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Pabradė</t>
+          <t>Visinčia</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Švenčionių r. sav.</t>
+          <t>Šalčininkų r. sav.</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Vilniaus g. 161, Pabradė, LT-18177 Švenčionių r.</t>
+          <t>Visinčia, Pabarės sen., Šalčininkų r. sav.</t>
         </is>
       </c>
       <c r="I64" s="3" t="n">
-        <v>54.9758768</v>
+        <v>54.4122467</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>25.7373849</v>
+        <v>25.1449142</v>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Tikslus oficialioje svetainėje pateiktos Google Maps nuorodos taškas</t>
+          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>Oficiali Pabradės betono Google Maps nuoroda</t>
+          <t>Naudotojo pateikta Google Maps lokacija</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/TQBCVR8DczDRvQaeA</t>
+          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
         </is>
       </c>
       <c r="N64" s="2" t="inlineStr">
@@ -7889,7 +7921,7 @@
       </c>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>Liebherr (tikėtina)</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr">
@@ -7904,35 +7936,35 @@
       </c>
       <c r="S64" s="4" t="inlineStr">
         <is>
-          <t>3x65 t</t>
+          <t>2x85 t</t>
         </is>
       </c>
       <c r="T64" s="2" t="inlineStr">
         <is>
-          <t>UAB Pabradės betonas Vilniaus g. 161, Pabradėje, gamina sertifikuotą normalųjį betoną ir oficialiai nurodo dirbanti 50 km spinduliu aplink Pabradę. Oficialios galerijos nuotraukose matoma stacionari gamybos bazė su trimis cemento silosais. Mazgo gamintojas tikėtinai Liebherr pagal oficialiose nuotraukose matomą Liebherr įrangą ir gamyklos konstrukcijos vizualinius požymius; gamintojo lentelė viešai neparodyta.</t>
+          <t>UAB Gevalda mobilus betono mazgas Visinčioje. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U64" s="5" t="n">
-        <v>0.72</v>
+        <v>0.95</v>
       </c>
       <c r="V64" s="2" t="inlineStr">
         <is>
-          <t>https://www.pabradesbetonas.lt/</t>
+          <t>https://www.gevalda.lt/</t>
         </is>
       </c>
       <c r="W64" s="2" t="inlineStr">
         <is>
-          <t>https://www.pabradesbetonas.lt/</t>
+          <t>https://www.gevalda.lt/paslaugos/gamyba</t>
         </is>
       </c>
       <c r="X64" s="2" t="inlineStr">
         <is>
-          <t>https://www.pabradesbetonas.lt/galerija/</t>
+          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
         </is>
       </c>
       <c r="Y64" s="2" t="inlineStr">
         <is>
-          <t>Adresas, įmonės kodas ir betono gamyba patvirtinti oficialioje svetainėje bei viešame gamybos kontrolės sertifikate. Koordinatės paimtos iš oficialioje svetainėje pateiktos Google Maps nuorodos. Maišyklės tūris 3 m³, realus našumas 60 m³/val. ir silosai 3x65 t įrašyti pagal naudotojo pateiktą informaciją. Gamintojas Liebherr nurodytas kaip tikėtinas pagal oficialios galerijos nuotraukas; viešo gamintojo ženklinimo ant paties mazgo nerasta.</t>
+          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris, našumas ir silosai įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z64" s="2" t="inlineStr">
@@ -7944,22 +7976,22 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>alkesta-marijampole-vasaros</t>
+          <t>gevalda-kaunas-palemonas</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>249672710</t>
+          <t>302592895</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>UAB Alkesta</t>
+          <t>UAB Gevalda</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>Alkesta</t>
+          <t>Gevalda</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -7969,24 +8001,24 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Marijampolė</t>
+          <t>Kaunas</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Marijampolės sav.</t>
+          <t>Kauno m. sav.</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Vasaros g. 14, Marijampolė, LT-68111</t>
+          <t>Kražantės g., Palemonas, Kaunas</t>
         </is>
       </c>
       <c r="I65" s="3" t="n">
-        <v>54.5686121</v>
+        <v>54.918</v>
       </c>
       <c r="J65" s="3" t="n">
-        <v>23.3895157</v>
+        <v>24.063</v>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
@@ -8000,7 +8032,7 @@
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
+          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
         </is>
       </c>
       <c r="N65" s="2" t="inlineStr">
@@ -8015,23 +8047,27 @@
       </c>
       <c r="P65" s="2" t="inlineStr">
         <is>
-          <t>Elba</t>
+          <t>Elkon</t>
         </is>
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>0,5 m³</t>
+          <t>3 m³</t>
         </is>
       </c>
       <c r="R65" s="2" t="inlineStr">
         <is>
-          <t>10 m³/val.</t>
-        </is>
-      </c>
-      <c r="S65" s="4" t="inlineStr"/>
+          <t>60 m³/val.</t>
+        </is>
+      </c>
+      <c r="S65" s="4" t="inlineStr">
+        <is>
+          <t>2x85 t</t>
+        </is>
+      </c>
       <c r="T65" s="2" t="inlineStr">
         <is>
-          <t>UAB Alkesta Marijampolės betono mazgas Vasaros g. 14. Mazgo gamintojas Elba, maišyklė 0,5 m³, našumas 10 m³/val.</t>
+          <t>UAB Gevalda mobilus betono mazgas Palemone, Kaune. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
         </is>
       </c>
       <c r="U65" s="5" t="n">
@@ -8039,22 +8075,22 @@
       </c>
       <c r="V65" s="2" t="inlineStr">
         <is>
-          <t>https://alkesta.lt/</t>
+          <t>https://www.gevalda.lt/</t>
         </is>
       </c>
       <c r="W65" s="2" t="inlineStr">
         <is>
-          <t>https://spsc.lt/registrai/regsapp/ser_produktai_view.php?editid1=13061</t>
+          <t>https://www.gevalda.lt/paslaugos/gamyba</t>
         </is>
       </c>
       <c r="X65" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/xKhbiD3KQWzTBzhK9?g_st=ic</t>
+          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
         </is>
       </c>
       <c r="Y65" s="2" t="inlineStr">
         <is>
-          <t>Oficialus SPSC sertifikatų registras patvirtina UAB Alkesta betono gamybą ir gamybos vietą Vasaros g. 14, Marijampolėje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris ir našumas įrašyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija ir analogiški techniniai duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
         </is>
       </c>
       <c r="Z65" s="2" t="inlineStr">
@@ -8066,22 +8102,22 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>gevalda-visincia</t>
+          <t>telsiu-gelzbetonis-telsiai</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>302592895</t>
+          <t>180245532</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>UAB Gevalda</t>
+          <t>UAB Telšių gelžbetonis</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Gevalda</t>
+          <t>Telšių gelžbetonis</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -8091,73 +8127,61 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Visinčia</t>
+          <t>Telšiai</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Šalčininkų r. sav.</t>
+          <t>Telšių r. sav.</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>Visinčia, Pabarės sen., Šalčininkų r. sav.</t>
+          <t>Statybininkų g. 2-8, LT-87101 Telšiai</t>
         </is>
       </c>
       <c r="I66" s="3" t="n">
-        <v>54.4122467</v>
+        <v>55.9947877</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>25.1449142</v>
+        <v>22.2517039</v>
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
+          <t>Oficialios svetainės žemėlapio adreso taškas</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>Naudotojo pateikta Google Maps lokacija</t>
+          <t>Google Maps (oficiali įmonės kontaktų nuoroda)</t>
         </is>
       </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
+          <t>https://maps.app.goo.gl/fJnDGN7yksUMAyQa9</t>
         </is>
       </c>
       <c r="N66" s="2" t="inlineStr">
         <is>
-          <t>ready_mix_concrete</t>
+          <t>precast_concrete</t>
         </is>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>Betono mišiniai</t>
-        </is>
-      </c>
-      <c r="P66" s="2" t="inlineStr">
-        <is>
-          <t>Elkon</t>
-        </is>
-      </c>
+          <t>Betono mišiniai ir gelžbetonio gaminiai</t>
+        </is>
+      </c>
+      <c r="P66" s="2" t="inlineStr"/>
       <c r="Q66" s="2" t="inlineStr">
         <is>
-          <t>3 m³</t>
-        </is>
-      </c>
-      <c r="R66" s="2" t="inlineStr">
-        <is>
-          <t>60 m³/val.</t>
-        </is>
-      </c>
-      <c r="S66" s="4" t="inlineStr">
-        <is>
-          <t>2x85 t</t>
-        </is>
-      </c>
+          <t>Sicoma OMG planetarinė maišyklė</t>
+        </is>
+      </c>
+      <c r="R66" s="2" t="inlineStr"/>
+      <c r="S66" s="4" t="inlineStr"/>
       <c r="T66" s="2" t="inlineStr">
         <is>
-          <t>UAB Gevalda mobilus betono mazgas Visinčioje. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
+          <t>Gamintojas siūlo betoninius ir gelžbetoninius gaminius bei prekinį betoną C8/10–C35/45. Oficialioje įmonės istorijoje nurodytas betono mazgo automatizavimas (2016 m.) ir Sicoma OMG planetarinės maišyklės sumontavimas (2023 m.).</t>
         </is>
       </c>
       <c r="U66" s="5" t="n">
@@ -8165,158 +8189,32 @@
       </c>
       <c r="V66" s="2" t="inlineStr">
         <is>
-          <t>https://www.gevalda.lt/</t>
+          <t>https://tgb.lt/</t>
         </is>
       </c>
       <c r="W66" s="2" t="inlineStr">
         <is>
-          <t>https://www.gevalda.lt/paslaugos/gamyba</t>
+          <t>https://tgb.lt/kontaktai/</t>
         </is>
       </c>
       <c r="X66" s="2" t="inlineStr">
         <is>
-          <t>https://maps.app.goo.gl/xuuJfukn3ApaYNME6?g_st=ic</t>
+          <t>https://tgb.lt/apie-imone/</t>
         </is>
       </c>
       <c r="Y66" s="2" t="inlineStr">
         <is>
-          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija, mazgo gamintojas, maišyklės tūris, našumas ir silosai įrašyti pagal naudotojo pateiktą informaciją.</t>
+          <t>Adresas ir Google Maps nuoroda paimti iš oficialios svetainės kontaktų. Nuoroda rodo Statybininkų g. 2 adreso tašką; tai nėra atskirai patvirtinta mazgo vieta sklype. Prekinio betono šaltinis: https://tgb.lt/prekinis-betonas/. Kontaktai: +370 679 89333, info@tgb.lt. Įmonės kodas patvirtintas Registrų centro leidinyje: https://www.registrucentras.lt/jar/infleid/download.do?oid=252865. Maišyklės tūris, našumas ir silosai viešai nenurodyti.</t>
         </is>
       </c>
       <c r="Z66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>gevalda-kaunas-palemonas</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>302592895</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>UAB Gevalda</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>Gevalda</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>Konkurentas</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="inlineStr">
-        <is>
-          <t>Kaunas</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>Kauno m. sav.</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>Kražantės g., Palemonas, Kaunas</t>
-        </is>
-      </c>
-      <c r="I67" s="3" t="n">
-        <v>54.918</v>
-      </c>
-      <c r="J67" s="3" t="n">
-        <v>24.063</v>
-      </c>
-      <c r="K67" s="2" t="inlineStr">
-        <is>
-          <t>Tikslus naudotojo pateiktos Google Maps nuorodos taškas</t>
-        </is>
-      </c>
-      <c r="L67" s="2" t="inlineStr">
-        <is>
-          <t>Naudotojo pateikta Google Maps lokacija</t>
-        </is>
-      </c>
-      <c r="M67" s="2" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
-        </is>
-      </c>
-      <c r="N67" s="2" t="inlineStr">
-        <is>
-          <t>ready_mix_concrete</t>
-        </is>
-      </c>
-      <c r="O67" s="2" t="inlineStr">
-        <is>
-          <t>Betono mišiniai</t>
-        </is>
-      </c>
-      <c r="P67" s="2" t="inlineStr">
-        <is>
-          <t>Elkon</t>
-        </is>
-      </c>
-      <c r="Q67" s="2" t="inlineStr">
-        <is>
-          <t>3 m³</t>
-        </is>
-      </c>
-      <c r="R67" s="2" t="inlineStr">
-        <is>
-          <t>60 m³/val.</t>
-        </is>
-      </c>
-      <c r="S67" s="4" t="inlineStr">
-        <is>
-          <t>2x85 t</t>
-        </is>
-      </c>
-      <c r="T67" s="2" t="inlineStr">
-        <is>
-          <t>UAB Gevalda mobilus betono mazgas Palemone, Kaune. Mazgo gamintojas Elkon, maišyklė 3 m³, našumas 60 m³/val., silosai 2x85 t.</t>
-        </is>
-      </c>
-      <c r="U67" s="5" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="V67" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gevalda.lt/</t>
-        </is>
-      </c>
-      <c r="W67" s="2" t="inlineStr">
-        <is>
-          <t>https://www.gevalda.lt/paslaugos/gamyba</t>
-        </is>
-      </c>
-      <c r="X67" s="2" t="inlineStr">
-        <is>
-          <t>https://maps.app.goo.gl/sKM8v9zqzZz9ZR8i8</t>
-        </is>
-      </c>
-      <c r="Y67" s="2" t="inlineStr">
-        <is>
-          <t>Oficiali UAB Gevalda svetainė patvirtina betono mišinių gamybą mobilioje gamykloje. Tiksli lokacija ir analogiški techniniai duomenys įrašyti pagal naudotojo pateiktą informaciją.</t>
-        </is>
-      </c>
-      <c r="Z67" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z67"/>
+  <autoFilter ref="A1:Z66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -8405,7 +8303,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-12T12:42:52.334852+00:00</t>
+          <t>2026-10-14T05:44:30.655552+00:00</t>
         </is>
       </c>
     </row>
@@ -8460,7 +8358,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-12T12:42:52.335562+00:00</t>
+          <t>2026-10-14T05:44:30.655552+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8474,7 +8372,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>

</xml_diff>